<commit_message>
Use one menu for language levels and spell out classroom activities.
Norsk is navigated by Om opplæringen, Før A1 and A1–B2, with the same sections in the sidebar and overview. Each level card now gives the teacher a prepare, do and look-for suggestion.

Co-authored-by: Ivar <IvarMolde@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/data/digitale-ferdigheter.xlsx
+++ b/public/data/digitale-ferdigheter.xlsx
@@ -72,13 +72,19 @@
     <t>Opptrer ansvarlig selvstendig i all digital kommunikasjon og ivaretar personvern.</t>
   </si>
   <si>
-    <t>Læreren viser tre skjermbilder av chatmeldinger på storskjerm: en vennlig melding, en uhøflig melding og en melding der noen deler et bilde av en annen uten å spørre. Elevene viser tommel opp eller ned for hver melding. Klassen lager sammen tre–fire enkle regler med ikoner («Vi skriver vennlig», «Vi spør før vi deler bilder»). Reglene henges opp ved PC-ene og leses høyt før hver digitale økt.</t>
-  </si>
-  <si>
-    <t>Elevene får situasjonskort, for eksempel «Du vil dele et klassebilde i gruppechatten». I par velger de hva de vil gjøre, og forklarer med setningsstarteren «Jeg gjør … fordi …». Hvert par presenterer ett valg for klassen, og læreren skriver begrunnelsene på tavla som felles ordforråd.</t>
-  </si>
-  <si>
-    <t>Elevene lager i grupper en digital plakat med regler for klassens kanal (f.eks. i Teams) om tone, bilder og personvern. Hver regel skal ha en kort begrunnelse. Etter en uke sjekker gruppene egne innlegg mot plakaten og foreslår eventuelle endringer.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser tre skjermbilder av chatmeldinger på storskjerm: en vennlig melding, en uhøflig melding og en melding der noen deler et bilde av en annen uten å spørre. Elevene viser tommel opp eller ned for hver melding. Klassen lager sammen tre–fire enkle regler med ikoner («Vi skriver vennlig», «Vi spør før vi deler bilder»). Reglene henges opp ved PC-ene og leses høyt før hver digitale økt. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar situasjonskort, setningsstartere og bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får situasjonskort, for eksempel «Du vil dele et klassebilde i gruppechatten». I par velger de hva de vil gjøre, og forklarer med setningsstarteren «Jeg gjør … fordi …». Hvert par presenterer ett valg for klassen, og læreren skriver begrunnelsene på tavla som felles ordforråd. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar plakaten, bilder og kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene lager i grupper en digital plakat med regler for klassens kanal (f.eks. i Teams) om tone, bilder og personvern. Hver regel skal ha en kort begrunnelse. Etter en uke sjekker gruppene egne innlegg mot plakaten og foreslår eventuelle endringer. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>2.3 – Grunnleggende ferdigheter</t>
@@ -99,13 +105,19 @@
     <t>Videreutvikler digitale ferdigheter selvstendig gjennom hele opplæringsløpet.</t>
   </si>
   <si>
-    <t>Innfør en fast digital startrutine hver økt: slå på PC, logge inn, åpne læringsplattformen og finne dagens oppgave. Læreren viser trinnene på storskjerm med nummererte bildekort (1–2–3–4). Elevene gjør det samme i sitt eget tempo, og sidemannen hjelper ved behov. Rutinen er lik hver dag til den sitter.</t>
-  </si>
-  <si>
-    <t>Elevene har en enkel sjekkliste med ikoner: logge inn, lagre, finne fil, sende. Etter hver økt krysser de av det de klarte alene. Læreren samler inn listene hver fredag og velger neste ferdighet klassen skal øve på ut fra hva mange mangler.</t>
-  </si>
-  <si>
-    <t>Elevene fører en digital logg der de hver uke skriver én ny ting de har lært å gjøre digitalt og ett mål for neste uke. En gang i måneden viser hver elev en ny ferdighet til en medelev («elev lærer elev»).</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, bildekort og læringsplattformen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Innfør en fast digital startrutine hver økt: slå på PC, logge inn, åpne læringsplattformen og finne dagens oppgave. Læreren viser trinnene på storskjerm med nummererte bildekort (1–2–3–4). Elevene gjør det samme i sitt eget tempo, og sidemannen hjelper ved behov. Rutinen er lik hver dag til den sitter. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene har en enkel sjekkliste med ikoner: logge inn, lagre, finne fil, sende. Etter hver økt krysser de av det de klarte alene. Læreren samler inn listene hver fredag og velger neste ferdighet klassen skal øve på ut fra hva mange mangler. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene fører en digital logg der de hver uke skriver én ny ting de har lært å gjøre digitalt og ett mål for neste uke. En gang i måneden viser hver elev en ny ferdighet til en medelev («elev lærer elev»). Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Digitale ferdigheter som del av faglig kompetanse og læring.</t>
@@ -120,13 +132,19 @@
     <t>Bruker digitale ferdigheter selvstendig som redskap for læring og samfunnsdeltakelse.</t>
   </si>
   <si>
-    <t>Elevene bruker en bildeordbok eller ordapp for å finne ord til dagens tema (f.eks. mat). Læreren viser trinnene: skriv ordet – trykk på lydknappen – lytt – si ordet høyt. Elevene gjør det samme med fem ord og viser bildene til partneren sin.</t>
-  </si>
-  <si>
-    <t>Etter å ha lest en fagtekst finner elevene selv tre nye ord i en digital ordbok, lytter til uttalen og lagrer ordene i sin egen digitale ordliste med bilde eller oversettelse til morsmålet. Neste dag forhører partneren dem på ordene.</t>
-  </si>
-  <si>
-    <t>Elevene lager et lite digitalt produkt om et tema fra undervisningen, for eksempel en kort presentasjon eller et lydopptak. De velger selv verktøy og kilder, og avslutter med å forklare hvordan verktøyet hjalp dem å lære.</t>
+    <t xml:space="preserve">Forbered: Legg klar ordboka og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene bruker en bildeordbok eller ordapp for å finne ord til dagens tema (f.eks. mat). Læreren viser trinnene: skriv ordet – trykk på lydknappen – lytt – si ordet høyt. Elevene gjør det samme med fem ord og viser bildene til partneren sin. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar ordboka og bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Etter å ha lest en fagtekst finner elevene selv tre nye ord i en digital ordbok, lytter til uttalen og lagrer ordene i sin egen digitale ordliste med bilde eller oversettelse til morsmålet. Neste dag forhører partneren dem på ordene. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene lager et lite digitalt produkt om et tema fra undervisningen, for eksempel en kort presentasjon eller et lydopptak. De velger selv verktøy og kilder, og avslutter med å forklare hvordan verktøyet hjalp dem å lære. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Integrer digitale ferdigheter på tvers av fag.</t>
@@ -141,13 +159,19 @@
     <t>Bruker digitale ferdigheter selvstendig og integrert på tvers av fag.</t>
   </si>
   <si>
-    <t>Handleoppgave: Læreren åpner en nettbutikk på storskjerm. Elevene leser navnet på tre varer (lesing), skriver dem i et dokument (skriving), sier dem høyt til partneren (muntlig) og legger sammen prisene med kalkulatoren på PC-en (regning). Læreren viser hvert trinn før elevene gjør det.</t>
-  </si>
-  <si>
-    <t>Elevene planlegger en busstur med en reiseapp eller nettside: de finner avgangstid (lesing), regner ut hvor lang tid turen tar (regning), skriver en kort melding om når de kommer fram (skriving) og forteller planen til partneren (muntlig).</t>
-  </si>
-  <si>
-    <t>Elevene planlegger et klassearrangement. De sammenligner priser på nett, lager et enkelt budsjett i regneark, skriver en digital invitasjon og presenterer planen muntlig for klassen. Elevene velger selv hvilke verktøy de bruker.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Handleoppgave: Læreren åpner en nettbutikk på storskjerm. Elevene leser navnet på tre varer (lesing), skriver dem i et dokument (skriving), sier dem høyt til partneren (muntlig) og legger sammen prisene med kalkulatoren på PC-en (regning). Læreren viser hvert trinn før elevene gjør det. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene planlegger en busstur med en reiseapp eller nettside: de finner avgangstid (lesing), regner ut hvor lang tid turen tar (regning), skriver en kort melding om når de kommer fram (skriving) og forteller planen til partneren (muntlig). Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene planlegger et klassearrangement. De sammenligner priser på nett, lager et enkelt budsjett i regneark, skriver en digital invitasjon og presenterer planen muntlig for klassen. Elevene velger selv hvilke verktøy de bruker. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>2.5.3 – Bærekraftig utvikling</t>
@@ -168,13 +192,19 @@
     <t>Forstår og drøfter selvstendig sammenhenger mellom teknologi og bærekraft.</t>
   </si>
   <si>
-    <t>Læreren viser bilder av en lader, en mobil, en PC og gamle mobiler i en skuff. Elevene sorterer bildene sammen med læreren i to grupper: «bruker strøm» og «kan gjenbrukes». Klassen øver på enkle setninger: «Mobilen bruker strøm.» «Den gamle mobilen kan leveres.»</t>
-  </si>
-  <si>
-    <t>I par får elevene dilemmakort, for eksempel «Bør man kjøpe ny mobil hvert år?» eller «Er det greit å strømme video hele dagen?». De svarer ja eller nei, begrunner med «fordi …» og sammenligner svarene med et annet par.</t>
-  </si>
-  <si>
-    <t>Elevene undersøker ett tema i digitale kilder, for eksempel elektronisk avfall eller netthandel med gratis retur. I gruppe drøfter de fordeler og ulemper for miljø, økonomi og mennesker, og presenterer en kort konklusjon for klassen.</t>
+    <t xml:space="preserve">Forbered: Legg klar mobilen og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser bilder av en lader, en mobil, en PC og gamle mobiler i en skuff. Elevene sorterer bildene sammen med læreren i to grupper: «bruker strøm» og «kan gjenbrukes». Klassen øver på enkle setninger: «Mobilen bruker strøm.» «Den gamle mobilen kan leveres.». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar dilemmakort, klippet og mobilen før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: I par får elevene dilemmakort, for eksempel «Bør man kjøpe ny mobil hvert år?» eller «Er det greit å strømme video hele dagen?». De svarer ja eller nei, begrunner med «fordi …» og sammenligner svarene med et annet par. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene undersøker ett tema i digitale kilder, for eksempel elektronisk avfall eller netthandel med gratis retur. I gruppe drøfter de fordeler og ulemper for miljø, økonomi og mennesker, og presenterer en kort konklusjon for klassen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>1.5 – Miljøbevissthet</t>
@@ -195,13 +225,19 @@
     <t>Reflekterer selvstendig over teknologiens rolle for bærekraft.</t>
   </si>
   <si>
-    <t>Læreren viser en sorteringsguide eller app fra det lokale renovasjonsselskapet på storskjerm. Klassen søker sammen på «batteri» og «gammel mobil», og elevene peker på svaret. Hver elev får et bildekort med én gjenstand og viser hvor den skal kastes.</t>
-  </si>
-  <si>
-    <t>Elevene bruker selv en sorteringsguide eller en nettside for bruktsalg for å finne ut hvordan tre gjenstander kan sorteres eller gjenbrukes. De skriver én setning om hver gjenstand: «Jeg kan … fordi …».</t>
-  </si>
-  <si>
-    <t>Elevene lager en liten digital guide for klassen: «Tre digitale verktøy som hjelper deg å leve miljøvennlig». De presenterer guiden og begrunner hvorfor de valgte akkurat disse verktøyene.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, bildekort og mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en sorteringsguide eller app fra det lokale renovasjonsselskapet på storskjerm. Klassen søker sammen på «batteri» og «gammel mobil», og elevene peker på svaret. Hver elev får et bildekort med én gjenstand og viser hvor den skal kastes. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker selv en sorteringsguide eller en nettside for bruktsalg for å finne ut hvordan tre gjenstander kan sorteres eller gjenbrukes. De skriver én setning om hver gjenstand: «Jeg kan … fordi …». Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene lager en liten digital guide for klassen: «Tre digitale verktøy som hjelper deg å leve miljøvennlig». De presenterer guiden og begrunner hvorfor de valgte akkurat disse verktøyene. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>2.4 – Å lære å lære</t>
@@ -222,13 +258,19 @@
     <t>Styrer egen læring med mangfold av digitale strategier.</t>
   </si>
   <si>
-    <t>Læreren gir et spørsmål med bilde, for eksempel «Når åpner biblioteket?», og en ferdig lenke. Elevene finner svaret med lærerens hjelp og svarer med en fast setning: «Biblioteket åpner klokka …». Samme type oppgave gjentas med nye spørsmål flere dager på rad.</t>
-  </si>
-  <si>
-    <t>Elevene lager selv ett spørsmål om nærmiljøet ved hjelp av kort med spørreord (hva, når, hvor, hvor mye). De velger om de vil bruke søkemotor eller en kjent nettside, finner svaret og forteller partneren hvordan de søkte.</t>
-  </si>
-  <si>
-    <t>Elevene formulerer tre egne spørsmål om et tema, planlegger søket (søkeord og kilder), søker og vurderer svarene. Til slutt skriver de kort hvilken strategi som fungerte best og hvorfor.</t>
+    <t xml:space="preserve">Forbered: Legg klar lenken og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren gir et spørsmål med bilde, for eksempel «Når åpner biblioteket?», og en ferdig lenke. Elevene finner svaret med lærerens hjelp og svarer med en fast setning: «Biblioteket åpner klokka …». Samme type oppgave gjentas med nye spørsmål flere dager på rad. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene lager selv ett spørsmål om nærmiljøet ved hjelp av kort med spørreord (hva, når, hvor, hvor mye). De velger om de vil bruke søkemotor eller en kjent nettside, finner svaret og forteller partneren hvordan de søkte. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene formulerer tre egne spørsmål om et tema, planlegger søket (søkeord og kilder), søker og vurderer svarene. Til slutt skriver de kort hvilken strategi som fungerte best og hvorfor. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>2.5.1 – Folkehelse</t>
@@ -249,13 +291,19 @@
     <t>Tar bevisste valg om mediebruk og digital økonomi selvstendig.</t>
   </si>
   <si>
-    <t>Elevene åpner skjermtid-oversikten på egen mobil sammen med læreren. Ved hjelp av bildekort (sove, jobbe, video, familie, nyheter) forteller de enkelt: «Jeg bruker mobilen til …». Klassen snakker om hvordan skjerm påvirker søvn, og øver på setningen «Jeg legger bort mobilen klokka …».</t>
-  </si>
-  <si>
-    <t>Elevene fører en enkel mediedagbok i tre dager (tabell: når – hva – hvor lenge). I par sammenligner de dagbøkene og foreslår én endring. De ser også på oversikten i bankappen og finner hva de har brukt penger på digitalt, for eksempel abonnementer.</t>
-  </si>
-  <si>
-    <t>Elevene setter et eget mål for mediebruk eller digital økonomi, for eksempel en skjermfri kveld i uka eller å si opp et abonnement de ikke bruker. De følger opp målet i to uker og forteller kort for klassen hva som skjedde.</t>
+    <t xml:space="preserve">Forbered: Legg klar bildekort, klippet og mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene åpner skjermtid-oversikten på egen mobil sammen med læreren. Ved hjelp av bildekort (sove, jobbe, video, familie, nyheter) forteller de enkelt: «Jeg bruker mobilen til …». Klassen snakker om hvordan skjerm påvirker søvn, og øver på setningen «Jeg legger bort mobilen klokka …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene fører en enkel mediedagbok i tre dager (tabell: når – hva – hvor lenge). I par sammenligner de dagbøkene og foreslår én endring. De ser også på oversikten i bankappen og finner hva de har brukt penger på digitalt, for eksempel abonnementer. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene setter et eget mål for mediebruk eller digital økonomi, for eksempel en skjermfri kveld i uka eller å si opp et abonnement de ikke bruker. De følger opp målet i to uker og forteller kort for klassen hva som skjedde. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>2.5.2 – Demokrati</t>
@@ -273,13 +321,19 @@
     <t>Deltar selvstendig og saklig i digital meningsbrytning.</t>
   </si>
   <si>
-    <t>Læreren viser et tilrettelagt skjermbilde av en nettdebatt med både høflige og uhøflige kommentarer. Elevene peker ut de høflige. Klassen øver på faste fraser for uenighet: «Jeg er uenig, fordi …» og «Jeg forstår deg, men …».</t>
-  </si>
-  <si>
-    <t>Læreren legger ut en enkel påstand i en lukket klassekanal, for eksempel «Barn under 13 år bør ikke ha mobil». Elevene skriver en kommentar med begrunnelse og svarer respektfullt på en medelev som mener noe annet. Frasene fra tavla kan brukes som støtte.</t>
-  </si>
-  <si>
-    <t>Elevene deltar i en strukturert digital debatt om en aktuell sak. De finner ett faktagrunnlag i en pålitelig kilde, skriver et saklig innlegg og svarer på motargumenter. Etterpå vurderer de sin egen tone ut fra klassens regler.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et tilrettelagt skjermbilde av en nettdebatt med både høflige og uhøflige kommentarer. Elevene peker ut de høflige. Klassen øver på faste fraser for uenighet: «Jeg er uenig, fordi …» og «Jeg forstår deg, men …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar mobilen før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Læreren legger ut en enkel påstand i en lukket klassekanal, for eksempel «Barn under 13 år bør ikke ha mobil». Elevene skriver en kommentar med begrunnelse og svarer respektfullt på en medelev som mener noe annet. Frasene fra tavla kan brukes som støtte. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene deltar i en strukturert digital debatt om en aktuell sak. De finner ett faktagrunnlag i en pålitelig kilde, skriver et saklig innlegg og svarer på motargumenter. Etterpå vurderer de sin egen tone ut fra klassens regler. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>3.1 – Inkluderende miljø</t>
@@ -300,13 +354,19 @@
     <t>Samhandler forsvarlig og selvstendig på alle digitale flater.</t>
   </si>
   <si>
-    <t>Klassen lager en plakat med ikoner: «Vi skriver vennlig om andre» og «Vi spør før vi deler bilder». Før hver bruk av klassechatten peker læreren på plakaten, og elevene øver på å sende ferdige, vennlige meldinger fra en frasebank.</t>
-  </si>
-  <si>
-    <t>Elevene får situasjonskort, for eksempel «Noen blir holdt utenfor i gruppechatten» eller «Noen har delt et bilde av deg uten å spørre». I par diskuterer de hva de kan gjøre, og skriver en passende melding til personen det gjelder.</t>
-  </si>
-  <si>
-    <t>Elevene evaluerer klassens digitale samhandling med et anonymt skjema og lager forslag til forbedringer. To og to elever har ansvaret for å ønske nye elever velkommen i klassens digitale kanal og hjelpe dem i gang.</t>
+    <t xml:space="preserve">Forbered: Legg klar fraser, plakaten og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Klassen lager en plakat med ikoner: «Vi skriver vennlig om andre» og «Vi spør før vi deler bilder». Før hver bruk av klassechatten peker læreren på plakaten, og elevene øver på å sende ferdige, vennlige meldinger fra en frasebank. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar situasjonskort og bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får situasjonskort, for eksempel «Noen blir holdt utenfor i gruppechatten» eller «Noen har delt et bilde av deg uten å spørre». I par diskuterer de hva de kan gjøre, og skriver en passende melding til personen det gjelder. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene evaluerer klassens digitale samhandling med et anonymt skjema og lager forslag til forbedringer. To og to elever har ansvaret for å ønske nye elever velkommen i klassens digitale kanal og hjelpe dem i gang. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>3.2 – Tilpasset opplæring</t>
@@ -327,13 +387,19 @@
     <t>Velger og bruker digitale læremidler selvstendig ut fra egne behov.</t>
   </si>
   <si>
-    <t>Læreren legger en snarvei til ett digitalt læremiddel på riktig nivå på elevens skrivebord eller hjemskjerm. Eleven åpner læremiddelet, velger oppgave etter fargekode og jobber ti minutter hver dag. De første gangene sitter læreren ved siden av og viser knappene.</t>
-  </si>
-  <si>
-    <t>Eleven velger blant to–tre kjente læremidler ved hjelp av et enkelt valgkart: «Vil du øve på ord? Lytte? Skrive?». Eleven jobber på egen stasjon og noterer hvilket læremiddel og nivå de brukte.</t>
-  </si>
-  <si>
-    <t>Eleven lager en egen ukeplan for digital øving basert på sine mål. Eleven velger læremidler og nivå selv, og forklarer valgene i en kort samtale med læreren.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren legger en snarvei til ett digitalt læremiddel på riktig nivå på elevens skrivebord eller hjemskjerm. Eleven åpner læremiddelet, velger oppgave etter fargekode og jobber ti minutter hver dag. De første gangene sitter læreren ved siden av og viser knappene. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Eleven velger blant to–tre kjente læremidler ved hjelp av et enkelt valgkart: «Vil du øve på ord? Lytte? Skrive?». Eleven jobber på egen stasjon og noterer hvilket læremiddel og nivå de brukte. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Eleven lager en egen ukeplan for digital øving basert på sine mål. Eleven velger læremidler og nivå selv, og forklarer valgene i en kort samtale med læreren. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Sette mål og vurdere egen utvikling i digitale sammenhenger.</t>
@@ -348,13 +414,19 @@
     <t>Setter, følger opp og vurderer egne digitale mål selvstendig.</t>
   </si>
   <si>
-    <t>Eleven velger sammen med læreren ett lite digitalt mål med bilde, for eksempel «sende en e-post». Målet skrives på et målkort. Når målet er nådd, viser eleven læreren hva hen kan, og setter et klistremerke på kortet.</t>
-  </si>
-  <si>
-    <t>Eleven skriver egne mål i et digitalt skjema med setningsstarteren «Jeg vil lære å …». Hver fredag vurderer eleven seg selv med en smilefjes-skala og skriver én setning om hva som gikk bra.</t>
-  </si>
-  <si>
-    <t>Eleven fører en digital mappe med mål, bevis (skjermbilder og filer) og refleksjon. Én gang i måneden har eleven en kort samtale med læreren og justerer målene sine.</t>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel, bilder og kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Eleven velger sammen med læreren ett lite digitalt mål med bilde, for eksempel «sende en e-post». Målet skrives på et målkort. Når målet er nådd, viser eleven læreren hva hen kan, og setter et klistremerke på kortet. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar setningsstartere og skjemaet før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Eleven skriver egne mål i et digitalt skjema med setningsstarteren «Jeg vil lære å …». Hver fredag vurderer eleven seg selv med en smilefjes-skala og skriver én setning om hva som gikk bra. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder og kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Eleven fører en digital mappe med mål, bevis (skjermbilder og filer) og refleksjon. Én gang i måneden har eleven en kort samtale med læreren og justerer målene sine. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Norsk</t>
@@ -378,13 +450,19 @@
     <t>Bruker digitale verktøy selvstendig som redskap for videre læring og arbeidsliv.</t>
   </si>
   <si>
-    <t>Læreren viser tre digitale verktøy med bilder: kamera, ordbok og melding. Elevene øver på å ta bilde av tavla, finne bildet igjen i galleriet og vise det til partneren. Læreren forklarer med enkle ord og bilder at dette også brukes på jobb, for eksempel for å ta bilde av en vaktliste.</t>
-  </si>
-  <si>
-    <t>Elevene får en jobbsituasjon: en vaktliste er sendt på e-post eller i en app. De åpner vaktlista, finner sin egen vakt og svarer med en kort bekreftelse: «Takk, jeg jobber mandag klokka 8.»</t>
-  </si>
-  <si>
-    <t>Elevene undersøker hvilke digitale verktøy som brukes i et yrke de er interessert i (f.eks. på utdanning.no). De lager en kort oversikt over hva de allerede kan og hva de må lære, og legger oversikten i sin digitale mappe.</t>
+    <t xml:space="preserve">Forbered: Legg klar ordboka og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser tre digitale verktøy med bilder: kamera, ordbok og melding. Elevene øver på å ta bilde av tavla, finne bildet igjen i galleriet og vise det til partneren. Læreren forklarer med enkle ord og bilder at dette også brukes på jobb, for eksempel for å ta bilde av en vaktliste. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får en jobbsituasjon: en vaktliste er sendt på e-post eller i en app. De åpner vaktlista, finner sin egen vakt og svarer med en kort bekreftelse: «Takk, jeg jobber mandag klokka 8.». Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene undersøker hvilke digitale verktøy som brukes i et yrke de er interessert i (f.eks. på utdanning.no). De lager en kort oversikt over hva de allerede kan og hva de må lære, og legger oversikten i sin digitale mappe. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 2 – Kartlegging</t>
@@ -405,13 +483,19 @@
     <t>Vurderer egen digital kompetanse underveis og justerer digitale mål.</t>
   </si>
   <si>
-    <t>Praktisk kartlegging: Eleven får bildekort med oppgaver (slå på PC, åpne en app, ta et bilde, sende en melding) og viser læreren hva hen kan. Læreren noterer underveis. Samtalen foregår på enkel norsk, med tolk eller morsmålsstøtte ved behov.</t>
-  </si>
-  <si>
-    <t>Eleven fyller ut en selvvurdering med ikoner og svaralternativene «kan», «kan litt» og «kan ikke». Etterpå forteller eleven læreren om én ting hen vil lære først.</t>
-  </si>
-  <si>
-    <t>Eleven fyller ut det samme kartleggingsskjemaet hver termin, sammenligner med forrige gang og setter nye digitale mål i samtale med læreren.</t>
+    <t xml:space="preserve">Forbered: Legg klar bildekort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Praktisk kartlegging: Eleven får bildekort med oppgaver (slå på PC, åpne en app, ta et bilde, sende en melding) og viser læreren hva hen kan. Læreren noterer underveis. Samtalen foregår på enkel norsk, med tolk eller morsmålsstøtte ved behov. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Eleven fyller ut en selvvurdering med ikoner og svaralternativene «kan», «kan litt» og «kan ikke». Etterpå forteller eleven læreren om én ting hen vil lære først. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Eleven fyller ut det samme kartleggingsskjemaet hver termin, sammenligner med forrige gang og setter nye digitale mål i samtale med læreren. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 2 – Organisering</t>
@@ -429,13 +513,19 @@
     <t>Utnytter digitale muligheter aktivt i egen læring.</t>
   </si>
   <si>
-    <t>Læreren legger dagens plan på samme sted på læringsplattformen hver dag. Klassen øver sammen på å finne den – samme knapper, samme rekkefølge – til alle klarer det. Elevene som er raske, hjelper sidemannen.</t>
-  </si>
-  <si>
-    <t>Elevene får en hjemmeoppgave på læringsplattformen. I klassen øver de på å åpne oppgaven på mobilen, og leverer den hjemmefra. Neste dag forteller de hvordan det gikk og hva som var vanskelig.</t>
-  </si>
-  <si>
-    <t>Elevene bruker plattformen aktivt: de leverer arbeid, bruker ressursbanken til ekstra øving og ordner egne filer i mapper. En gang i uka viser de læreren hva de har øvd på hjemme.</t>
+    <t xml:space="preserve">Forbered: Legg klar læringsplattformen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren legger dagens plan på samme sted på læringsplattformen hver dag. Klassen øver sammen på å finne den – samme knapper, samme rekkefølge – til alle klarer det. Elevene som er raske, hjelper sidemannen. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar læringsplattformen og mobilen før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får en hjemmeoppgave på læringsplattformen. I klassen øver de på å åpne oppgaven på mobilen, og leverer den hjemmefra. Neste dag forteller de hvordan det gikk og hva som var vanskelig. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar læringsplattformen før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker plattformen aktivt: de leverer arbeid, bruker ressursbanken til ekstra øving og ordner egne filer i mapper. En gang i uka viser de læreren hva de har øvd på hjemme. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 3 – Språklæringsstrategier</t>
@@ -456,13 +546,19 @@
     <t>Bruker digital teknologi strategisk og kritisk som språklæringsstrategi.</t>
   </si>
   <si>
-    <t>Læreren viser ett hjelpemiddel, for eksempel opplesning (talesyntese) eller en bildeordbok. Elevene gjør samme øvelse hver dag i en uke: skriv ordet – lytt – si ordet. Når rutinen sitter, innføres neste hjelpemiddel.</t>
-  </si>
-  <si>
-    <t>Elevene har en «verktøykasse» med kjente hjelpemidler: ordbok, tale-til-tekst og oversettelse. Ved hver skriveoppgave velger de selv hjelpemiddel og noterer hvilket de brukte og om det hjalp.</t>
-  </si>
-  <si>
-    <t>Elevene sammenligner en maskinoversettelse med sin egen tekst, finner feil i oversettelsen og forklarer når oversettelse hjelper og når den kan gi feil. De lager sammen en liste med råd om bruk av oversettelsesverktøy.</t>
+    <t xml:space="preserve">Forbered: Legg klar ordboka og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser ett hjelpemiddel, for eksempel opplesning (talesyntese) eller en bildeordbok. Elevene gjør samme øvelse hver dag i en uke: skriv ordet – lytt – si ordet. Når rutinen sitter, innføres neste hjelpemiddel. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar ordboka før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene har en «verktøykasse» med kjente hjelpemidler: ordbok, tale-til-tekst og oversettelse. Ved hver skriveoppgave velger de selv hjelpemiddel og noterer hvilket de brukte og om det hjalp. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene sammenligner en maskinoversettelse med sin egen tekst, finner feil i oversettelsen og forklarer når oversettelse hjelper og når den kan gi feil. De lager sammen en liste med råd om bruk av oversettelsesverktøy. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 3 – Resepsjon</t>
@@ -480,13 +576,19 @@
     <t>Henter informasjon fra ulike digitale kilder og vurderer den kritisk.</t>
   </si>
   <si>
-    <t>Læreren gir elevene en lenke til nettsiden til et legekontor. Elevene finner åpningstiden med støtte (læreren peker på hvor de skal se) og svarer med fast setning: «Legekontoret er åpent fra … til …».</t>
-  </si>
-  <si>
-    <t>Elevene leser en kort nyhetssak på et lettlest nettsted og lytter til lydversjonen. Etterpå svarer de på tre enkle spørsmål om hva, hvor og når.</t>
-  </si>
-  <si>
-    <t>Elevene får to nettsider om samme tema – én seriøs og én med reklame eller falsk informasjon. De sammenligner avsender, dato og formål, og begrunner hvilken side de stoler på.</t>
+    <t xml:space="preserve">Forbered: Legg klar lenken og nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren gir elevene en lenke til nettsiden til et legekontor. Elevene finner åpningstiden med støtte (læreren peker på hvor de skal se) og svarer med fast setning: «Legekontoret er åpent fra … til …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene leser en kort nyhetssak på et lettlest nettsted og lytter til lydversjonen. Etterpå svarer de på tre enkle spørsmål om hva, hvor og når. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene får to nettsider om samme tema – én seriøs og én med reklame eller falsk informasjon. De sammenligner avsender, dato og formål, og begrunner hvilken side de stoler på. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 3 – Produksjon</t>
@@ -504,13 +606,19 @@
     <t>Veksler selvstendig mellom muntlig og skriftlig på digitale flater og tilpasser til mottaker og kanal.</t>
   </si>
   <si>
-    <t>Læreren viser en modell-SMS på storskjerm: «Hei! Jeg er syk i dag. Hilsen Amina.» Elevene skriver den samme meldingen på egen mobil, bytter ut navnet og sender den til læreren. Neste dag byttes ett ord ut (syk → forsinket).</t>
-  </si>
-  <si>
-    <t>Elevene skriver én melding til en venn og én melding til en arbeidsgiver om samme sak, for eksempel at de blir forsinket. De kan skrive eller bruke tale-til-tekst. I par sammenligner de hvordan meldingene er forskjellige.</t>
-  </si>
-  <si>
-    <t>Elevene får et scenario (flytte, invitere, klage på en vare) og velger selv kanal (SMS, e-post eller talemelding) og form ut fra hvem mottakeren er. De begrunner valget sitt for partneren.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en modell-SMS på storskjerm: «Hei! Jeg er syk i dag. Hilsen Amina.» Elevene skriver den samme meldingen på egen mobil, bytter ut navnet og sender den til læreren. Neste dag byttes ett ord ut (syk → forsinket). Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver én melding til en venn og én melding til en arbeidsgiver om samme sak, for eksempel at de blir forsinket. De kan skrive eller bruke tale-til-tekst. I par sammenligner de hvordan meldingene er forskjellige. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene får et scenario (flytte, invitere, klage på en vare) og velger selv kanal (SMS, e-post eller talemelding) og form ut fra hvem mottakeren er. De begrunner valget sitt for partneren. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 3 – Samhandling</t>
@@ -531,13 +639,19 @@
     <t>Samhandler selvstendig i ulike digitale medier og bruker strategier for oppklaring.</t>
   </si>
   <si>
-    <t>Læreren sender en enkel melding i klassechatten: «Kommer du på skolen i morgen?». Elevene svarer med faste fraser fra en frasebank på tavla: «Ja, jeg kommer.» eller «Nei, jeg er syk.»</t>
-  </si>
-  <si>
-    <t>Elevene har en chat-samtale i par der de skal avtale et møte (dag, tid og sted). De bruker frasebanken ved behov, og læreren går rundt og hjelper.</t>
-  </si>
-  <si>
-    <t>Elevene får en chat med en misforståelse (feil tid eller uklar beskjed) og skal oppklare den med strategier som «Mener du …?» og «Kan du forklare?». Klassen sammenligner hvilke strategier som fungerte.</t>
+    <t xml:space="preserve">Forbered: Legg klar fraser før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren sender en enkel melding i klassechatten: «Kommer du på skolen i morgen?». Elevene svarer med faste fraser fra en frasebank på tavla: «Ja, jeg kommer.» eller «Nei, jeg er syk.». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar fraser før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene har en chat-samtale i par der de skal avtale et møte (dag, tid og sted). De bruker frasebanken ved behov, og læreren går rundt og hjelper. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene får en chat med en misforståelse (feil tid eller uklar beskjed) og skal oppklare den med strategier som «Mener du …?» og «Kan du forklare?». Klassen sammenligner hvilke strategier som fungerte. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Grunnleggende ferdigheter</t>
@@ -558,13 +672,19 @@
     <t>Overfører digitale ferdigheter selvstendig i nye norskspråklige sammenhenger.</t>
   </si>
   <si>
-    <t>Elevene viser hverandre hva de allerede kan på mobilen, for eksempel ta bilde eller sende en talemelding. Læreren bygger videre på dette: elevene tar bilde av dagens ordliste og sender det til seg selv, slik at de kan øve hjemme.</t>
-  </si>
-  <si>
-    <t>Hver uke får elevene én digital oppgave knyttet til norsktemaet. Tema bolig: finn en leilighet på Finn.no og skriv tre setninger om den («Leiligheten har … rom. Den koster …»).</t>
-  </si>
-  <si>
-    <t>Elevene bruker det de kan i nye situasjoner, for eksempel ved å legge inn avtaler på norsk i kalenderen på mobilen og sette påminnelser. De viser læreren kalenderen for neste uke.</t>
+    <t xml:space="preserve">Forbered: Legg klar mobilen og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene viser hverandre hva de allerede kan på mobilen, for eksempel ta bilde eller sende en talemelding. Læreren bygger videre på dette: elevene tar bilde av dagens ordliste og sender det til seg selv, slik at de kan øve hjemme. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Hver uke får elevene én digital oppgave knyttet til norsktemaet. Tema bolig: finn en leilighet på Finn.no og skriv tre setninger om den («Leiligheten har … rom. Den koster …»). Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar mobilen før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker det de kan i nye situasjoner, for eksempel ved å legge inn avtaler på norsk i kalenderen på mobilen og sette påminnelser. De viser læreren kalenderen for neste uke. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Digitale ferdigheter</t>
@@ -579,13 +699,19 @@
     <t>Overfører og videreutvikler digitale ferdigheter selvstendig i nye norskspråklige sammenhenger.</t>
   </si>
   <si>
-    <t>Elevene tar opp seg selv på mobilen mens de sier tre setninger om seg selv. Læreren gir en modell først. Elevene lytter til opptaket, prøver igjen og velger det beste opptaket.</t>
-  </si>
-  <si>
-    <t>Hver uke sender elevene en talemelding på norsk til en fast medelev om et gitt tema (f.eks. «Helgen min»), og svarer på medelevens melding. Læreren gir spørsmål som støtte.</t>
-  </si>
-  <si>
-    <t>Elevene lager et kort lydopptak eller en video om et tema, bruker tale-til-tekst for å sjekke om uttalen blir forstått, og deler produktet med klassen for tilbakemelding.</t>
+    <t xml:space="preserve">Forbered: Legg klar mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene tar opp seg selv på mobilen mens de sier tre setninger om seg selv. Læreren gir en modell først. Elevene lytter til opptaket, prøver igjen og velger det beste opptaket. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Hver uke sender elevene en talemelding på norsk til en fast medelev om et gitt tema (f.eks. «Helgen min»), og svarer på medelevens melding. Læreren gir spørsmål som støtte. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene lager et kort lydopptak eller en video om et tema, bruker tale-til-tekst for å sjekke om uttalen blir forstått, og deler produktet med klassen for tilbakemelding. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Digitale ferdigheter integreres der det er relevant for deltakerens nivå og behov.</t>
@@ -600,13 +726,19 @@
     <t>Bruker digitale ferdigheter selvstendig som integrert del av alle språkferdighetene.</t>
   </si>
   <si>
-    <t>I temaet «Å handle» skriver elevene en handleliste i notatappen på mobilen. Læreren gir ord med bilder, og elevene skriver av med støtte.</t>
-  </si>
-  <si>
-    <t>I hvert tema er én oppgave digital for hver ferdighet: lytte (lydklipp), lese (nettside), skrive (melding) og snakke (opptak). Elevene roterer mellom stasjoner, og hver stasjon har en oppgavebeskrivelse med ikoner.</t>
-  </si>
-  <si>
-    <t>Elevene velger selv digitale verktøy som støtter arbeidet i alle ferdigheter, for eksempel opptak for muntlig trening og stavekontroll for skriving, og forklarer valgene sine for læreren.</t>
+    <t xml:space="preserve">Forbered: Legg klar mobilen og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: I temaet «Å handle» skriver elevene en handleliste i notatappen på mobilen. Læreren gir ord med bilder, og elevene skriver av med støtte. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: I hvert tema er én oppgave digital for hver ferdighet: lytte (lydklipp), lese (nettside), skrive (melding) og snakke (opptak). Elevene roterer mellom stasjoner, og hver stasjon har en oppgavebeskrivelse med ikoner. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene velger selv digitale verktøy som støtter arbeidet i alle ferdigheter, for eksempel opptak for muntlig trening og stavekontroll for skriving, og forklarer valgene sine for læreren. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Bruke digitale ressurser til samhandling, informasjonssøk, tekstskaping og dokumentasjon.</t>
@@ -624,13 +756,19 @@
     <t>Bruker digitale ressurser selvstendig til samhandling, søk, tekstskaping og til å dokumentere kompetanse.</t>
   </si>
   <si>
-    <t>Elevene får ett søkeord og en anvist nettside. De finner et bilde som passer, limer det inn i et delt klassedokument og skriver én setning under. Læreren viser hvert trinn på storskjerm.</t>
-  </si>
-  <si>
-    <t>I par finner elevene informasjon om et sted i byen, lager et delt dokument med tekst og bilde, og presenterer det for klassen på ett–to lysbilder.</t>
-  </si>
-  <si>
-    <t>Elevene lager en digital mappe med tekster, lydopptak og skjermbilder som viser hva de kan. De bruker mappen i samtale med læreren, og kan senere vise den til en arbeidsgiver.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, nettsiden og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene får ett søkeord og en anvist nettside. De finner et bilde som passer, limer det inn i et delt klassedokument og skriver én setning under. Læreren viser hvert trinn på storskjerm. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: I par finner elevene informasjon om et sted i byen, lager et delt dokument med tekst og bilde, og presenterer det for klassen på ett–to lysbilder. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene lager en digital mappe med tekster, lydopptak og skjermbilder som viser hva de kan. De bruker mappen i samtale med læreren, og kan senere vise den til en arbeidsgiver. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Håndtere digitale hverdagsoppgaver på norsk.</t>
@@ -645,13 +783,19 @@
     <t>Håndterer nye og ukjente digitale tjenester på norsk selvstendig.</t>
   </si>
   <si>
-    <t>Læreren viser et skjermbilde av en beskjed fra skole eller barnehage i en app. Elevene markerer hva, når og hvor med tre farger. Deretter øver de på å betale med app i en demo- eller øvingsversjon.</t>
-  </si>
-  <si>
-    <t>Stasjonsarbeid med hverdagsoppgaver: sjekke busstider, lese en beskjed fra barnehagen og finne åpningstider på apoteket. Elevene løser oppgavene i par og hjelper hverandre.</t>
-  </si>
-  <si>
-    <t>Elevene prøver en tjeneste de ikke har brukt før, for eksempel å reservere en bok på biblioteket eller bestille time hos frisør. De forteller klassen hvordan de fant ut av tjenesten.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et skjermbilde av en beskjed fra skole eller barnehage i en app. Elevene markerer hva, når og hvor med tre farger. Deretter øver de på å betale med app i en demo- eller øvingsversjon. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Stasjonsarbeid med hverdagsoppgaver: sjekke busstider, lese en beskjed fra barnehagen og finne åpningstider på apoteket. Elevene løser oppgavene i par og hjelper hverandre. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene prøver en tjeneste de ikke har brukt før, for eksempel å reservere en bok på biblioteket eller bestille time hos frisør. De forteller klassen hvordan de fant ut av tjenesten. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Utvikle digital dømmekraft og strategier for nettbruk.</t>
@@ -666,13 +810,19 @@
     <t>Viser selvstendig digital dømmekraft og vurderer digitale verktøy kritisk ut fra formål.</t>
   </si>
   <si>
-    <t>Læreren viser et eksempel på en svindel-SMS («Du har vunnet en iPhone! Trykk her»). Klassen lærer regelen: «Ikke trykk på lenker du ikke kjenner. Spør noen først.» Elevene øver med ekte og falske meldinger og viser tommel opp eller ned.</t>
-  </si>
-  <si>
-    <t>Elevene får fem meldinger og e-poster og sorterer dem i «trygg» og «svindel» ved hjelp av en sjekkliste: Hvem er avsender? Er det en lenke? Haster det veldig?</t>
-  </si>
-  <si>
-    <t>Elevene lager en kort guide om trygg nettbruk til familie eller venner. De vurderer også to verktøy for samme oppgave (f.eks. to oversettelsesapper) ut fra hva de skal brukes til og hvordan de behandler personopplysninger.</t>
+    <t xml:space="preserve">Forbered: Legg klar lenken før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et eksempel på en svindel-SMS («Du har vunnet en iPhone! Trykk her»). Klassen lærer regelen: «Ikke trykk på lenker du ikke kjenner. Spør noen først.» Elevene øver med ekte og falske meldinger og viser tommel opp eller ned. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten, et e-posteksempel og lenken før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får fem meldinger og e-poster og sorterer dem i «trygg» og «svindel» ved hjelp av en sjekkliste: Hvem er avsender? Er det en lenke? Haster det veldig? Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene lager en kort guide om trygg nettbruk til familie eller venner. De vurderer også to verktøy for samme oppgave (f.eks. to oversettelsesapper) ut fra hva de skal brukes til og hvordan de behandler personopplysninger. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – Lese- og skriveforberedende</t>
@@ -693,13 +843,19 @@
     <t>Skriver bokstaver og kjente ord selvstendig og med økende tempo på tastatur.</t>
   </si>
   <si>
-    <t>Elevene finner bokstavene i sitt eget navn på tastaturet ved hjelp av et tastaturkart med store bokstaver. Deretter sier læreren en lyd, og elevene finner og trykker på bokstaven.</t>
-  </si>
-  <si>
-    <t>Elevene skriver ord fra dagens tema etter ordkort med bilder, og øver på stor forbokstav med shift-tasten. Partneren sjekker at ordene er riktige.</t>
-  </si>
-  <si>
-    <t>Elevene skriver kjente ord i et tastaturspill eller skriveprogram med tidtaking, og prøver å slå sin egen rekord fra forrige uke.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene finner bokstavene i sitt eget navn på tastaturet ved hjelp av et tastaturkart med store bokstaver. Deretter sier læreren en lyd, og elevene finner og trykker på bokstaven. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver ord fra dagens tema etter ordkort med bilder, og øver på stor forbokstav med shift-tasten. Partneren sjekker at ordene er riktige. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene skriver kjente ord i et tastaturspill eller skriveprogram med tidtaking, og prøver å slå sin egen rekord fra forrige uke. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Gjenkjenne ord og symboler i digitale tekster (animasjon, reklame).</t>
@@ -714,13 +870,19 @@
     <t>Leser og tolker ord og symboler i varierte digitale tekster selvstendig.</t>
   </si>
   <si>
-    <t>Læreren viser en kort reklamefilm eller animasjon og stopper filmen underveis. Elevene peker på kjente symboler (pris, %, logo) og ord («Tilbud», «Salg») som læreren har vist på forhånd.</t>
-  </si>
-  <si>
-    <t>Elevene blar i en digital tilbudsavis og markerer ord de kjenner igjen. De viser partneren tre ord og sier dem høyt.</t>
-  </si>
-  <si>
-    <t>Elevene ser på ulike digitale tekster – reklame, en advarsel i en app og en informasjonsanimasjon – og forklarer hva ord og symboler betyr.</t>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en kort reklamefilm eller animasjon og stopper filmen underveis. Elevene peker på kjente symboler (pris, %, logo) og ord («Tilbud», «Salg») som læreren har vist på forhånd. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene blar i en digital tilbudsavis og markerer ord de kjenner igjen. De viser partneren tre ord og sier dem høyt. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene ser på ulike digitale tekster – reklame, en advarsel i en app og en informasjonsanimasjon – og forklarer hva ord og symboler betyr. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – Grunnleggende lesing</t>
@@ -738,13 +900,19 @@
     <t>Gjør relevante valg selvstendig i apper, automater og enkle nettsider nødvendige i dagliglivet.</t>
   </si>
   <si>
-    <t>Ikonbingo: Læreren viser et ikon på storskjerm (hjem, søk, tilbake, send, meny) og sier ordet. Elevene finner ikonet på bingobrettet og deretter på egen mobil. Til slutt trykker de på riktig ikon når læreren bare sier ordet.</t>
-  </si>
-  <si>
-    <t>Elevene kjøper en bussbillett i en kjent app trinn for trinn ved hjelp av oppgavekort med skjermbilder. Læreren hjelper ved behov.</t>
-  </si>
-  <si>
-    <t>Elevene løser dagligdagse oppgaver på egen hånd: finne været for i morgen, kjøpe billett i en app og sjekke saldo i nettbanken. De forteller hvilke valg de gjorde.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Ikonbingo: Læreren viser et ikon på storskjerm (hjem, søk, tilbake, send, meny) og sier ordet. Elevene finner ikonet på bingobrettet og deretter på egen mobil. Til slutt trykker de på riktig ikon når læreren bare sier ordet. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene kjøper en bussbillett i en kjent app trinn for trinn ved hjelp av oppgavekort med skjermbilder. Læreren hjelper ved behov. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene løser dagligdagse oppgaver på egen hånd: finne været for i morgen, kjøpe billett i en app og sjekke saldo i nettbanken. De forteller hvilke valg de gjorde. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – Grunnleggende skriving</t>
@@ -762,13 +930,19 @@
     <t>Kommenterer innlegg selvstendig og viser bevissthet om passende innhold.</t>
   </si>
   <si>
-    <t>Læreren legger ut et bilde i en lukket klassegruppe, for eksempel av en matrett. Elevene reagerer med emoji og ett ord, for eksempel «Fint!» eller «Nam!».</t>
-  </si>
-  <si>
-    <t>Elevene legger ut et bilde hver og kommenterer hverandres bilder med faste fraser: «Så fint!», «Hvor er det?», «Jeg liker …».</t>
-  </si>
-  <si>
-    <t>Elevene kommenterer innlegg selvstendig. Klassen diskuterer hva som er passende å skrive offentlig og hva som hører hjemme i private meldinger.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren legger ut et bilde i en lukket klassegruppe, for eksempel av en matrett. Elevene reagerer med emoji og ett ord, for eksempel «Fint!» eller «Nam!». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene legger ut et bilde hver og kommenterer hverandres bilder med faste fraser: «Så fint!», «Hvor er det?», «Jeg liker …». Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene kommenterer innlegg selvstendig. Klassen diskuterer hva som er passende å skrive offentlig og hva som hører hjemme i private meldinger. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Fylle inn personlige opplysninger i enkle digitale skjema.</t>
@@ -783,13 +957,19 @@
     <t>Fyller inn personlige opplysninger på riktig sted i enkle digitale skjema og sender inn selvstendig.</t>
   </si>
   <si>
-    <t>Læreren lager et enkelt digitalt skjema med feltene navn og telefonnummer. Elevene har et kort med egne opplysninger og fyller inn felt for felt mens læreren viser på storskjerm.</t>
-  </si>
-  <si>
-    <t>Skjemaet utvides med adresse og fødselsdato. Elevene øver på riktige formater (dd.mm.åååå, postnummer) og fyller ut skjemaet i par.</t>
-  </si>
-  <si>
-    <t>Elevene fyller inn et ekte skjema, for eksempel påmelding til et bibliotekarrangement, sjekker opplysningene og sender det inn selv.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, skjemaet og kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren lager et enkelt digitalt skjema med feltene navn og telefonnummer. Elevene har et kort med egne opplysninger og fyller inn felt for felt mens læreren viser på storskjerm. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Skjemaet utvides med adresse og fødselsdato. Elevene øver på riktige formater (dd.mm.åååå, postnummer) og fyller ut skjemaet i par. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene fyller inn et ekte skjema, for eksempel påmelding til et bibliotekarrangement, sjekker opplysningene og sender det inn selv. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Videreformidle informasjon fra enkle digitale og visuelle tekster.</t>
@@ -804,13 +984,19 @@
     <t>Videreformidler muntlig relevant informasjon fra enkle digitale tekster selvstendig.</t>
   </si>
   <si>
-    <t>Læreren viser en kort animasjon med lite tekst og stopper den underveis: «Hva ser du?». Elevene peker på skjermen og sier ett–to ord.</t>
-  </si>
-  <si>
-    <t>Elevene ser en kort reklamefilm og gjenforteller med bildestøtte og setningsstartere: «Det er en reklame for … Den koster …».</t>
-  </si>
-  <si>
-    <t>Elevene ser en kort informasjonsvideo, for eksempel fra kommunen, og forteller partneren det viktigste. Partneren sjekker mot videoen.</t>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en kort animasjon med lite tekst og stopper den underveis: «Hva ser du?». Elevene peker på skjermen og sier ett–to ord. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar setningsstartere, bilder og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene ser en kort reklamefilm og gjenforteller med bildestøtte og setningsstartere: «Det er en reklame for … Den koster …». Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene ser en kort informasjonsvideo, for eksempel fra kommunen, og forteller partneren det viktigste. Partneren sjekker mot videoen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A1 lytte</t>
@@ -828,13 +1014,19 @@
     <t>Finner og bruker enkle digitale lytte-/videoressurser selvstendig.</t>
   </si>
   <si>
-    <t>Læreren spiller korte digitale klipp med tall og ukedager flere ganger. Elevene holder opp kort med ordet eller tallet de hører.</t>
-  </si>
-  <si>
-    <t>Elevene spiller av korte klipp på egen PC med hodetelefoner i sitt eget tempo, og krysser av informasjonen de hører på et arbeidsark.</t>
-  </si>
-  <si>
-    <t>Elevene finner selv lyttestoff på et anbefalt nettsted på sitt nivå og lager en liste over ord og informasjon de forsto.</t>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren spiller korte digitale klipp med tall og ukedager flere ganger. Elevene holder opp kort med ordet eller tallet de hører. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene spiller av korte klipp på egen PC med hodetelefoner i sitt eget tempo, og krysser av informasjonen de hører på et arbeidsark. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene finner selv lyttestoff på et anbefalt nettsted på sitt nivå og lager en liste over ord og informasjon de forsto. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Skrive ved bruk av tilpassede dataprogrammer og apper.</t>
@@ -849,13 +1041,19 @@
     <t>Skriver selvstendig i tilpassede dataprogrammer og bruker støttefunksjoner hensiktsmessig.</t>
   </si>
   <si>
-    <t>Elevene bruker en skriveapp som sier bokstavene høyt, og skriver ord til bilder. Læreren sitter ved og viser.</t>
-  </si>
-  <si>
-    <t>Elevene skriver korte tekster i et tekstprogram og øver på å lagre filen og rette feil med stavekontrollen.</t>
-  </si>
-  <si>
-    <t>Elevene bruker støttefunksjoner som ordforslag, opplesning og stavekontroll, og vurderer når de hjelper og når de ikke gjør det.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene bruker en skriveapp som sier bokstavene høyt, og skriver ord til bilder. Læreren sitter ved og viser. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver korte tekster i et tekstprogram og øver på å lagre filen og rette feil med stavekontrollen. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker støttefunksjoner som ordforslag, opplesning og stavekontroll, og vurderer når de hjelper og når de ikke gjør det. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A1 lese</t>
@@ -876,13 +1074,19 @@
     <t>Navigerer selvstendig på enkle autentiske nettsider og finner ord og fraser.</t>
   </si>
   <si>
-    <t>Læreren åpner nettsiden til en matbutikk på storskjerm. Elevene finner kjente ord (melk, brød, epler) og navn, og kommer fram og peker.</t>
-  </si>
-  <si>
-    <t>Elevene åpner selv en kjent nettside (bibliotek eller kommune) og finner fem kjente ord eller fraser, som de skriver i en liste.</t>
-  </si>
-  <si>
-    <t>Elevene navigerer på enkle autentiske nettsider for å finne åpningstider, priser eller tilbud, og noterer det de finner.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren åpner nettsiden til en matbutikk på storskjerm. Elevene finner kjente ord (melk, brød, epler) og navn, og kommer fram og peker. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene åpner selv en kjent nettside (bibliotek eller kommune) og finner fem kjente ord eller fraser, som de skriver i en liste. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene navigerer på enkle autentiske nettsider for å finne åpningstider, priser eller tilbud, og noterer det de finner. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A1 skrive</t>
@@ -900,13 +1104,19 @@
     <t>Skriver og kommenterer enkle innlegg selvstendig og bruker passende hilsen/avslutning.</t>
   </si>
   <si>
-    <t>Læreren viser en modell: «Hei! I dag spiser jeg fisk.» Elevene skriver et eget innlegg på én–to setninger i den lukkede klassegruppen.</t>
-  </si>
-  <si>
-    <t>Elevene skriver et innlegg om helgen og kommenterer to av medelevenes innlegg.</t>
-  </si>
-  <si>
-    <t>Elevene skriver og kommenterer innlegg med passende hilsen og avslutning, og tilpasser språket til hvem som skal lese det.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en modell: «Hei! I dag spiser jeg fisk.» Elevene skriver et eget innlegg på én–to setninger i den lukkede klassegruppen. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver et innlegg om helgen og kommenterer to av medelevenes innlegg. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene skriver og kommenterer innlegg med passende hilsen og avslutning, og tilpasser språket til hvem som skal lese det. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Fylle inn personlige opplysninger i nettskjemaer og apper.</t>
@@ -921,13 +1131,19 @@
     <t>Fyller inn og sender inn enkle nettskjemaer selvstendig og kontrollerer opplysningene.</t>
   </si>
   <si>
-    <t>Læreren viser et nettskjema på storskjerm. Elevene fyller inn felt for felt ved hjelp av eget kort med personopplysninger, mens læreren viser hvert felt.</t>
-  </si>
-  <si>
-    <t>Elevene registrerer seg i en app (f.eks. bibliotekets app) ved hjelp av oppgavekort med skjermbilder.</t>
-  </si>
-  <si>
-    <t>Elevene fyller inn og sender inn skjemaer selv, og kontrollerer opplysningene mot en sjekkliste før de trykker «send».</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, skjemaet og kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et nettskjema på storskjerm. Elevene fyller inn felt for felt ved hjelp av eget kort med personopplysninger, mens læreren viser hvert felt. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene registrerer seg i en app (f.eks. bibliotekets app) ved hjelp av oppgavekort med skjermbilder. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten og skjemaet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene fyller inn og sender inn skjemaer selv, og kontrollerer opplysningene mot en sjekkliste før de trykker «send». Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A2 lese</t>
@@ -945,13 +1161,19 @@
     <t>Søker selvstendig på nett og finner og forstår spesifikk informasjon.</t>
   </si>
   <si>
-    <t>Læreren gir et søkeord og en nettside: «Finn prisen på en liter melk.» Elevene søker og skriver svaret.</t>
-  </si>
-  <si>
-    <t>Elevene bruker søkefeltet og menyene på en kjent nettside for å finne informasjon, for eksempel åpningstidene til svømmehallen.</t>
-  </si>
-  <si>
-    <t>Elevene får oppgaven «Planlegg en tur på lørdag». De søker selv etter tider, priser og værmelding, og forteller partneren planen.</t>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren gir et søkeord og en nettside: «Finn prisen på en liter melk.» Elevene søker og skriver svaret. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker søkefeltet og menyene på en kjent nettside for å finne informasjon, for eksempel åpningstidene til svømmehallen. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene får oppgaven «Planlegg en tur på lørdag». De søker selv etter tider, priser og værmelding, og forteller partneren planen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A2 skrive</t>
@@ -969,13 +1191,19 @@
     <t>Skriver, svarer og kommenterer enkelt selvstendig i digital kommunikasjon.</t>
   </si>
   <si>
-    <t>Elevene får en invitasjon i en melding: «Vil du komme på kaffe på lørdag?». De svarer ved hjelp av en modell: «Ja, takk! Jeg kommer klokka …».</t>
-  </si>
-  <si>
-    <t>Elevene skriver og svarer på meldinger i klassekanalen om en felles aktivitet, for eksempel en tur eller et spleiselag.</t>
-  </si>
-  <si>
-    <t>Elevene svarer og kommenterer selvstendig, også på meldinger de ikke har forberedt seg på.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene får en invitasjon i en melding: «Vil du komme på kaffe på lørdag?». De svarer ved hjelp av en modell: «Ja, takk! Jeg kommer klokka …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver og svarer på meldinger i klassekanalen om en felles aktivitet, for eksempel en tur eller et spleiselag. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene svarer og kommenterer selvstendig, også på meldinger de ikke har forberedt seg på. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Skrive korte og enkle e-poster og personlige brev.</t>
@@ -990,13 +1218,19 @@
     <t>Skriver og sender enkle e-poster selvstendig, også med vedlegg.</t>
   </si>
   <si>
-    <t>Elevene skriver en e-post etter mal («Hei …, jeg …, Hilsen …») med støtte fra læreren, og sender den til læreren.</t>
-  </si>
-  <si>
-    <t>Elevene skriver en e-post til læreren om fravær. De øver på å skrive inn riktig mottaker, emnefelt og innhold.</t>
-  </si>
-  <si>
-    <t>Elevene skriver og sender en e-post med vedlegg, for eksempel et bilde eller et dokument, og sjekker at vedlegget kom fram.</t>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene skriver en e-post etter mal («Hei …, jeg …, Hilsen …») med støtte fra læreren, og sender den til læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver en e-post til læreren om fravær. De øver på å skrive inn riktig mottaker, emnefelt og innhold. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel og bilder før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene skriver og sender en e-post med vedlegg, for eksempel et bilde eller et dokument, og sjekker at vedlegget kom fram. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Fylle inn opplysninger i digitale skjemaer (netthandel, bank, bestillinger).</t>
@@ -1011,13 +1245,19 @@
     <t>Bruker digitale tjenester selvstendig (netthandel, bank, bestilling, påmelding).</t>
   </si>
   <si>
-    <t>Læreren bruker en øvingsnettbutikk på storskjerm. Elevene fyller inn navn og adresse i bestillingsskjemaet med veiledning.</t>
-  </si>
-  <si>
-    <t>Elevene bestiller en vare i øvingsnettbutikken eller melder seg på et kurs, og viser partneren bekreftelsen.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale tjenester selvstendig, for eksempel for å bestille time eller melde seg på en aktivitet, og forteller klassen hvordan de gjorde det.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og skjemaet før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren bruker en øvingsnettbutikk på storskjerm. Elevene fyller inn navn og adresse i bestillingsskjemaet med veiledning. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bestiller en vare i øvingsnettbutikken eller melder seg på et kurs, og viser partneren bekreftelsen. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale tjenester selvstendig, for eksempel for å bestille time eller melde seg på en aktivitet, og forteller klassen hvordan de gjorde det. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Presentere egen kompetanse i en enkel CV og digitalt skjema.</t>
@@ -1032,13 +1272,19 @@
     <t>Presenterer egen kompetanse selvstendig i digital CV og oppdaterer ved behov.</t>
   </si>
   <si>
-    <t>Elevene fyller inn en enkel CV-mal (navn, adresse, språk, erfaring) med hjelp fra læreren. Læreren viser en ferdig CV som modell.</t>
-  </si>
-  <si>
-    <t>Elevene lager en CV i et tekstprogram og fyller inn et digitalt kompetanseskjema. Partneren leser og gir én tilbakemelding.</t>
-  </si>
-  <si>
-    <t>Elevene oppdaterer sin egen CV og tilpasser den til en ekte stillingsannonse de har funnet.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene fyller inn en enkel CV-mal (navn, adresse, språk, erfaring) med hjelp fra læreren. Læreren viser en ferdig CV som modell. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene lager en CV i et tekstprogram og fyller inn et digitalt kompetanseskjema. Partneren leser og gir én tilbakemelding. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene oppdaterer sin egen CV og tilpasser den til en ekte stillingsannonse de har funnet. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A2 muntlig</t>
@@ -1056,13 +1302,19 @@
     <t>Lager og bruker digitale verktøy selvstendig i presentasjon.</t>
   </si>
   <si>
-    <t>Elevene lager sammen med læreren to–tre lysbilder om seg selv (ett bilde og én setning per lysbilde) og presenterer for en liten gruppe.</t>
-  </si>
-  <si>
-    <t>Elevene lager lysbilder selv om hjemlandet eller en hobby, og bruker dem i en kort presentasjon for klassen.</t>
-  </si>
-  <si>
-    <t>Elevene velger selv presentasjonsverktøy, lager en presentasjon med bilder og tekst og presenterer for klassen.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene lager sammen med læreren to–tre lysbilder om seg selv (ett bilde og én setning per lysbilde) og presenterer for en liten gruppe. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene lager lysbilder selv om hjemlandet eller en hobby, og bruker dem i en kort presentasjon for klassen. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene velger selv presentasjonsverktøy, lager en presentasjon med bilder og tekst og presenterer for klassen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B1 lese</t>
@@ -1080,13 +1332,19 @@
     <t>Søker selvstendig på tvers av nettsider og digitale dokumenter.</t>
   </si>
   <si>
-    <t>Læreren viser helsenorge.no på storskjerm. Elevene finner informasjon om hvordan man bytter fastlege, med veiledning trinn for trinn.</t>
-  </si>
-  <si>
-    <t>Elevene får oppgavekort med spørsmål om rettigheter (f.eks. barnetrygd eller foreldrepenger) og søker etter svar på nav.no og andre offentlige nettsider.</t>
-  </si>
-  <si>
-    <t>Elevene løser et praktisk problem, for eksempel «Du skal flytte – hva må du gjøre?». De søker på tvers av offentlige nettsider og dokumenter og lager en sjekkliste.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser helsenorge.no på storskjerm. Elevene finner informasjon om hvordan man bytter fastlege, med veiledning trinn for trinn. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får oppgavekort med spørsmål om rettigheter (f.eks. barnetrygd eller foreldrepenger) og søker etter svar på nav.no og andre offentlige nettsider. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten og nettsiden før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene løser et praktisk problem, for eksempel «Du skal flytte – hva må du gjøre?». De søker på tvers av offentlige nettsider og dokumenter og lager en sjekkliste. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B1 skrive</t>
@@ -1104,13 +1362,19 @@
     <t>Deltar selvstendig i digitale diskusjoner med saklig tone og respekt.</t>
   </si>
   <si>
-    <t>Elevene skriver et innlegg og en kommentar i et lukket digitalt forum ved hjelp av setningsstartere som «Jeg mener at …» og «Jeg er enig fordi …».</t>
-  </si>
-  <si>
-    <t>Elevene deltar i en digital diskusjon om et hverdagstema og svarer på minst to medelevers innlegg.</t>
-  </si>
-  <si>
-    <t>Elevene deltar selvstendig i digitale diskusjoner med saklig tone, og vurderer etterpå sin egen tone ut fra klassens regler.</t>
+    <t xml:space="preserve">Forbered: Legg klar setningsstartere før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene skriver et innlegg og en kommentar i et lukket digitalt forum ved hjelp av setningsstartere som «Jeg mener at …» og «Jeg er enig fordi …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene deltar i en digital diskusjon om et hverdagstema og svarer på minst to medelevers innlegg. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene deltar selvstendig i digitale diskusjoner med saklig tone, og vurderer etterpå sin egen tone ut fra klassens regler. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Skrive enkle formelle e-poster.</t>
@@ -1125,13 +1389,19 @@
     <t>Skriver og sender formelle e-poster med vedlegg selvstendig.</t>
   </si>
   <si>
-    <t>Elevene skriver en enkel formell e-post etter mal, for eksempel til en arbeidsgiver for å spørre om praksisplass. Læreren viser hvordan en formell e-post skiller seg fra en SMS.</t>
-  </si>
-  <si>
-    <t>Elevene skriver en formell e-post og legger ved CV eller søknad. Partneren sjekker hilsen, emnefelt og vedlegg.</t>
-  </si>
-  <si>
-    <t>Elevene skriver og sender formelle e-poster med vedlegg selvstendig, for eksempel til en ekte arbeidsgiver eller til NAV.</t>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene skriver en enkel formell e-post etter mal, for eksempel til en arbeidsgiver for å spørre om praksisplass. Læreren viser hvordan en formell e-post skiller seg fra en SMS. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver en formell e-post og legger ved CV eller søknad. Partneren sjekker hilsen, emnefelt og vedlegg. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene skriver og sender formelle e-poster med vedlegg selvstendig, for eksempel til en ekte arbeidsgiver eller til NAV. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Skrive inn opplysninger i ulike typer digitale skjemaer.</t>
@@ -1146,13 +1416,19 @@
     <t>Håndterer ulike typer digitale skjema i offentlige og private tjenester selvstendig.</t>
   </si>
   <si>
-    <t>Elevene fyller ut et lengre digitalt skjema (f.eks. en søknad) med veiledning fra læreren. Læreren viser hvert felt og forklarer ukjente ord.</t>
-  </si>
-  <si>
-    <t>Elevene øver på å logge inn med BankID og laste opp et dokument i et øvingsskjema eller en ekte tjeneste.</t>
-  </si>
-  <si>
-    <t>Elevene fyller ut ulike skjemaer selv, både i offentlige og private tjenester, og forteller hva som var vanskelig.</t>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene fyller ut et lengre digitalt skjema (f.eks. en søknad) med veiledning fra læreren. Læreren viser hvert felt og forklarer ukjente ord. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene øver på å logge inn med BankID og laste opp et dokument i et øvingsskjema eller en ekte tjeneste. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene fyller ut ulike skjemaer selv, både i offentlige og private tjenester, og forteller hva som var vanskelig. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B1 muntlig</t>
@@ -1170,13 +1446,19 @@
     <t>Velger og bruker digitale presentasjonsverktøy selvstendig og hensiktsmessig.</t>
   </si>
   <si>
-    <t>Elevene lager en presentasjon med lysbilder etter en mal og holder den med støtte fra læreren.</t>
-  </si>
-  <si>
-    <t>Elevene lager en strukturert presentasjon med tekst, bilder og lyd eller video, og holder den for klassen.</t>
-  </si>
-  <si>
-    <t>Elevene velger selv presentasjonsverktøy og bruker det hensiktsmessig i en presentasjon for klassen.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene lager en presentasjon med lysbilder etter en mal og holder den med støtte fra læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene lager en strukturert presentasjon med tekst, bilder og lyd eller video, og holder den for klassen. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene velger selv presentasjonsverktøy og bruker det hensiktsmessig i en presentasjon for klassen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B2 lese</t>
@@ -1194,13 +1476,19 @@
     <t>Bruker søketeknikker og lesemåter selvstendig og effektivt på tvers av nettsteder.</t>
   </si>
   <si>
-    <t>Læreren viser hvordan søkeord og enkle filtre (dato, sted) virker. Elevene øver på samme søk med veiledning.</t>
-  </si>
-  <si>
-    <t>Elevene øver på ulike søketeknikker og skumlesing: de får fem spørsmål og skal finne svarene så raskt som mulig på ulike nettsider.</t>
-  </si>
-  <si>
-    <t>Elevene bruker søketeknikker og lesemåter selvstendig for å løse en sammensatt oppgave, for eksempel å sammenligne tre kurs eller tre boliger.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser hvordan søkeord og enkle filtre (dato, sted) virker. Elevene øver på samme søk med veiledning. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene øver på ulike søketeknikker og skumlesing: de får fem spørsmål og skal finne svarene så raskt som mulig på ulike nettsider. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker søketeknikker og lesemåter selvstendig for å løse en sammensatt oppgave, for eksempel å sammenligne tre kurs eller tre boliger. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B2 skrive</t>
@@ -1221,13 +1509,19 @@
     <t>Deltar selvstendig i digitale diskusjoner med nyansert argumentasjon.</t>
   </si>
   <si>
-    <t>Elevene uttrykker meninger i et lukket forum med støtte fra en frasebank med nyanserte uttrykk: «På den ene siden …, på den andre siden …».</t>
-  </si>
-  <si>
-    <t>Elevene diskuterer og kommenterer i et digitalt forum om en aktuell sak, og bruker minst ett argument og ett motargument.</t>
-  </si>
-  <si>
-    <t>Elevene deltar i en digital diskusjon med nyansert argumentasjon og viser til kilder.</t>
+    <t xml:space="preserve">Forbered: Legg klar fraser før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene uttrykker meninger i et lukket forum med støtte fra en frasebank med nyanserte uttrykk: «På den ene siden …, på den andre siden …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene diskuterer og kommenterer i et digitalt forum om en aktuell sak, og bruker minst ett argument og ett motargument. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene deltar i en digital diskusjon med nyansert argumentasjon og viser til kilder. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Skrive detaljerte beskjeder, e-poster og brev.</t>
@@ -1242,13 +1536,19 @@
     <t>Skriver selvstendig detaljerte e-poster tilpasset mottaker og formål.</t>
   </si>
   <si>
-    <t>Elevene skriver en detaljert e-post etter modell, for eksempel en klage på en vare, med støtte fra læreren.</t>
-  </si>
-  <si>
-    <t>Elevene skriver en detaljert e-post tilpasset mottakeren, for eksempel til utleier om en skade i leiligheten.</t>
-  </si>
-  <si>
-    <t>Elevene skriver selvstendig detaljerte e-poster tilpasset mottaker og formål, og vurderer tone og innhold i etterkant.</t>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene skriver en detaljert e-post etter modell, for eksempel en klage på en vare, med støtte fra læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver en detaljert e-post tilpasset mottakeren, for eksempel til utleier om en skade i leiligheten. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene skriver selvstendig detaljerte e-poster tilpasset mottaker og formål, og vurderer tone og innhold i etterkant. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B2 muntlig</t>
@@ -1266,13 +1566,19 @@
     <t>Bruker digitale verktøy selvstendig og profesjonelt i presentasjoner.</t>
   </si>
   <si>
-    <t>Elevene holder en velstrukturert presentasjon med digitale lysbilder etter mal (innledning – hoveddel – avslutning).</t>
-  </si>
-  <si>
-    <t>Elevene lager selv en velstrukturert digital presentasjon om et fagtema og får tilbakemelding fra medelever.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale verktøy selvstendig og profesjonelt i en presentasjon, for eksempel i en rollespilt jobbsituasjon.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene holder en velstrukturert presentasjon med digitale lysbilder etter mal (innledning – hoveddel – avslutning). Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene lager selv en velstrukturert digital presentasjon om et fagtema og får tilbakemelding fra medelever. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale verktøy selvstendig og profesjonelt i en presentasjon, for eksempel i en rollespilt jobbsituasjon. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A2 lytte</t>
@@ -1290,13 +1596,19 @@
     <t>Forstår enkel informasjon i digitale presentasjoner og kan notere stikkord.</t>
   </si>
   <si>
-    <t>Læreren holder en enkel digital presentasjon med tydelige bilder og stopper ofte. Elevene svarer på ja/nei-spørsmål.</t>
-  </si>
-  <si>
-    <t>Elevene ser en kort digital presentasjon eller video og svarer på spørsmål om det viktigste innholdet.</t>
-  </si>
-  <si>
-    <t>Elevene ser en digital presentasjon og noterer stikkord, som de bruker til å fortelle partneren om innholdet.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren holder en enkel digital presentasjon med tydelige bilder og stopper ofte. Elevene svarer på ja/nei-spørsmål. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene ser en kort digital presentasjon eller video og svarer på spørsmål om det viktigste innholdet. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene ser en digital presentasjon og noterer stikkord, som de bruker til å fortelle partneren om innholdet. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Oppfatte viktig informasjon fra korte digitale klipp.</t>
@@ -1311,13 +1623,19 @@
     <t>Bruker nyhets- og videotjenester selvstendig for å holde seg informert.</t>
   </si>
   <si>
-    <t>Læreren spiller av et kort klipp, for eksempel en værmelding, to–tre ganger. Elevene finner viktig informasjon (temperatur, vær) med bildestøtte.</t>
-  </si>
-  <si>
-    <t>Elevene finner og spiller av korte klipp selv fra kjente kilder, for eksempel NRK, og forteller partneren hva klippet handlet om.</t>
-  </si>
-  <si>
-    <t>Elevene bruker nyhets- og videotjenester selvstendig for å følge med på nyheter, og forteller om én nyhet i klassen hver uke.</t>
+    <t xml:space="preserve">Forbered: Legg klar klippet, bilder og kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren spiller av et kort klipp, for eksempel en værmelding, to–tre ganger. Elevene finner viktig informasjon (temperatur, vær) med bildestøtte. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene finner og spiller av korte klipp selv fra kjente kilder, for eksempel NRK, og forteller partneren hva klippet handlet om. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker nyhets- og videotjenester selvstendig for å følge med på nyheter, og forteller om én nyhet i klassen hver uke. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B1 lytte</t>
@@ -1335,13 +1653,19 @@
     <t>Bruker digitale medier selvstendig og kritisk som kilde til informasjon.</t>
   </si>
   <si>
-    <t>Læreren velger et klipp eller en podkastepisode og gir elevene spørsmål før de lytter. Elevene finner hovedpunktene med støtte.</t>
-  </si>
-  <si>
-    <t>Elevene finner og bruker podkaster og filmer i strømmetjenester, og skriver tre hovedpunkter fra det de har lyttet til.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale medier selvstendig og kritisk: de lytter til to kilder om samme tema og sammenligner hovedpunktene.</t>
+    <t xml:space="preserve">Forbered: Legg klar klippet før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren velger et klipp eller en podkastepisode og gir elevene spørsmål før de lytter. Elevene finner hovedpunktene med støtte. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene finner og bruker podkaster og filmer i strømmetjenester, og skriver tre hovedpunkter fra det de har lyttet til. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale medier selvstendig og kritisk: de lytter til to kilder om samme tema og sammenligner hovedpunktene. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Lese og forstå hverdagslige tekster på digitale flater.</t>
@@ -1356,13 +1680,19 @@
     <t>Leser og forstår hverdagslige digitale tekster og skiller mellom fakta, meninger og reklame.</t>
   </si>
   <si>
-    <t>Elevene leser en hverdagslig e-post, for eksempel fra skolen, med støtte fra læreren, og finner hva, når og hvor.</t>
-  </si>
-  <si>
-    <t>Elevene leser e-poster og innlegg på sosiale medier og svarer på spørsmål om innholdet.</t>
-  </si>
-  <si>
-    <t>Elevene leser hverdagslige digitale tekster og sorterer utsagn i fakta, meninger og reklame.</t>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene leser en hverdagslig e-post, for eksempel fra skolen, med støtte fra læreren, og finner hva, når og hvor. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene leser e-poster og innlegg på sosiale medier og svarer på spørsmål om innholdet. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene leser hverdagslige digitale tekster og sorterer utsagn i fakta, meninger og reklame. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B2 lytte</t>
@@ -1380,13 +1710,19 @@
     <t>Finner selv relevant digitalt lytte-/videomateriale og forstår det.</t>
   </si>
   <si>
-    <t>Læreren velger ut digitalt lyttestoff og gir elevene en ordliste før de lytter. Elevene svarer på spørsmål om innholdet.</t>
-  </si>
-  <si>
-    <t>Elevene finner selv relevant digitalt lytte- eller videostoff, lytter og lager et kort sammendrag.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale medier selvstendig og kritisk, og vurderer hvem som står bak, og hva hensikten er.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren velger ut digitalt lyttestoff og gir elevene en ordliste før de lytter. Elevene svarer på spørsmål om innholdet. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene finner selv relevant digitalt lytte- eller videostoff, lytter og lager et kort sammendrag. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale medier selvstendig og kritisk, og vurderer hvem som står bak, og hva hensikten er. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Forstå informasjonsutveksling i formelle og uformelle digitale tekster.</t>
@@ -1401,13 +1737,19 @@
     <t>Forstår formell og uformell digital informasjonsutveksling og oppfatter tone og hensikt.</t>
   </si>
   <si>
-    <t>Elevene leser en formell digital melding, for eksempel fra NAV eller Skatteetaten, med støtte fra læreren, og finner det vesentligste: hva må jeg gjøre, og når?</t>
-  </si>
-  <si>
-    <t>Elevene sammenligner en formell e-post og et uformelt innlegg om samme tema, og finner forskjeller i språk og tone.</t>
-  </si>
-  <si>
-    <t>Elevene leser ulike digitale tekster og vurderer tone og hensikt: Er dette en informasjon, en klage, et salgsforsøk eller en invitasjon?</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene leser en formell digital melding, for eksempel fra NAV eller Skatteetaten, med støtte fra læreren, og finner det vesentligste: hva må jeg gjøre, og når? Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene sammenligner en formell e-post og et uformelt innlegg om samme tema, og finner forskjeller i språk og tone. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene leser ulike digitale tekster og vurderer tone og hensikt: Er dette en informasjon, en klage, et salgsforsøk eller en invitasjon? Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Samfunn</t>
@@ -1425,13 +1767,19 @@
     <t>Viser digital dømmekraft i egne vurderinger og kan begrunne valg med referanse til personvern og etikk.</t>
   </si>
   <si>
-    <t>Læreren forklarer begrepet digital dømmekraft med bilder av trygge og utrygge situasjoner på nett (dele passord, klikke på ukjente lenker, bruke BankID riktig). Elevene sorterer bildene i «trygt» og «utrygt» og lager sammen en liste med tre regler.</t>
-  </si>
-  <si>
-    <t>Elevene drøfter eksempler fra eget liv i par: deling av bilder, falske nyheter og svindel. De skriver ned ett eksempel og hva de gjorde eller burde ha gjort.</t>
-  </si>
-  <si>
-    <t>Elevene vurderer en ukjent situasjon (f.eks. en venneforespørsel fra en fremmed eller en melding om en «pakke på vei») og begrunner valget sitt med henvisning til personvern og etikk.</t>
+    <t xml:space="preserve">Forbered: Legg klar lenken og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren forklarer begrepet digital dømmekraft med bilder av trygge og utrygge situasjoner på nett (dele passord, klikke på ukjente lenker, bruke BankID riktig). Elevene sorterer bildene i «trygt» og «utrygt» og lager sammen en liste med tre regler. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene drøfter eksempler fra eget liv i par: deling av bilder, falske nyheter og svindel. De skriver ned ett eksempel og hva de gjorde eller burde ha gjort. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene vurderer en ukjent situasjon (f.eks. en venneforespørsel fra en fremmed eller en melding om en «pakke på vei») og begrunner valget sitt med henvisning til personvern og etikk. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 2 – Perspektivmangfold</t>
@@ -1449,13 +1797,19 @@
     <t>Finner, sammenligner og vurderer digitale kilder selvstendig.</t>
   </si>
   <si>
-    <t>Læreren gir en lenke til en offentlig nettside, og elevene finner svar på et konkret spørsmål. Deretter viser læreren en upålitelig side om samme tema, og klassen snakker om hvorfor alle kilder ikke er pålitelige.</t>
-  </si>
-  <si>
-    <t>Elevene bruker to–tre digitale kilder om samme tema, og vurderer enkelt: Hvem er avsender? Hva vil de oppnå? Er informasjonen ny?</t>
-  </si>
-  <si>
-    <t>Elevene finner, sammenligner og vurderer digitale kilder selvstendig, og lager en kort oversikt over hvilke kilder de stoler på og hvorfor.</t>
+    <t xml:space="preserve">Forbered: Legg klar lenken og nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren gir en lenke til en offentlig nettside, og elevene finner svar på et konkret spørsmål. Deretter viser læreren en upålitelig side om samme tema, og klassen snakker om hvorfor alle kilder ikke er pålitelige. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker to–tre digitale kilder om samme tema, og vurderer enkelt: Hvem er avsender? Hva vil de oppnå? Er informasjonen ny? Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene finner, sammenligner og vurderer digitale kilder selvstendig, og lager en kort oversikt over hvilke kilder de stoler på og hvorfor. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 4 – Digitale ferdigheter</t>
@@ -1473,13 +1827,19 @@
     <t>Tilegner seg selvstendig informasjon og kunnskap gjennom digital teknologi.</t>
   </si>
   <si>
-    <t>Læreren viser viktige digitale kanaler for samfunnsinformasjon, for eksempel kommunens nettside, nav.no og helsenorge.no. Elevene åpner kanalene med støtte og finner én opplysning på hver.</t>
-  </si>
-  <si>
-    <t>Elevene får oppgaver der de skal finne samfunnsinformasjon, for eksempel om skolestart eller valg, og bruker digitale kanaler delvis selvstendig.</t>
-  </si>
-  <si>
-    <t>Elevene tilegner seg informasjon selvstendig om et samfunnsspørsmål de er interessert i, og presenterer det de har lært.</t>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser viktige digitale kanaler for samfunnsinformasjon, for eksempel kommunens nettside, nav.no og helsenorge.no. Elevene åpner kanalene med støtte og finner én opplysning på hver. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får oppgaver der de skal finne samfunnsinformasjon, for eksempel om skolestart eller valg, og bruker digitale kanaler delvis selvstendig. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene tilegner seg informasjon selvstendig om et samfunnsspørsmål de er interessert i, og presenterer det de har lært. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Utvikle digital dømmekraft og bevissthet om nettbruk.</t>
@@ -1494,13 +1854,19 @@
     <t>Viser digital dømmekraft og bevisst nettbruk og kan veilede andre.</t>
   </si>
   <si>
-    <t>Læreren forklarer med bilder hva Norge som digitalt samfunn betyr: BankID, digital postkasse og digitale tjenester. Elevene kobler bilde og ord, og forteller hvilke tjenester de har brukt.</t>
-  </si>
-  <si>
-    <t>Elevene drøfter i par muligheter og utfordringer ved digital samhandling, for eksempel at det er raskt, men at ikke alle har tilgang. De skriver to fordeler og to ulemper.</t>
-  </si>
-  <si>
-    <t>Elevene viser digital dømmekraft og bevisst nettbruk ved å veilede en medelev eller et familiemedlem i å bruke en digital tjeneste trygt.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren forklarer med bilder hva Norge som digitalt samfunn betyr: BankID, digital postkasse og digitale tjenester. Elevene kobler bilde og ord, og forteller hvilke tjenester de har brukt. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene drøfter i par muligheter og utfordringer ved digital samhandling, for eksempel at det er raskt, men at ikke alle har tilgang. De skriver to fordeler og to ulemper. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene viser digital dømmekraft og bevisst nettbruk ved å veilede en medelev eller et familiemedlem i å bruke en digital tjeneste trygt. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Vise etisk refleksjon og vurdering av egen rolle på nett.</t>
@@ -1515,13 +1881,19 @@
     <t>Reflekterer selvstendig og etisk over egen rolle på nett og handler tilsvarende.</t>
   </si>
   <si>
-    <t>Læreren viser eksempler på enkle etiske regler for sosiale medier: spør før du deler bilder, vær vennlig og ikke del falske nyheter. Elevene kobler hver regel til et eksempel.</t>
-  </si>
-  <si>
-    <t>Elevene drøfter dilemmaer knyttet til egen rolle på nett, for eksempel om man skal dele en video av en krangel, og vurderer egne vaner.</t>
-  </si>
-  <si>
-    <t>Elevene reflekterer selvstendig og etisk over sin egen rolle på nett, og lager tre personlige regler de vil følge.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser eksempler på enkle etiske regler for sosiale medier: spør før du deler bilder, vær vennlig og ikke del falske nyheter. Elevene kobler hver regel til et eksempel. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene drøfter dilemmaer knyttet til egen rolle på nett, for eksempel om man skal dele en video av en krangel, og vurderer egne vaner. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene reflekterer selvstendig og etisk over sin egen rolle på nett, og lager tre personlige regler de vil følge. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Forstå at digitale ferdigheter er forutsetning for arbeids- og samfunnsliv.</t>
@@ -1536,13 +1908,19 @@
     <t>Bruker digitale ferdigheter selvstendig til videre læring og deltakelse.</t>
   </si>
   <si>
-    <t>Læreren viser bilder av ulike yrker og hvilke digitale ferdigheter som trengs (f.eks. vaktliste i app for en renholder, e-post for en kontorarbeider). Elevene kobler yrke og ferdighet.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale verktøy som brukes i utdanning og arbeid, for eksempel for å registrere seg som arbeidssøker eller søke på et kurs.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale ferdigheter selvstendig til videre læring og deltakelse, for eksempel ved å finne og melde seg på et relevant kurs.</t>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser bilder av ulike yrker og hvilke digitale ferdigheter som trengs (f.eks. vaktliste i app for en renholder, e-post for en kontorarbeider). Elevene kobler yrke og ferdighet. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker digitale verktøy som brukes i utdanning og arbeid, for eksempel for å registrere seg som arbeidssøker eller søke på et kurs. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale ferdigheter selvstendig til videre læring og deltakelse, for eksempel ved å finne og melde seg på et relevant kurs. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Personvern og opphavsrett</t>
@@ -1560,13 +1938,19 @@
     <t>Bruker kunnskapen selvstendig og vurderer rettigheter i nye digitale situasjoner.</t>
   </si>
   <si>
-    <t>Læreren forklarer grunnreglene for personvern og opphavsrett med eksempler: ikke del andres bilder uten lov, og ikke bruk bilder fra nett uten å sjekke om det er lov. Elevene sorterer eksempler i «lov» og «ikke lov».</t>
-  </si>
-  <si>
-    <t>Elevene bruker det de har lært i konkrete situasjoner: de finner bilder med fri bruk til en presentasjon og spør medelever om lov før de tar bilder.</t>
-  </si>
-  <si>
-    <t>Elevene vurderer rettigheter i nye situasjoner, for eksempel ved deling av video fra et arrangement eller bruk av musikk i en video, og begrunner valgene.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren forklarer grunnreglene for personvern og opphavsrett med eksempler: ikke del andres bilder uten lov, og ikke bruk bilder fra nett uten å sjekke om det er lov. Elevene sorterer eksempler i «lov» og «ikke lov». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker det de har lært i konkrete situasjoner: de finner bilder med fri bruk til en presentasjon og spør medelever om lov før de tar bilder. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene vurderer rettigheter i nye situasjoner, for eksempel ved deling av video fra et arrangement eller bruk av musikk i en video, og begrunner valgene. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Kritisk tenkning</t>
@@ -1584,13 +1968,19 @@
     <t>Drøfter selvstendig betydningen av digital dømmekraft og begrunner standpunkt.</t>
   </si>
   <si>
-    <t>Læreren leder en samtale med bilder og enkle spørsmål: Hvorfor er det viktig å tenke kritisk på nett? Elevene svarer med setningsstartere som «Det er viktig fordi …».</t>
-  </si>
-  <si>
-    <t>Elevene samtaler i par og gir egne eksempler på kritisk tenkning i digitale sammenhenger, for eksempel om en nyhet eller et tilbud på nett.</t>
-  </si>
-  <si>
-    <t>Elevene drøfter selvstendig betydningen av digital dømmekraft i samfunnet, og begrunner sitt eget standpunkt i en kort tekst eller muntlig.</t>
+    <t xml:space="preserve">Forbered: Legg klar setningsstartere og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren leder en samtale med bilder og enkle spørsmål: Hvorfor er det viktig å tenke kritisk på nett? Elevene svarer med setningsstartere som «Det er viktig fordi …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene samtaler i par og gir egne eksempler på kritisk tenkning i digitale sammenhenger, for eksempel om en nyhet eller et tilbud på nett. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene drøfter selvstendig betydningen av digital dømmekraft i samfunnet, og begrunner sitt eget standpunkt i en kort tekst eller muntlig. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Helsetjenester</t>
@@ -1608,13 +1998,19 @@
     <t>Bruker digitale helsetjenester selvstendig for seg selv og eventuelt familie.</t>
   </si>
   <si>
-    <t>Læreren viser helsenorge.no og viser hvordan man logger inn med BankID. Elevene øver på å logge inn med støtte.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale helsetjenester delvis selvstendig: de bestiller time hos fastlegen eller leser en melding i en øvingssituasjon.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale helsetjenester selvstendig, for seg selv og eventuelt for barna sine, og viser en medelev hvordan det gjøres.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser helsenorge.no og viser hvordan man logger inn med BankID. Elevene øver på å logge inn med støtte. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker digitale helsetjenester delvis selvstendig: de bestiller time hos fastlegen eller leser en melding i en øvingssituasjon. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale helsetjenester selvstendig, for seg selv og eventuelt for barna sine, og viser en medelev hvordan det gjøres. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Rettigheter</t>
@@ -1632,13 +2028,19 @@
     <t>Bruker digitale tjenester selvstendig og finner nye ved behov.</t>
   </si>
   <si>
-    <t>Læreren viser digitale tjenester som gjelder elevenes rettigheter, for eksempel NAV og Skatteetaten. Elevene åpner tjenestene med støtte og finner én opplysning.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale offentlige tjenester delvis selvstendig, for eksempel for å sjekke skattekortet eller sende en melding til NAV.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale tjenester selvstendig og finner nye tjenester ved behov, for eksempel når de flytter eller får barn.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser digitale tjenester som gjelder elevenes rettigheter, for eksempel NAV og Skatteetaten. Elevene åpner tjenestene med støtte og finner én opplysning. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker digitale offentlige tjenester delvis selvstendig, for eksempel for å sjekke skattekortet eller sende en melding til NAV. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale tjenester selvstendig og finner nye tjenester ved behov, for eksempel når de flytter eller får barn. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Samfunnsdeltakelse</t>
@@ -1656,13 +2058,19 @@
     <t>Deltar aktivt og selvstendig på digitale sosiale og frivillige arenaer.</t>
   </si>
   <si>
-    <t>Læreren viser hvordan en lokal forening (f.eks. idrettslag eller frivilligsentral) bruker nettside og sosiale medier. Elevene ser på kanalene sammen med læreren.</t>
-  </si>
-  <si>
-    <t>Elevene finner relevante digitale fellesskap i nærmiljøet og melder seg inn i ett av dem, delvis selvstendig.</t>
-  </si>
-  <si>
-    <t>Elevene deltar aktivt og selvstendig på digitale sosiale og frivillige arenaer, og forteller klassen om hva de deltar i.</t>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser hvordan en lokal forening (f.eks. idrettslag eller frivilligsentral) bruker nettside og sosiale medier. Elevene ser på kanalene sammen med læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene finner relevante digitale fellesskap i nærmiljøet og melder seg inn i ett av dem, delvis selvstendig. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene deltar aktivt og selvstendig på digitale sosiale og frivillige arenaer, og forteller klassen om hva de deltar i. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Kunnskapssøking</t>
@@ -1680,13 +2088,19 @@
     <t>Driver selvstendig kunnskapssøking i digitale kilder og vurderer dem kritisk.</t>
   </si>
   <si>
-    <t>Læreren gir elevene anviste digitale ressurser, for eksempel en lettlest nettside om et samfunnstema, og elevene finner mer kunnskap med støtte.</t>
-  </si>
-  <si>
-    <t>Elevene søker selv etter mer kunnskap i anbefalte digitale kilder og noterer hva de fant.</t>
-  </si>
-  <si>
-    <t>Elevene søker selvstendig etter kunnskap i digitale kilder, vurderer kildene kritisk og presenterer det de har lært.</t>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren gir elevene anviste digitale ressurser, for eksempel en lettlest nettside om et samfunnstema, og elevene finner mer kunnskap med støtte. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene søker selv etter mer kunnskap i anbefalte digitale kilder og noterer hva de fant. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene søker selvstendig etter kunnskap i digitale kilder, vurderer kildene kritisk og presenterer det de har lært. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Use one menu for language levels and spell out classroom activities. (#1)
Norsk is navigated by Om opplæringen, Før A1 and A1–B2, with the same sections in the sidebar and overview. Each level card now gives the teacher a prepare, do and look-for suggestion.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: Ivar <IvarMolde@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/data/digitale-ferdigheter.xlsx
+++ b/public/data/digitale-ferdigheter.xlsx
@@ -72,13 +72,19 @@
     <t>Opptrer ansvarlig selvstendig i all digital kommunikasjon og ivaretar personvern.</t>
   </si>
   <si>
-    <t>Læreren viser tre skjermbilder av chatmeldinger på storskjerm: en vennlig melding, en uhøflig melding og en melding der noen deler et bilde av en annen uten å spørre. Elevene viser tommel opp eller ned for hver melding. Klassen lager sammen tre–fire enkle regler med ikoner («Vi skriver vennlig», «Vi spør før vi deler bilder»). Reglene henges opp ved PC-ene og leses høyt før hver digitale økt.</t>
-  </si>
-  <si>
-    <t>Elevene får situasjonskort, for eksempel «Du vil dele et klassebilde i gruppechatten». I par velger de hva de vil gjøre, og forklarer med setningsstarteren «Jeg gjør … fordi …». Hvert par presenterer ett valg for klassen, og læreren skriver begrunnelsene på tavla som felles ordforråd.</t>
-  </si>
-  <si>
-    <t>Elevene lager i grupper en digital plakat med regler for klassens kanal (f.eks. i Teams) om tone, bilder og personvern. Hver regel skal ha en kort begrunnelse. Etter en uke sjekker gruppene egne innlegg mot plakaten og foreslår eventuelle endringer.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser tre skjermbilder av chatmeldinger på storskjerm: en vennlig melding, en uhøflig melding og en melding der noen deler et bilde av en annen uten å spørre. Elevene viser tommel opp eller ned for hver melding. Klassen lager sammen tre–fire enkle regler med ikoner («Vi skriver vennlig», «Vi spør før vi deler bilder»). Reglene henges opp ved PC-ene og leses høyt før hver digitale økt. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar situasjonskort, setningsstartere og bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får situasjonskort, for eksempel «Du vil dele et klassebilde i gruppechatten». I par velger de hva de vil gjøre, og forklarer med setningsstarteren «Jeg gjør … fordi …». Hvert par presenterer ett valg for klassen, og læreren skriver begrunnelsene på tavla som felles ordforråd. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar plakaten, bilder og kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene lager i grupper en digital plakat med regler for klassens kanal (f.eks. i Teams) om tone, bilder og personvern. Hver regel skal ha en kort begrunnelse. Etter en uke sjekker gruppene egne innlegg mot plakaten og foreslår eventuelle endringer. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>2.3 – Grunnleggende ferdigheter</t>
@@ -99,13 +105,19 @@
     <t>Videreutvikler digitale ferdigheter selvstendig gjennom hele opplæringsløpet.</t>
   </si>
   <si>
-    <t>Innfør en fast digital startrutine hver økt: slå på PC, logge inn, åpne læringsplattformen og finne dagens oppgave. Læreren viser trinnene på storskjerm med nummererte bildekort (1–2–3–4). Elevene gjør det samme i sitt eget tempo, og sidemannen hjelper ved behov. Rutinen er lik hver dag til den sitter.</t>
-  </si>
-  <si>
-    <t>Elevene har en enkel sjekkliste med ikoner: logge inn, lagre, finne fil, sende. Etter hver økt krysser de av det de klarte alene. Læreren samler inn listene hver fredag og velger neste ferdighet klassen skal øve på ut fra hva mange mangler.</t>
-  </si>
-  <si>
-    <t>Elevene fører en digital logg der de hver uke skriver én ny ting de har lært å gjøre digitalt og ett mål for neste uke. En gang i måneden viser hver elev en ny ferdighet til en medelev («elev lærer elev»).</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, bildekort og læringsplattformen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Innfør en fast digital startrutine hver økt: slå på PC, logge inn, åpne læringsplattformen og finne dagens oppgave. Læreren viser trinnene på storskjerm med nummererte bildekort (1–2–3–4). Elevene gjør det samme i sitt eget tempo, og sidemannen hjelper ved behov. Rutinen er lik hver dag til den sitter. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene har en enkel sjekkliste med ikoner: logge inn, lagre, finne fil, sende. Etter hver økt krysser de av det de klarte alene. Læreren samler inn listene hver fredag og velger neste ferdighet klassen skal øve på ut fra hva mange mangler. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene fører en digital logg der de hver uke skriver én ny ting de har lært å gjøre digitalt og ett mål for neste uke. En gang i måneden viser hver elev en ny ferdighet til en medelev («elev lærer elev»). Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Digitale ferdigheter som del av faglig kompetanse og læring.</t>
@@ -120,13 +132,19 @@
     <t>Bruker digitale ferdigheter selvstendig som redskap for læring og samfunnsdeltakelse.</t>
   </si>
   <si>
-    <t>Elevene bruker en bildeordbok eller ordapp for å finne ord til dagens tema (f.eks. mat). Læreren viser trinnene: skriv ordet – trykk på lydknappen – lytt – si ordet høyt. Elevene gjør det samme med fem ord og viser bildene til partneren sin.</t>
-  </si>
-  <si>
-    <t>Etter å ha lest en fagtekst finner elevene selv tre nye ord i en digital ordbok, lytter til uttalen og lagrer ordene i sin egen digitale ordliste med bilde eller oversettelse til morsmålet. Neste dag forhører partneren dem på ordene.</t>
-  </si>
-  <si>
-    <t>Elevene lager et lite digitalt produkt om et tema fra undervisningen, for eksempel en kort presentasjon eller et lydopptak. De velger selv verktøy og kilder, og avslutter med å forklare hvordan verktøyet hjalp dem å lære.</t>
+    <t xml:space="preserve">Forbered: Legg klar ordboka og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene bruker en bildeordbok eller ordapp for å finne ord til dagens tema (f.eks. mat). Læreren viser trinnene: skriv ordet – trykk på lydknappen – lytt – si ordet høyt. Elevene gjør det samme med fem ord og viser bildene til partneren sin. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar ordboka og bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Etter å ha lest en fagtekst finner elevene selv tre nye ord i en digital ordbok, lytter til uttalen og lagrer ordene i sin egen digitale ordliste med bilde eller oversettelse til morsmålet. Neste dag forhører partneren dem på ordene. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene lager et lite digitalt produkt om et tema fra undervisningen, for eksempel en kort presentasjon eller et lydopptak. De velger selv verktøy og kilder, og avslutter med å forklare hvordan verktøyet hjalp dem å lære. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Integrer digitale ferdigheter på tvers av fag.</t>
@@ -141,13 +159,19 @@
     <t>Bruker digitale ferdigheter selvstendig og integrert på tvers av fag.</t>
   </si>
   <si>
-    <t>Handleoppgave: Læreren åpner en nettbutikk på storskjerm. Elevene leser navnet på tre varer (lesing), skriver dem i et dokument (skriving), sier dem høyt til partneren (muntlig) og legger sammen prisene med kalkulatoren på PC-en (regning). Læreren viser hvert trinn før elevene gjør det.</t>
-  </si>
-  <si>
-    <t>Elevene planlegger en busstur med en reiseapp eller nettside: de finner avgangstid (lesing), regner ut hvor lang tid turen tar (regning), skriver en kort melding om når de kommer fram (skriving) og forteller planen til partneren (muntlig).</t>
-  </si>
-  <si>
-    <t>Elevene planlegger et klassearrangement. De sammenligner priser på nett, lager et enkelt budsjett i regneark, skriver en digital invitasjon og presenterer planen muntlig for klassen. Elevene velger selv hvilke verktøy de bruker.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Handleoppgave: Læreren åpner en nettbutikk på storskjerm. Elevene leser navnet på tre varer (lesing), skriver dem i et dokument (skriving), sier dem høyt til partneren (muntlig) og legger sammen prisene med kalkulatoren på PC-en (regning). Læreren viser hvert trinn før elevene gjør det. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene planlegger en busstur med en reiseapp eller nettside: de finner avgangstid (lesing), regner ut hvor lang tid turen tar (regning), skriver en kort melding om når de kommer fram (skriving) og forteller planen til partneren (muntlig). Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene planlegger et klassearrangement. De sammenligner priser på nett, lager et enkelt budsjett i regneark, skriver en digital invitasjon og presenterer planen muntlig for klassen. Elevene velger selv hvilke verktøy de bruker. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>2.5.3 – Bærekraftig utvikling</t>
@@ -168,13 +192,19 @@
     <t>Forstår og drøfter selvstendig sammenhenger mellom teknologi og bærekraft.</t>
   </si>
   <si>
-    <t>Læreren viser bilder av en lader, en mobil, en PC og gamle mobiler i en skuff. Elevene sorterer bildene sammen med læreren i to grupper: «bruker strøm» og «kan gjenbrukes». Klassen øver på enkle setninger: «Mobilen bruker strøm.» «Den gamle mobilen kan leveres.»</t>
-  </si>
-  <si>
-    <t>I par får elevene dilemmakort, for eksempel «Bør man kjøpe ny mobil hvert år?» eller «Er det greit å strømme video hele dagen?». De svarer ja eller nei, begrunner med «fordi …» og sammenligner svarene med et annet par.</t>
-  </si>
-  <si>
-    <t>Elevene undersøker ett tema i digitale kilder, for eksempel elektronisk avfall eller netthandel med gratis retur. I gruppe drøfter de fordeler og ulemper for miljø, økonomi og mennesker, og presenterer en kort konklusjon for klassen.</t>
+    <t xml:space="preserve">Forbered: Legg klar mobilen og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser bilder av en lader, en mobil, en PC og gamle mobiler i en skuff. Elevene sorterer bildene sammen med læreren i to grupper: «bruker strøm» og «kan gjenbrukes». Klassen øver på enkle setninger: «Mobilen bruker strøm.» «Den gamle mobilen kan leveres.». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar dilemmakort, klippet og mobilen før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: I par får elevene dilemmakort, for eksempel «Bør man kjøpe ny mobil hvert år?» eller «Er det greit å strømme video hele dagen?». De svarer ja eller nei, begrunner med «fordi …» og sammenligner svarene med et annet par. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene undersøker ett tema i digitale kilder, for eksempel elektronisk avfall eller netthandel med gratis retur. I gruppe drøfter de fordeler og ulemper for miljø, økonomi og mennesker, og presenterer en kort konklusjon for klassen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>1.5 – Miljøbevissthet</t>
@@ -195,13 +225,19 @@
     <t>Reflekterer selvstendig over teknologiens rolle for bærekraft.</t>
   </si>
   <si>
-    <t>Læreren viser en sorteringsguide eller app fra det lokale renovasjonsselskapet på storskjerm. Klassen søker sammen på «batteri» og «gammel mobil», og elevene peker på svaret. Hver elev får et bildekort med én gjenstand og viser hvor den skal kastes.</t>
-  </si>
-  <si>
-    <t>Elevene bruker selv en sorteringsguide eller en nettside for bruktsalg for å finne ut hvordan tre gjenstander kan sorteres eller gjenbrukes. De skriver én setning om hver gjenstand: «Jeg kan … fordi …».</t>
-  </si>
-  <si>
-    <t>Elevene lager en liten digital guide for klassen: «Tre digitale verktøy som hjelper deg å leve miljøvennlig». De presenterer guiden og begrunner hvorfor de valgte akkurat disse verktøyene.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, bildekort og mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en sorteringsguide eller app fra det lokale renovasjonsselskapet på storskjerm. Klassen søker sammen på «batteri» og «gammel mobil», og elevene peker på svaret. Hver elev får et bildekort med én gjenstand og viser hvor den skal kastes. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker selv en sorteringsguide eller en nettside for bruktsalg for å finne ut hvordan tre gjenstander kan sorteres eller gjenbrukes. De skriver én setning om hver gjenstand: «Jeg kan … fordi …». Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene lager en liten digital guide for klassen: «Tre digitale verktøy som hjelper deg å leve miljøvennlig». De presenterer guiden og begrunner hvorfor de valgte akkurat disse verktøyene. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>2.4 – Å lære å lære</t>
@@ -222,13 +258,19 @@
     <t>Styrer egen læring med mangfold av digitale strategier.</t>
   </si>
   <si>
-    <t>Læreren gir et spørsmål med bilde, for eksempel «Når åpner biblioteket?», og en ferdig lenke. Elevene finner svaret med lærerens hjelp og svarer med en fast setning: «Biblioteket åpner klokka …». Samme type oppgave gjentas med nye spørsmål flere dager på rad.</t>
-  </si>
-  <si>
-    <t>Elevene lager selv ett spørsmål om nærmiljøet ved hjelp av kort med spørreord (hva, når, hvor, hvor mye). De velger om de vil bruke søkemotor eller en kjent nettside, finner svaret og forteller partneren hvordan de søkte.</t>
-  </si>
-  <si>
-    <t>Elevene formulerer tre egne spørsmål om et tema, planlegger søket (søkeord og kilder), søker og vurderer svarene. Til slutt skriver de kort hvilken strategi som fungerte best og hvorfor.</t>
+    <t xml:space="preserve">Forbered: Legg klar lenken og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren gir et spørsmål med bilde, for eksempel «Når åpner biblioteket?», og en ferdig lenke. Elevene finner svaret med lærerens hjelp og svarer med en fast setning: «Biblioteket åpner klokka …». Samme type oppgave gjentas med nye spørsmål flere dager på rad. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene lager selv ett spørsmål om nærmiljøet ved hjelp av kort med spørreord (hva, når, hvor, hvor mye). De velger om de vil bruke søkemotor eller en kjent nettside, finner svaret og forteller partneren hvordan de søkte. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene formulerer tre egne spørsmål om et tema, planlegger søket (søkeord og kilder), søker og vurderer svarene. Til slutt skriver de kort hvilken strategi som fungerte best og hvorfor. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>2.5.1 – Folkehelse</t>
@@ -249,13 +291,19 @@
     <t>Tar bevisste valg om mediebruk og digital økonomi selvstendig.</t>
   </si>
   <si>
-    <t>Elevene åpner skjermtid-oversikten på egen mobil sammen med læreren. Ved hjelp av bildekort (sove, jobbe, video, familie, nyheter) forteller de enkelt: «Jeg bruker mobilen til …». Klassen snakker om hvordan skjerm påvirker søvn, og øver på setningen «Jeg legger bort mobilen klokka …».</t>
-  </si>
-  <si>
-    <t>Elevene fører en enkel mediedagbok i tre dager (tabell: når – hva – hvor lenge). I par sammenligner de dagbøkene og foreslår én endring. De ser også på oversikten i bankappen og finner hva de har brukt penger på digitalt, for eksempel abonnementer.</t>
-  </si>
-  <si>
-    <t>Elevene setter et eget mål for mediebruk eller digital økonomi, for eksempel en skjermfri kveld i uka eller å si opp et abonnement de ikke bruker. De følger opp målet i to uker og forteller kort for klassen hva som skjedde.</t>
+    <t xml:space="preserve">Forbered: Legg klar bildekort, klippet og mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene åpner skjermtid-oversikten på egen mobil sammen med læreren. Ved hjelp av bildekort (sove, jobbe, video, familie, nyheter) forteller de enkelt: «Jeg bruker mobilen til …». Klassen snakker om hvordan skjerm påvirker søvn, og øver på setningen «Jeg legger bort mobilen klokka …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene fører en enkel mediedagbok i tre dager (tabell: når – hva – hvor lenge). I par sammenligner de dagbøkene og foreslår én endring. De ser også på oversikten i bankappen og finner hva de har brukt penger på digitalt, for eksempel abonnementer. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene setter et eget mål for mediebruk eller digital økonomi, for eksempel en skjermfri kveld i uka eller å si opp et abonnement de ikke bruker. De følger opp målet i to uker og forteller kort for klassen hva som skjedde. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>2.5.2 – Demokrati</t>
@@ -273,13 +321,19 @@
     <t>Deltar selvstendig og saklig i digital meningsbrytning.</t>
   </si>
   <si>
-    <t>Læreren viser et tilrettelagt skjermbilde av en nettdebatt med både høflige og uhøflige kommentarer. Elevene peker ut de høflige. Klassen øver på faste fraser for uenighet: «Jeg er uenig, fordi …» og «Jeg forstår deg, men …».</t>
-  </si>
-  <si>
-    <t>Læreren legger ut en enkel påstand i en lukket klassekanal, for eksempel «Barn under 13 år bør ikke ha mobil». Elevene skriver en kommentar med begrunnelse og svarer respektfullt på en medelev som mener noe annet. Frasene fra tavla kan brukes som støtte.</t>
-  </si>
-  <si>
-    <t>Elevene deltar i en strukturert digital debatt om en aktuell sak. De finner ett faktagrunnlag i en pålitelig kilde, skriver et saklig innlegg og svarer på motargumenter. Etterpå vurderer de sin egen tone ut fra klassens regler.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et tilrettelagt skjermbilde av en nettdebatt med både høflige og uhøflige kommentarer. Elevene peker ut de høflige. Klassen øver på faste fraser for uenighet: «Jeg er uenig, fordi …» og «Jeg forstår deg, men …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar mobilen før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Læreren legger ut en enkel påstand i en lukket klassekanal, for eksempel «Barn under 13 år bør ikke ha mobil». Elevene skriver en kommentar med begrunnelse og svarer respektfullt på en medelev som mener noe annet. Frasene fra tavla kan brukes som støtte. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene deltar i en strukturert digital debatt om en aktuell sak. De finner ett faktagrunnlag i en pålitelig kilde, skriver et saklig innlegg og svarer på motargumenter. Etterpå vurderer de sin egen tone ut fra klassens regler. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>3.1 – Inkluderende miljø</t>
@@ -300,13 +354,19 @@
     <t>Samhandler forsvarlig og selvstendig på alle digitale flater.</t>
   </si>
   <si>
-    <t>Klassen lager en plakat med ikoner: «Vi skriver vennlig om andre» og «Vi spør før vi deler bilder». Før hver bruk av klassechatten peker læreren på plakaten, og elevene øver på å sende ferdige, vennlige meldinger fra en frasebank.</t>
-  </si>
-  <si>
-    <t>Elevene får situasjonskort, for eksempel «Noen blir holdt utenfor i gruppechatten» eller «Noen har delt et bilde av deg uten å spørre». I par diskuterer de hva de kan gjøre, og skriver en passende melding til personen det gjelder.</t>
-  </si>
-  <si>
-    <t>Elevene evaluerer klassens digitale samhandling med et anonymt skjema og lager forslag til forbedringer. To og to elever har ansvaret for å ønske nye elever velkommen i klassens digitale kanal og hjelpe dem i gang.</t>
+    <t xml:space="preserve">Forbered: Legg klar fraser, plakaten og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Klassen lager en plakat med ikoner: «Vi skriver vennlig om andre» og «Vi spør før vi deler bilder». Før hver bruk av klassechatten peker læreren på plakaten, og elevene øver på å sende ferdige, vennlige meldinger fra en frasebank. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar situasjonskort og bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får situasjonskort, for eksempel «Noen blir holdt utenfor i gruppechatten» eller «Noen har delt et bilde av deg uten å spørre». I par diskuterer de hva de kan gjøre, og skriver en passende melding til personen det gjelder. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene evaluerer klassens digitale samhandling med et anonymt skjema og lager forslag til forbedringer. To og to elever har ansvaret for å ønske nye elever velkommen i klassens digitale kanal og hjelpe dem i gang. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>3.2 – Tilpasset opplæring</t>
@@ -327,13 +387,19 @@
     <t>Velger og bruker digitale læremidler selvstendig ut fra egne behov.</t>
   </si>
   <si>
-    <t>Læreren legger en snarvei til ett digitalt læremiddel på riktig nivå på elevens skrivebord eller hjemskjerm. Eleven åpner læremiddelet, velger oppgave etter fargekode og jobber ti minutter hver dag. De første gangene sitter læreren ved siden av og viser knappene.</t>
-  </si>
-  <si>
-    <t>Eleven velger blant to–tre kjente læremidler ved hjelp av et enkelt valgkart: «Vil du øve på ord? Lytte? Skrive?». Eleven jobber på egen stasjon og noterer hvilket læremiddel og nivå de brukte.</t>
-  </si>
-  <si>
-    <t>Eleven lager en egen ukeplan for digital øving basert på sine mål. Eleven velger læremidler og nivå selv, og forklarer valgene i en kort samtale med læreren.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren legger en snarvei til ett digitalt læremiddel på riktig nivå på elevens skrivebord eller hjemskjerm. Eleven åpner læremiddelet, velger oppgave etter fargekode og jobber ti minutter hver dag. De første gangene sitter læreren ved siden av og viser knappene. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Eleven velger blant to–tre kjente læremidler ved hjelp av et enkelt valgkart: «Vil du øve på ord? Lytte? Skrive?». Eleven jobber på egen stasjon og noterer hvilket læremiddel og nivå de brukte. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Eleven lager en egen ukeplan for digital øving basert på sine mål. Eleven velger læremidler og nivå selv, og forklarer valgene i en kort samtale med læreren. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Sette mål og vurdere egen utvikling i digitale sammenhenger.</t>
@@ -348,13 +414,19 @@
     <t>Setter, følger opp og vurderer egne digitale mål selvstendig.</t>
   </si>
   <si>
-    <t>Eleven velger sammen med læreren ett lite digitalt mål med bilde, for eksempel «sende en e-post». Målet skrives på et målkort. Når målet er nådd, viser eleven læreren hva hen kan, og setter et klistremerke på kortet.</t>
-  </si>
-  <si>
-    <t>Eleven skriver egne mål i et digitalt skjema med setningsstarteren «Jeg vil lære å …». Hver fredag vurderer eleven seg selv med en smilefjes-skala og skriver én setning om hva som gikk bra.</t>
-  </si>
-  <si>
-    <t>Eleven fører en digital mappe med mål, bevis (skjermbilder og filer) og refleksjon. Én gang i måneden har eleven en kort samtale med læreren og justerer målene sine.</t>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel, bilder og kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Eleven velger sammen med læreren ett lite digitalt mål med bilde, for eksempel «sende en e-post». Målet skrives på et målkort. Når målet er nådd, viser eleven læreren hva hen kan, og setter et klistremerke på kortet. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar setningsstartere og skjemaet før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Eleven skriver egne mål i et digitalt skjema med setningsstarteren «Jeg vil lære å …». Hver fredag vurderer eleven seg selv med en smilefjes-skala og skriver én setning om hva som gikk bra. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder og kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Eleven fører en digital mappe med mål, bevis (skjermbilder og filer) og refleksjon. Én gang i måneden har eleven en kort samtale med læreren og justerer målene sine. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Norsk</t>
@@ -378,13 +450,19 @@
     <t>Bruker digitale verktøy selvstendig som redskap for videre læring og arbeidsliv.</t>
   </si>
   <si>
-    <t>Læreren viser tre digitale verktøy med bilder: kamera, ordbok og melding. Elevene øver på å ta bilde av tavla, finne bildet igjen i galleriet og vise det til partneren. Læreren forklarer med enkle ord og bilder at dette også brukes på jobb, for eksempel for å ta bilde av en vaktliste.</t>
-  </si>
-  <si>
-    <t>Elevene får en jobbsituasjon: en vaktliste er sendt på e-post eller i en app. De åpner vaktlista, finner sin egen vakt og svarer med en kort bekreftelse: «Takk, jeg jobber mandag klokka 8.»</t>
-  </si>
-  <si>
-    <t>Elevene undersøker hvilke digitale verktøy som brukes i et yrke de er interessert i (f.eks. på utdanning.no). De lager en kort oversikt over hva de allerede kan og hva de må lære, og legger oversikten i sin digitale mappe.</t>
+    <t xml:space="preserve">Forbered: Legg klar ordboka og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser tre digitale verktøy med bilder: kamera, ordbok og melding. Elevene øver på å ta bilde av tavla, finne bildet igjen i galleriet og vise det til partneren. Læreren forklarer med enkle ord og bilder at dette også brukes på jobb, for eksempel for å ta bilde av en vaktliste. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får en jobbsituasjon: en vaktliste er sendt på e-post eller i en app. De åpner vaktlista, finner sin egen vakt og svarer med en kort bekreftelse: «Takk, jeg jobber mandag klokka 8.». Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene undersøker hvilke digitale verktøy som brukes i et yrke de er interessert i (f.eks. på utdanning.no). De lager en kort oversikt over hva de allerede kan og hva de må lære, og legger oversikten i sin digitale mappe. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 2 – Kartlegging</t>
@@ -405,13 +483,19 @@
     <t>Vurderer egen digital kompetanse underveis og justerer digitale mål.</t>
   </si>
   <si>
-    <t>Praktisk kartlegging: Eleven får bildekort med oppgaver (slå på PC, åpne en app, ta et bilde, sende en melding) og viser læreren hva hen kan. Læreren noterer underveis. Samtalen foregår på enkel norsk, med tolk eller morsmålsstøtte ved behov.</t>
-  </si>
-  <si>
-    <t>Eleven fyller ut en selvvurdering med ikoner og svaralternativene «kan», «kan litt» og «kan ikke». Etterpå forteller eleven læreren om én ting hen vil lære først.</t>
-  </si>
-  <si>
-    <t>Eleven fyller ut det samme kartleggingsskjemaet hver termin, sammenligner med forrige gang og setter nye digitale mål i samtale med læreren.</t>
+    <t xml:space="preserve">Forbered: Legg klar bildekort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Praktisk kartlegging: Eleven får bildekort med oppgaver (slå på PC, åpne en app, ta et bilde, sende en melding) og viser læreren hva hen kan. Læreren noterer underveis. Samtalen foregår på enkel norsk, med tolk eller morsmålsstøtte ved behov. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Eleven fyller ut en selvvurdering med ikoner og svaralternativene «kan», «kan litt» og «kan ikke». Etterpå forteller eleven læreren om én ting hen vil lære først. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Eleven fyller ut det samme kartleggingsskjemaet hver termin, sammenligner med forrige gang og setter nye digitale mål i samtale med læreren. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 2 – Organisering</t>
@@ -429,13 +513,19 @@
     <t>Utnytter digitale muligheter aktivt i egen læring.</t>
   </si>
   <si>
-    <t>Læreren legger dagens plan på samme sted på læringsplattformen hver dag. Klassen øver sammen på å finne den – samme knapper, samme rekkefølge – til alle klarer det. Elevene som er raske, hjelper sidemannen.</t>
-  </si>
-  <si>
-    <t>Elevene får en hjemmeoppgave på læringsplattformen. I klassen øver de på å åpne oppgaven på mobilen, og leverer den hjemmefra. Neste dag forteller de hvordan det gikk og hva som var vanskelig.</t>
-  </si>
-  <si>
-    <t>Elevene bruker plattformen aktivt: de leverer arbeid, bruker ressursbanken til ekstra øving og ordner egne filer i mapper. En gang i uka viser de læreren hva de har øvd på hjemme.</t>
+    <t xml:space="preserve">Forbered: Legg klar læringsplattformen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren legger dagens plan på samme sted på læringsplattformen hver dag. Klassen øver sammen på å finne den – samme knapper, samme rekkefølge – til alle klarer det. Elevene som er raske, hjelper sidemannen. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar læringsplattformen og mobilen før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får en hjemmeoppgave på læringsplattformen. I klassen øver de på å åpne oppgaven på mobilen, og leverer den hjemmefra. Neste dag forteller de hvordan det gikk og hva som var vanskelig. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar læringsplattformen før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker plattformen aktivt: de leverer arbeid, bruker ressursbanken til ekstra øving og ordner egne filer i mapper. En gang i uka viser de læreren hva de har øvd på hjemme. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 3 – Språklæringsstrategier</t>
@@ -456,13 +546,19 @@
     <t>Bruker digital teknologi strategisk og kritisk som språklæringsstrategi.</t>
   </si>
   <si>
-    <t>Læreren viser ett hjelpemiddel, for eksempel opplesning (talesyntese) eller en bildeordbok. Elevene gjør samme øvelse hver dag i en uke: skriv ordet – lytt – si ordet. Når rutinen sitter, innføres neste hjelpemiddel.</t>
-  </si>
-  <si>
-    <t>Elevene har en «verktøykasse» med kjente hjelpemidler: ordbok, tale-til-tekst og oversettelse. Ved hver skriveoppgave velger de selv hjelpemiddel og noterer hvilket de brukte og om det hjalp.</t>
-  </si>
-  <si>
-    <t>Elevene sammenligner en maskinoversettelse med sin egen tekst, finner feil i oversettelsen og forklarer når oversettelse hjelper og når den kan gi feil. De lager sammen en liste med råd om bruk av oversettelsesverktøy.</t>
+    <t xml:space="preserve">Forbered: Legg klar ordboka og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser ett hjelpemiddel, for eksempel opplesning (talesyntese) eller en bildeordbok. Elevene gjør samme øvelse hver dag i en uke: skriv ordet – lytt – si ordet. Når rutinen sitter, innføres neste hjelpemiddel. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar ordboka før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene har en «verktøykasse» med kjente hjelpemidler: ordbok, tale-til-tekst og oversettelse. Ved hver skriveoppgave velger de selv hjelpemiddel og noterer hvilket de brukte og om det hjalp. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene sammenligner en maskinoversettelse med sin egen tekst, finner feil i oversettelsen og forklarer når oversettelse hjelper og når den kan gi feil. De lager sammen en liste med råd om bruk av oversettelsesverktøy. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 3 – Resepsjon</t>
@@ -480,13 +576,19 @@
     <t>Henter informasjon fra ulike digitale kilder og vurderer den kritisk.</t>
   </si>
   <si>
-    <t>Læreren gir elevene en lenke til nettsiden til et legekontor. Elevene finner åpningstiden med støtte (læreren peker på hvor de skal se) og svarer med fast setning: «Legekontoret er åpent fra … til …».</t>
-  </si>
-  <si>
-    <t>Elevene leser en kort nyhetssak på et lettlest nettsted og lytter til lydversjonen. Etterpå svarer de på tre enkle spørsmål om hva, hvor og når.</t>
-  </si>
-  <si>
-    <t>Elevene får to nettsider om samme tema – én seriøs og én med reklame eller falsk informasjon. De sammenligner avsender, dato og formål, og begrunner hvilken side de stoler på.</t>
+    <t xml:space="preserve">Forbered: Legg klar lenken og nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren gir elevene en lenke til nettsiden til et legekontor. Elevene finner åpningstiden med støtte (læreren peker på hvor de skal se) og svarer med fast setning: «Legekontoret er åpent fra … til …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene leser en kort nyhetssak på et lettlest nettsted og lytter til lydversjonen. Etterpå svarer de på tre enkle spørsmål om hva, hvor og når. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene får to nettsider om samme tema – én seriøs og én med reklame eller falsk informasjon. De sammenligner avsender, dato og formål, og begrunner hvilken side de stoler på. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 3 – Produksjon</t>
@@ -504,13 +606,19 @@
     <t>Veksler selvstendig mellom muntlig og skriftlig på digitale flater og tilpasser til mottaker og kanal.</t>
   </si>
   <si>
-    <t>Læreren viser en modell-SMS på storskjerm: «Hei! Jeg er syk i dag. Hilsen Amina.» Elevene skriver den samme meldingen på egen mobil, bytter ut navnet og sender den til læreren. Neste dag byttes ett ord ut (syk → forsinket).</t>
-  </si>
-  <si>
-    <t>Elevene skriver én melding til en venn og én melding til en arbeidsgiver om samme sak, for eksempel at de blir forsinket. De kan skrive eller bruke tale-til-tekst. I par sammenligner de hvordan meldingene er forskjellige.</t>
-  </si>
-  <si>
-    <t>Elevene får et scenario (flytte, invitere, klage på en vare) og velger selv kanal (SMS, e-post eller talemelding) og form ut fra hvem mottakeren er. De begrunner valget sitt for partneren.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en modell-SMS på storskjerm: «Hei! Jeg er syk i dag. Hilsen Amina.» Elevene skriver den samme meldingen på egen mobil, bytter ut navnet og sender den til læreren. Neste dag byttes ett ord ut (syk → forsinket). Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver én melding til en venn og én melding til en arbeidsgiver om samme sak, for eksempel at de blir forsinket. De kan skrive eller bruke tale-til-tekst. I par sammenligner de hvordan meldingene er forskjellige. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene får et scenario (flytte, invitere, klage på en vare) og velger selv kanal (SMS, e-post eller talemelding) og form ut fra hvem mottakeren er. De begrunner valget sitt for partneren. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 3 – Samhandling</t>
@@ -531,13 +639,19 @@
     <t>Samhandler selvstendig i ulike digitale medier og bruker strategier for oppklaring.</t>
   </si>
   <si>
-    <t>Læreren sender en enkel melding i klassechatten: «Kommer du på skolen i morgen?». Elevene svarer med faste fraser fra en frasebank på tavla: «Ja, jeg kommer.» eller «Nei, jeg er syk.»</t>
-  </si>
-  <si>
-    <t>Elevene har en chat-samtale i par der de skal avtale et møte (dag, tid og sted). De bruker frasebanken ved behov, og læreren går rundt og hjelper.</t>
-  </si>
-  <si>
-    <t>Elevene får en chat med en misforståelse (feil tid eller uklar beskjed) og skal oppklare den med strategier som «Mener du …?» og «Kan du forklare?». Klassen sammenligner hvilke strategier som fungerte.</t>
+    <t xml:space="preserve">Forbered: Legg klar fraser før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren sender en enkel melding i klassechatten: «Kommer du på skolen i morgen?». Elevene svarer med faste fraser fra en frasebank på tavla: «Ja, jeg kommer.» eller «Nei, jeg er syk.». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar fraser før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene har en chat-samtale i par der de skal avtale et møte (dag, tid og sted). De bruker frasebanken ved behov, og læreren går rundt og hjelper. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene får en chat med en misforståelse (feil tid eller uklar beskjed) og skal oppklare den med strategier som «Mener du …?» og «Kan du forklare?». Klassen sammenligner hvilke strategier som fungerte. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Grunnleggende ferdigheter</t>
@@ -558,13 +672,19 @@
     <t>Overfører digitale ferdigheter selvstendig i nye norskspråklige sammenhenger.</t>
   </si>
   <si>
-    <t>Elevene viser hverandre hva de allerede kan på mobilen, for eksempel ta bilde eller sende en talemelding. Læreren bygger videre på dette: elevene tar bilde av dagens ordliste og sender det til seg selv, slik at de kan øve hjemme.</t>
-  </si>
-  <si>
-    <t>Hver uke får elevene én digital oppgave knyttet til norsktemaet. Tema bolig: finn en leilighet på Finn.no og skriv tre setninger om den («Leiligheten har … rom. Den koster …»).</t>
-  </si>
-  <si>
-    <t>Elevene bruker det de kan i nye situasjoner, for eksempel ved å legge inn avtaler på norsk i kalenderen på mobilen og sette påminnelser. De viser læreren kalenderen for neste uke.</t>
+    <t xml:space="preserve">Forbered: Legg klar mobilen og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene viser hverandre hva de allerede kan på mobilen, for eksempel ta bilde eller sende en talemelding. Læreren bygger videre på dette: elevene tar bilde av dagens ordliste og sender det til seg selv, slik at de kan øve hjemme. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Hver uke får elevene én digital oppgave knyttet til norsktemaet. Tema bolig: finn en leilighet på Finn.no og skriv tre setninger om den («Leiligheten har … rom. Den koster …»). Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar mobilen før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker det de kan i nye situasjoner, for eksempel ved å legge inn avtaler på norsk i kalenderen på mobilen og sette påminnelser. De viser læreren kalenderen for neste uke. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Digitale ferdigheter</t>
@@ -579,13 +699,19 @@
     <t>Overfører og videreutvikler digitale ferdigheter selvstendig i nye norskspråklige sammenhenger.</t>
   </si>
   <si>
-    <t>Elevene tar opp seg selv på mobilen mens de sier tre setninger om seg selv. Læreren gir en modell først. Elevene lytter til opptaket, prøver igjen og velger det beste opptaket.</t>
-  </si>
-  <si>
-    <t>Hver uke sender elevene en talemelding på norsk til en fast medelev om et gitt tema (f.eks. «Helgen min»), og svarer på medelevens melding. Læreren gir spørsmål som støtte.</t>
-  </si>
-  <si>
-    <t>Elevene lager et kort lydopptak eller en video om et tema, bruker tale-til-tekst for å sjekke om uttalen blir forstått, og deler produktet med klassen for tilbakemelding.</t>
+    <t xml:space="preserve">Forbered: Legg klar mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene tar opp seg selv på mobilen mens de sier tre setninger om seg selv. Læreren gir en modell først. Elevene lytter til opptaket, prøver igjen og velger det beste opptaket. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Hver uke sender elevene en talemelding på norsk til en fast medelev om et gitt tema (f.eks. «Helgen min»), og svarer på medelevens melding. Læreren gir spørsmål som støtte. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene lager et kort lydopptak eller en video om et tema, bruker tale-til-tekst for å sjekke om uttalen blir forstått, og deler produktet med klassen for tilbakemelding. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Digitale ferdigheter integreres der det er relevant for deltakerens nivå og behov.</t>
@@ -600,13 +726,19 @@
     <t>Bruker digitale ferdigheter selvstendig som integrert del av alle språkferdighetene.</t>
   </si>
   <si>
-    <t>I temaet «Å handle» skriver elevene en handleliste i notatappen på mobilen. Læreren gir ord med bilder, og elevene skriver av med støtte.</t>
-  </si>
-  <si>
-    <t>I hvert tema er én oppgave digital for hver ferdighet: lytte (lydklipp), lese (nettside), skrive (melding) og snakke (opptak). Elevene roterer mellom stasjoner, og hver stasjon har en oppgavebeskrivelse med ikoner.</t>
-  </si>
-  <si>
-    <t>Elevene velger selv digitale verktøy som støtter arbeidet i alle ferdigheter, for eksempel opptak for muntlig trening og stavekontroll for skriving, og forklarer valgene sine for læreren.</t>
+    <t xml:space="preserve">Forbered: Legg klar mobilen og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: I temaet «Å handle» skriver elevene en handleliste i notatappen på mobilen. Læreren gir ord med bilder, og elevene skriver av med støtte. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: I hvert tema er én oppgave digital for hver ferdighet: lytte (lydklipp), lese (nettside), skrive (melding) og snakke (opptak). Elevene roterer mellom stasjoner, og hver stasjon har en oppgavebeskrivelse med ikoner. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene velger selv digitale verktøy som støtter arbeidet i alle ferdigheter, for eksempel opptak for muntlig trening og stavekontroll for skriving, og forklarer valgene sine for læreren. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Bruke digitale ressurser til samhandling, informasjonssøk, tekstskaping og dokumentasjon.</t>
@@ -624,13 +756,19 @@
     <t>Bruker digitale ressurser selvstendig til samhandling, søk, tekstskaping og til å dokumentere kompetanse.</t>
   </si>
   <si>
-    <t>Elevene får ett søkeord og en anvist nettside. De finner et bilde som passer, limer det inn i et delt klassedokument og skriver én setning under. Læreren viser hvert trinn på storskjerm.</t>
-  </si>
-  <si>
-    <t>I par finner elevene informasjon om et sted i byen, lager et delt dokument med tekst og bilde, og presenterer det for klassen på ett–to lysbilder.</t>
-  </si>
-  <si>
-    <t>Elevene lager en digital mappe med tekster, lydopptak og skjermbilder som viser hva de kan. De bruker mappen i samtale med læreren, og kan senere vise den til en arbeidsgiver.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, nettsiden og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene får ett søkeord og en anvist nettside. De finner et bilde som passer, limer det inn i et delt klassedokument og skriver én setning under. Læreren viser hvert trinn på storskjerm. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: I par finner elevene informasjon om et sted i byen, lager et delt dokument med tekst og bilde, og presenterer det for klassen på ett–to lysbilder. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene lager en digital mappe med tekster, lydopptak og skjermbilder som viser hva de kan. De bruker mappen i samtale med læreren, og kan senere vise den til en arbeidsgiver. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Håndtere digitale hverdagsoppgaver på norsk.</t>
@@ -645,13 +783,19 @@
     <t>Håndterer nye og ukjente digitale tjenester på norsk selvstendig.</t>
   </si>
   <si>
-    <t>Læreren viser et skjermbilde av en beskjed fra skole eller barnehage i en app. Elevene markerer hva, når og hvor med tre farger. Deretter øver de på å betale med app i en demo- eller øvingsversjon.</t>
-  </si>
-  <si>
-    <t>Stasjonsarbeid med hverdagsoppgaver: sjekke busstider, lese en beskjed fra barnehagen og finne åpningstider på apoteket. Elevene løser oppgavene i par og hjelper hverandre.</t>
-  </si>
-  <si>
-    <t>Elevene prøver en tjeneste de ikke har brukt før, for eksempel å reservere en bok på biblioteket eller bestille time hos frisør. De forteller klassen hvordan de fant ut av tjenesten.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et skjermbilde av en beskjed fra skole eller barnehage i en app. Elevene markerer hva, når og hvor med tre farger. Deretter øver de på å betale med app i en demo- eller øvingsversjon. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Stasjonsarbeid med hverdagsoppgaver: sjekke busstider, lese en beskjed fra barnehagen og finne åpningstider på apoteket. Elevene løser oppgavene i par og hjelper hverandre. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene prøver en tjeneste de ikke har brukt før, for eksempel å reservere en bok på biblioteket eller bestille time hos frisør. De forteller klassen hvordan de fant ut av tjenesten. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Utvikle digital dømmekraft og strategier for nettbruk.</t>
@@ -666,13 +810,19 @@
     <t>Viser selvstendig digital dømmekraft og vurderer digitale verktøy kritisk ut fra formål.</t>
   </si>
   <si>
-    <t>Læreren viser et eksempel på en svindel-SMS («Du har vunnet en iPhone! Trykk her»). Klassen lærer regelen: «Ikke trykk på lenker du ikke kjenner. Spør noen først.» Elevene øver med ekte og falske meldinger og viser tommel opp eller ned.</t>
-  </si>
-  <si>
-    <t>Elevene får fem meldinger og e-poster og sorterer dem i «trygg» og «svindel» ved hjelp av en sjekkliste: Hvem er avsender? Er det en lenke? Haster det veldig?</t>
-  </si>
-  <si>
-    <t>Elevene lager en kort guide om trygg nettbruk til familie eller venner. De vurderer også to verktøy for samme oppgave (f.eks. to oversettelsesapper) ut fra hva de skal brukes til og hvordan de behandler personopplysninger.</t>
+    <t xml:space="preserve">Forbered: Legg klar lenken før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et eksempel på en svindel-SMS («Du har vunnet en iPhone! Trykk her»). Klassen lærer regelen: «Ikke trykk på lenker du ikke kjenner. Spør noen først.» Elevene øver med ekte og falske meldinger og viser tommel opp eller ned. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten, et e-posteksempel og lenken før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får fem meldinger og e-poster og sorterer dem i «trygg» og «svindel» ved hjelp av en sjekkliste: Hvem er avsender? Er det en lenke? Haster det veldig? Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene lager en kort guide om trygg nettbruk til familie eller venner. De vurderer også to verktøy for samme oppgave (f.eks. to oversettelsesapper) ut fra hva de skal brukes til og hvordan de behandler personopplysninger. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – Lese- og skriveforberedende</t>
@@ -693,13 +843,19 @@
     <t>Skriver bokstaver og kjente ord selvstendig og med økende tempo på tastatur.</t>
   </si>
   <si>
-    <t>Elevene finner bokstavene i sitt eget navn på tastaturet ved hjelp av et tastaturkart med store bokstaver. Deretter sier læreren en lyd, og elevene finner og trykker på bokstaven.</t>
-  </si>
-  <si>
-    <t>Elevene skriver ord fra dagens tema etter ordkort med bilder, og øver på stor forbokstav med shift-tasten. Partneren sjekker at ordene er riktige.</t>
-  </si>
-  <si>
-    <t>Elevene skriver kjente ord i et tastaturspill eller skriveprogram med tidtaking, og prøver å slå sin egen rekord fra forrige uke.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene finner bokstavene i sitt eget navn på tastaturet ved hjelp av et tastaturkart med store bokstaver. Deretter sier læreren en lyd, og elevene finner og trykker på bokstaven. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver ord fra dagens tema etter ordkort med bilder, og øver på stor forbokstav med shift-tasten. Partneren sjekker at ordene er riktige. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene skriver kjente ord i et tastaturspill eller skriveprogram med tidtaking, og prøver å slå sin egen rekord fra forrige uke. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Gjenkjenne ord og symboler i digitale tekster (animasjon, reklame).</t>
@@ -714,13 +870,19 @@
     <t>Leser og tolker ord og symboler i varierte digitale tekster selvstendig.</t>
   </si>
   <si>
-    <t>Læreren viser en kort reklamefilm eller animasjon og stopper filmen underveis. Elevene peker på kjente symboler (pris, %, logo) og ord («Tilbud», «Salg») som læreren har vist på forhånd.</t>
-  </si>
-  <si>
-    <t>Elevene blar i en digital tilbudsavis og markerer ord de kjenner igjen. De viser partneren tre ord og sier dem høyt.</t>
-  </si>
-  <si>
-    <t>Elevene ser på ulike digitale tekster – reklame, en advarsel i en app og en informasjonsanimasjon – og forklarer hva ord og symboler betyr.</t>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en kort reklamefilm eller animasjon og stopper filmen underveis. Elevene peker på kjente symboler (pris, %, logo) og ord («Tilbud», «Salg») som læreren har vist på forhånd. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene blar i en digital tilbudsavis og markerer ord de kjenner igjen. De viser partneren tre ord og sier dem høyt. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene ser på ulike digitale tekster – reklame, en advarsel i en app og en informasjonsanimasjon – og forklarer hva ord og symboler betyr. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – Grunnleggende lesing</t>
@@ -738,13 +900,19 @@
     <t>Gjør relevante valg selvstendig i apper, automater og enkle nettsider nødvendige i dagliglivet.</t>
   </si>
   <si>
-    <t>Ikonbingo: Læreren viser et ikon på storskjerm (hjem, søk, tilbake, send, meny) og sier ordet. Elevene finner ikonet på bingobrettet og deretter på egen mobil. Til slutt trykker de på riktig ikon når læreren bare sier ordet.</t>
-  </si>
-  <si>
-    <t>Elevene kjøper en bussbillett i en kjent app trinn for trinn ved hjelp av oppgavekort med skjermbilder. Læreren hjelper ved behov.</t>
-  </si>
-  <si>
-    <t>Elevene løser dagligdagse oppgaver på egen hånd: finne været for i morgen, kjøpe billett i en app og sjekke saldo i nettbanken. De forteller hvilke valg de gjorde.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Ikonbingo: Læreren viser et ikon på storskjerm (hjem, søk, tilbake, send, meny) og sier ordet. Elevene finner ikonet på bingobrettet og deretter på egen mobil. Til slutt trykker de på riktig ikon når læreren bare sier ordet. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene kjøper en bussbillett i en kjent app trinn for trinn ved hjelp av oppgavekort med skjermbilder. Læreren hjelper ved behov. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene løser dagligdagse oppgaver på egen hånd: finne været for i morgen, kjøpe billett i en app og sjekke saldo i nettbanken. De forteller hvilke valg de gjorde. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – Grunnleggende skriving</t>
@@ -762,13 +930,19 @@
     <t>Kommenterer innlegg selvstendig og viser bevissthet om passende innhold.</t>
   </si>
   <si>
-    <t>Læreren legger ut et bilde i en lukket klassegruppe, for eksempel av en matrett. Elevene reagerer med emoji og ett ord, for eksempel «Fint!» eller «Nam!».</t>
-  </si>
-  <si>
-    <t>Elevene legger ut et bilde hver og kommenterer hverandres bilder med faste fraser: «Så fint!», «Hvor er det?», «Jeg liker …».</t>
-  </si>
-  <si>
-    <t>Elevene kommenterer innlegg selvstendig. Klassen diskuterer hva som er passende å skrive offentlig og hva som hører hjemme i private meldinger.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren legger ut et bilde i en lukket klassegruppe, for eksempel av en matrett. Elevene reagerer med emoji og ett ord, for eksempel «Fint!» eller «Nam!». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene legger ut et bilde hver og kommenterer hverandres bilder med faste fraser: «Så fint!», «Hvor er det?», «Jeg liker …». Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene kommenterer innlegg selvstendig. Klassen diskuterer hva som er passende å skrive offentlig og hva som hører hjemme i private meldinger. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Fylle inn personlige opplysninger i enkle digitale skjema.</t>
@@ -783,13 +957,19 @@
     <t>Fyller inn personlige opplysninger på riktig sted i enkle digitale skjema og sender inn selvstendig.</t>
   </si>
   <si>
-    <t>Læreren lager et enkelt digitalt skjema med feltene navn og telefonnummer. Elevene har et kort med egne opplysninger og fyller inn felt for felt mens læreren viser på storskjerm.</t>
-  </si>
-  <si>
-    <t>Skjemaet utvides med adresse og fødselsdato. Elevene øver på riktige formater (dd.mm.åååå, postnummer) og fyller ut skjemaet i par.</t>
-  </si>
-  <si>
-    <t>Elevene fyller inn et ekte skjema, for eksempel påmelding til et bibliotekarrangement, sjekker opplysningene og sender det inn selv.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, skjemaet og kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren lager et enkelt digitalt skjema med feltene navn og telefonnummer. Elevene har et kort med egne opplysninger og fyller inn felt for felt mens læreren viser på storskjerm. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Skjemaet utvides med adresse og fødselsdato. Elevene øver på riktige formater (dd.mm.åååå, postnummer) og fyller ut skjemaet i par. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene fyller inn et ekte skjema, for eksempel påmelding til et bibliotekarrangement, sjekker opplysningene og sender det inn selv. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Videreformidle informasjon fra enkle digitale og visuelle tekster.</t>
@@ -804,13 +984,19 @@
     <t>Videreformidler muntlig relevant informasjon fra enkle digitale tekster selvstendig.</t>
   </si>
   <si>
-    <t>Læreren viser en kort animasjon med lite tekst og stopper den underveis: «Hva ser du?». Elevene peker på skjermen og sier ett–to ord.</t>
-  </si>
-  <si>
-    <t>Elevene ser en kort reklamefilm og gjenforteller med bildestøtte og setningsstartere: «Det er en reklame for … Den koster …».</t>
-  </si>
-  <si>
-    <t>Elevene ser en kort informasjonsvideo, for eksempel fra kommunen, og forteller partneren det viktigste. Partneren sjekker mot videoen.</t>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en kort animasjon med lite tekst og stopper den underveis: «Hva ser du?». Elevene peker på skjermen og sier ett–to ord. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar setningsstartere, bilder og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene ser en kort reklamefilm og gjenforteller med bildestøtte og setningsstartere: «Det er en reklame for … Den koster …». Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene ser en kort informasjonsvideo, for eksempel fra kommunen, og forteller partneren det viktigste. Partneren sjekker mot videoen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A1 lytte</t>
@@ -828,13 +1014,19 @@
     <t>Finner og bruker enkle digitale lytte-/videoressurser selvstendig.</t>
   </si>
   <si>
-    <t>Læreren spiller korte digitale klipp med tall og ukedager flere ganger. Elevene holder opp kort med ordet eller tallet de hører.</t>
-  </si>
-  <si>
-    <t>Elevene spiller av korte klipp på egen PC med hodetelefoner i sitt eget tempo, og krysser av informasjonen de hører på et arbeidsark.</t>
-  </si>
-  <si>
-    <t>Elevene finner selv lyttestoff på et anbefalt nettsted på sitt nivå og lager en liste over ord og informasjon de forsto.</t>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren spiller korte digitale klipp med tall og ukedager flere ganger. Elevene holder opp kort med ordet eller tallet de hører. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene spiller av korte klipp på egen PC med hodetelefoner i sitt eget tempo, og krysser av informasjonen de hører på et arbeidsark. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene finner selv lyttestoff på et anbefalt nettsted på sitt nivå og lager en liste over ord og informasjon de forsto. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Skrive ved bruk av tilpassede dataprogrammer og apper.</t>
@@ -849,13 +1041,19 @@
     <t>Skriver selvstendig i tilpassede dataprogrammer og bruker støttefunksjoner hensiktsmessig.</t>
   </si>
   <si>
-    <t>Elevene bruker en skriveapp som sier bokstavene høyt, og skriver ord til bilder. Læreren sitter ved og viser.</t>
-  </si>
-  <si>
-    <t>Elevene skriver korte tekster i et tekstprogram og øver på å lagre filen og rette feil med stavekontrollen.</t>
-  </si>
-  <si>
-    <t>Elevene bruker støttefunksjoner som ordforslag, opplesning og stavekontroll, og vurderer når de hjelper og når de ikke gjør det.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene bruker en skriveapp som sier bokstavene høyt, og skriver ord til bilder. Læreren sitter ved og viser. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver korte tekster i et tekstprogram og øver på å lagre filen og rette feil med stavekontrollen. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker støttefunksjoner som ordforslag, opplesning og stavekontroll, og vurderer når de hjelper og når de ikke gjør det. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A1 lese</t>
@@ -876,13 +1074,19 @@
     <t>Navigerer selvstendig på enkle autentiske nettsider og finner ord og fraser.</t>
   </si>
   <si>
-    <t>Læreren åpner nettsiden til en matbutikk på storskjerm. Elevene finner kjente ord (melk, brød, epler) og navn, og kommer fram og peker.</t>
-  </si>
-  <si>
-    <t>Elevene åpner selv en kjent nettside (bibliotek eller kommune) og finner fem kjente ord eller fraser, som de skriver i en liste.</t>
-  </si>
-  <si>
-    <t>Elevene navigerer på enkle autentiske nettsider for å finne åpningstider, priser eller tilbud, og noterer det de finner.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren åpner nettsiden til en matbutikk på storskjerm. Elevene finner kjente ord (melk, brød, epler) og navn, og kommer fram og peker. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene åpner selv en kjent nettside (bibliotek eller kommune) og finner fem kjente ord eller fraser, som de skriver i en liste. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene navigerer på enkle autentiske nettsider for å finne åpningstider, priser eller tilbud, og noterer det de finner. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A1 skrive</t>
@@ -900,13 +1104,19 @@
     <t>Skriver og kommenterer enkle innlegg selvstendig og bruker passende hilsen/avslutning.</t>
   </si>
   <si>
-    <t>Læreren viser en modell: «Hei! I dag spiser jeg fisk.» Elevene skriver et eget innlegg på én–to setninger i den lukkede klassegruppen.</t>
-  </si>
-  <si>
-    <t>Elevene skriver et innlegg om helgen og kommenterer to av medelevenes innlegg.</t>
-  </si>
-  <si>
-    <t>Elevene skriver og kommenterer innlegg med passende hilsen og avslutning, og tilpasser språket til hvem som skal lese det.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en modell: «Hei! I dag spiser jeg fisk.» Elevene skriver et eget innlegg på én–to setninger i den lukkede klassegruppen. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver et innlegg om helgen og kommenterer to av medelevenes innlegg. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene skriver og kommenterer innlegg med passende hilsen og avslutning, og tilpasser språket til hvem som skal lese det. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Fylle inn personlige opplysninger i nettskjemaer og apper.</t>
@@ -921,13 +1131,19 @@
     <t>Fyller inn og sender inn enkle nettskjemaer selvstendig og kontrollerer opplysningene.</t>
   </si>
   <si>
-    <t>Læreren viser et nettskjema på storskjerm. Elevene fyller inn felt for felt ved hjelp av eget kort med personopplysninger, mens læreren viser hvert felt.</t>
-  </si>
-  <si>
-    <t>Elevene registrerer seg i en app (f.eks. bibliotekets app) ved hjelp av oppgavekort med skjermbilder.</t>
-  </si>
-  <si>
-    <t>Elevene fyller inn og sender inn skjemaer selv, og kontrollerer opplysningene mot en sjekkliste før de trykker «send».</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, skjemaet og kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et nettskjema på storskjerm. Elevene fyller inn felt for felt ved hjelp av eget kort med personopplysninger, mens læreren viser hvert felt. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene registrerer seg i en app (f.eks. bibliotekets app) ved hjelp av oppgavekort med skjermbilder. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten og skjemaet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene fyller inn og sender inn skjemaer selv, og kontrollerer opplysningene mot en sjekkliste før de trykker «send». Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A2 lese</t>
@@ -945,13 +1161,19 @@
     <t>Søker selvstendig på nett og finner og forstår spesifikk informasjon.</t>
   </si>
   <si>
-    <t>Læreren gir et søkeord og en nettside: «Finn prisen på en liter melk.» Elevene søker og skriver svaret.</t>
-  </si>
-  <si>
-    <t>Elevene bruker søkefeltet og menyene på en kjent nettside for å finne informasjon, for eksempel åpningstidene til svømmehallen.</t>
-  </si>
-  <si>
-    <t>Elevene får oppgaven «Planlegg en tur på lørdag». De søker selv etter tider, priser og værmelding, og forteller partneren planen.</t>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren gir et søkeord og en nettside: «Finn prisen på en liter melk.» Elevene søker og skriver svaret. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker søkefeltet og menyene på en kjent nettside for å finne informasjon, for eksempel åpningstidene til svømmehallen. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene får oppgaven «Planlegg en tur på lørdag». De søker selv etter tider, priser og værmelding, og forteller partneren planen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A2 skrive</t>
@@ -969,13 +1191,19 @@
     <t>Skriver, svarer og kommenterer enkelt selvstendig i digital kommunikasjon.</t>
   </si>
   <si>
-    <t>Elevene får en invitasjon i en melding: «Vil du komme på kaffe på lørdag?». De svarer ved hjelp av en modell: «Ja, takk! Jeg kommer klokka …».</t>
-  </si>
-  <si>
-    <t>Elevene skriver og svarer på meldinger i klassekanalen om en felles aktivitet, for eksempel en tur eller et spleiselag.</t>
-  </si>
-  <si>
-    <t>Elevene svarer og kommenterer selvstendig, også på meldinger de ikke har forberedt seg på.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene får en invitasjon i en melding: «Vil du komme på kaffe på lørdag?». De svarer ved hjelp av en modell: «Ja, takk! Jeg kommer klokka …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver og svarer på meldinger i klassekanalen om en felles aktivitet, for eksempel en tur eller et spleiselag. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene svarer og kommenterer selvstendig, også på meldinger de ikke har forberedt seg på. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Skrive korte og enkle e-poster og personlige brev.</t>
@@ -990,13 +1218,19 @@
     <t>Skriver og sender enkle e-poster selvstendig, også med vedlegg.</t>
   </si>
   <si>
-    <t>Elevene skriver en e-post etter mal («Hei …, jeg …, Hilsen …») med støtte fra læreren, og sender den til læreren.</t>
-  </si>
-  <si>
-    <t>Elevene skriver en e-post til læreren om fravær. De øver på å skrive inn riktig mottaker, emnefelt og innhold.</t>
-  </si>
-  <si>
-    <t>Elevene skriver og sender en e-post med vedlegg, for eksempel et bilde eller et dokument, og sjekker at vedlegget kom fram.</t>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene skriver en e-post etter mal («Hei …, jeg …, Hilsen …») med støtte fra læreren, og sender den til læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver en e-post til læreren om fravær. De øver på å skrive inn riktig mottaker, emnefelt og innhold. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel og bilder før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene skriver og sender en e-post med vedlegg, for eksempel et bilde eller et dokument, og sjekker at vedlegget kom fram. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Fylle inn opplysninger i digitale skjemaer (netthandel, bank, bestillinger).</t>
@@ -1011,13 +1245,19 @@
     <t>Bruker digitale tjenester selvstendig (netthandel, bank, bestilling, påmelding).</t>
   </si>
   <si>
-    <t>Læreren bruker en øvingsnettbutikk på storskjerm. Elevene fyller inn navn og adresse i bestillingsskjemaet med veiledning.</t>
-  </si>
-  <si>
-    <t>Elevene bestiller en vare i øvingsnettbutikken eller melder seg på et kurs, og viser partneren bekreftelsen.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale tjenester selvstendig, for eksempel for å bestille time eller melde seg på en aktivitet, og forteller klassen hvordan de gjorde det.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og skjemaet før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren bruker en øvingsnettbutikk på storskjerm. Elevene fyller inn navn og adresse i bestillingsskjemaet med veiledning. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bestiller en vare i øvingsnettbutikken eller melder seg på et kurs, og viser partneren bekreftelsen. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale tjenester selvstendig, for eksempel for å bestille time eller melde seg på en aktivitet, og forteller klassen hvordan de gjorde det. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Presentere egen kompetanse i en enkel CV og digitalt skjema.</t>
@@ -1032,13 +1272,19 @@
     <t>Presenterer egen kompetanse selvstendig i digital CV og oppdaterer ved behov.</t>
   </si>
   <si>
-    <t>Elevene fyller inn en enkel CV-mal (navn, adresse, språk, erfaring) med hjelp fra læreren. Læreren viser en ferdig CV som modell.</t>
-  </si>
-  <si>
-    <t>Elevene lager en CV i et tekstprogram og fyller inn et digitalt kompetanseskjema. Partneren leser og gir én tilbakemelding.</t>
-  </si>
-  <si>
-    <t>Elevene oppdaterer sin egen CV og tilpasser den til en ekte stillingsannonse de har funnet.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene fyller inn en enkel CV-mal (navn, adresse, språk, erfaring) med hjelp fra læreren. Læreren viser en ferdig CV som modell. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene lager en CV i et tekstprogram og fyller inn et digitalt kompetanseskjema. Partneren leser og gir én tilbakemelding. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene oppdaterer sin egen CV og tilpasser den til en ekte stillingsannonse de har funnet. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A2 muntlig</t>
@@ -1056,13 +1302,19 @@
     <t>Lager og bruker digitale verktøy selvstendig i presentasjon.</t>
   </si>
   <si>
-    <t>Elevene lager sammen med læreren to–tre lysbilder om seg selv (ett bilde og én setning per lysbilde) og presenterer for en liten gruppe.</t>
-  </si>
-  <si>
-    <t>Elevene lager lysbilder selv om hjemlandet eller en hobby, og bruker dem i en kort presentasjon for klassen.</t>
-  </si>
-  <si>
-    <t>Elevene velger selv presentasjonsverktøy, lager en presentasjon med bilder og tekst og presenterer for klassen.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene lager sammen med læreren to–tre lysbilder om seg selv (ett bilde og én setning per lysbilde) og presenterer for en liten gruppe. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene lager lysbilder selv om hjemlandet eller en hobby, og bruker dem i en kort presentasjon for klassen. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene velger selv presentasjonsverktøy, lager en presentasjon med bilder og tekst og presenterer for klassen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B1 lese</t>
@@ -1080,13 +1332,19 @@
     <t>Søker selvstendig på tvers av nettsider og digitale dokumenter.</t>
   </si>
   <si>
-    <t>Læreren viser helsenorge.no på storskjerm. Elevene finner informasjon om hvordan man bytter fastlege, med veiledning trinn for trinn.</t>
-  </si>
-  <si>
-    <t>Elevene får oppgavekort med spørsmål om rettigheter (f.eks. barnetrygd eller foreldrepenger) og søker etter svar på nav.no og andre offentlige nettsider.</t>
-  </si>
-  <si>
-    <t>Elevene løser et praktisk problem, for eksempel «Du skal flytte – hva må du gjøre?». De søker på tvers av offentlige nettsider og dokumenter og lager en sjekkliste.</t>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser helsenorge.no på storskjerm. Elevene finner informasjon om hvordan man bytter fastlege, med veiledning trinn for trinn. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får oppgavekort med spørsmål om rettigheter (f.eks. barnetrygd eller foreldrepenger) og søker etter svar på nav.no og andre offentlige nettsider. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten og nettsiden før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene løser et praktisk problem, for eksempel «Du skal flytte – hva må du gjøre?». De søker på tvers av offentlige nettsider og dokumenter og lager en sjekkliste. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B1 skrive</t>
@@ -1104,13 +1362,19 @@
     <t>Deltar selvstendig i digitale diskusjoner med saklig tone og respekt.</t>
   </si>
   <si>
-    <t>Elevene skriver et innlegg og en kommentar i et lukket digitalt forum ved hjelp av setningsstartere som «Jeg mener at …» og «Jeg er enig fordi …».</t>
-  </si>
-  <si>
-    <t>Elevene deltar i en digital diskusjon om et hverdagstema og svarer på minst to medelevers innlegg.</t>
-  </si>
-  <si>
-    <t>Elevene deltar selvstendig i digitale diskusjoner med saklig tone, og vurderer etterpå sin egen tone ut fra klassens regler.</t>
+    <t xml:space="preserve">Forbered: Legg klar setningsstartere før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene skriver et innlegg og en kommentar i et lukket digitalt forum ved hjelp av setningsstartere som «Jeg mener at …» og «Jeg er enig fordi …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene deltar i en digital diskusjon om et hverdagstema og svarer på minst to medelevers innlegg. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene deltar selvstendig i digitale diskusjoner med saklig tone, og vurderer etterpå sin egen tone ut fra klassens regler. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Skrive enkle formelle e-poster.</t>
@@ -1125,13 +1389,19 @@
     <t>Skriver og sender formelle e-poster med vedlegg selvstendig.</t>
   </si>
   <si>
-    <t>Elevene skriver en enkel formell e-post etter mal, for eksempel til en arbeidsgiver for å spørre om praksisplass. Læreren viser hvordan en formell e-post skiller seg fra en SMS.</t>
-  </si>
-  <si>
-    <t>Elevene skriver en formell e-post og legger ved CV eller søknad. Partneren sjekker hilsen, emnefelt og vedlegg.</t>
-  </si>
-  <si>
-    <t>Elevene skriver og sender formelle e-poster med vedlegg selvstendig, for eksempel til en ekte arbeidsgiver eller til NAV.</t>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene skriver en enkel formell e-post etter mal, for eksempel til en arbeidsgiver for å spørre om praksisplass. Læreren viser hvordan en formell e-post skiller seg fra en SMS. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver en formell e-post og legger ved CV eller søknad. Partneren sjekker hilsen, emnefelt og vedlegg. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene skriver og sender formelle e-poster med vedlegg selvstendig, for eksempel til en ekte arbeidsgiver eller til NAV. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Skrive inn opplysninger i ulike typer digitale skjemaer.</t>
@@ -1146,13 +1416,19 @@
     <t>Håndterer ulike typer digitale skjema i offentlige og private tjenester selvstendig.</t>
   </si>
   <si>
-    <t>Elevene fyller ut et lengre digitalt skjema (f.eks. en søknad) med veiledning fra læreren. Læreren viser hvert felt og forklarer ukjente ord.</t>
-  </si>
-  <si>
-    <t>Elevene øver på å logge inn med BankID og laste opp et dokument i et øvingsskjema eller en ekte tjeneste.</t>
-  </si>
-  <si>
-    <t>Elevene fyller ut ulike skjemaer selv, både i offentlige og private tjenester, og forteller hva som var vanskelig.</t>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene fyller ut et lengre digitalt skjema (f.eks. en søknad) med veiledning fra læreren. Læreren viser hvert felt og forklarer ukjente ord. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene øver på å logge inn med BankID og laste opp et dokument i et øvingsskjema eller en ekte tjeneste. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene fyller ut ulike skjemaer selv, både i offentlige og private tjenester, og forteller hva som var vanskelig. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B1 muntlig</t>
@@ -1170,13 +1446,19 @@
     <t>Velger og bruker digitale presentasjonsverktøy selvstendig og hensiktsmessig.</t>
   </si>
   <si>
-    <t>Elevene lager en presentasjon med lysbilder etter en mal og holder den med støtte fra læreren.</t>
-  </si>
-  <si>
-    <t>Elevene lager en strukturert presentasjon med tekst, bilder og lyd eller video, og holder den for klassen.</t>
-  </si>
-  <si>
-    <t>Elevene velger selv presentasjonsverktøy og bruker det hensiktsmessig i en presentasjon for klassen.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene lager en presentasjon med lysbilder etter en mal og holder den med støtte fra læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene lager en strukturert presentasjon med tekst, bilder og lyd eller video, og holder den for klassen. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene velger selv presentasjonsverktøy og bruker det hensiktsmessig i en presentasjon for klassen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B2 lese</t>
@@ -1194,13 +1476,19 @@
     <t>Bruker søketeknikker og lesemåter selvstendig og effektivt på tvers av nettsteder.</t>
   </si>
   <si>
-    <t>Læreren viser hvordan søkeord og enkle filtre (dato, sted) virker. Elevene øver på samme søk med veiledning.</t>
-  </si>
-  <si>
-    <t>Elevene øver på ulike søketeknikker og skumlesing: de får fem spørsmål og skal finne svarene så raskt som mulig på ulike nettsider.</t>
-  </si>
-  <si>
-    <t>Elevene bruker søketeknikker og lesemåter selvstendig for å løse en sammensatt oppgave, for eksempel å sammenligne tre kurs eller tre boliger.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser hvordan søkeord og enkle filtre (dato, sted) virker. Elevene øver på samme søk med veiledning. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene øver på ulike søketeknikker og skumlesing: de får fem spørsmål og skal finne svarene så raskt som mulig på ulike nettsider. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker søketeknikker og lesemåter selvstendig for å løse en sammensatt oppgave, for eksempel å sammenligne tre kurs eller tre boliger. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B2 skrive</t>
@@ -1221,13 +1509,19 @@
     <t>Deltar selvstendig i digitale diskusjoner med nyansert argumentasjon.</t>
   </si>
   <si>
-    <t>Elevene uttrykker meninger i et lukket forum med støtte fra en frasebank med nyanserte uttrykk: «På den ene siden …, på den andre siden …».</t>
-  </si>
-  <si>
-    <t>Elevene diskuterer og kommenterer i et digitalt forum om en aktuell sak, og bruker minst ett argument og ett motargument.</t>
-  </si>
-  <si>
-    <t>Elevene deltar i en digital diskusjon med nyansert argumentasjon og viser til kilder.</t>
+    <t xml:space="preserve">Forbered: Legg klar fraser før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene uttrykker meninger i et lukket forum med støtte fra en frasebank med nyanserte uttrykk: «På den ene siden …, på den andre siden …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene diskuterer og kommenterer i et digitalt forum om en aktuell sak, og bruker minst ett argument og ett motargument. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene deltar i en digital diskusjon med nyansert argumentasjon og viser til kilder. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Skrive detaljerte beskjeder, e-poster og brev.</t>
@@ -1242,13 +1536,19 @@
     <t>Skriver selvstendig detaljerte e-poster tilpasset mottaker og formål.</t>
   </si>
   <si>
-    <t>Elevene skriver en detaljert e-post etter modell, for eksempel en klage på en vare, med støtte fra læreren.</t>
-  </si>
-  <si>
-    <t>Elevene skriver en detaljert e-post tilpasset mottakeren, for eksempel til utleier om en skade i leiligheten.</t>
-  </si>
-  <si>
-    <t>Elevene skriver selvstendig detaljerte e-poster tilpasset mottaker og formål, og vurderer tone og innhold i etterkant.</t>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene skriver en detaljert e-post etter modell, for eksempel en klage på en vare, med støtte fra læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene skriver en detaljert e-post tilpasset mottakeren, for eksempel til utleier om en skade i leiligheten. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene skriver selvstendig detaljerte e-poster tilpasset mottaker og formål, og vurderer tone og innhold i etterkant. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B2 muntlig</t>
@@ -1266,13 +1566,19 @@
     <t>Bruker digitale verktøy selvstendig og profesjonelt i presentasjoner.</t>
   </si>
   <si>
-    <t>Elevene holder en velstrukturert presentasjon med digitale lysbilder etter mal (innledning – hoveddel – avslutning).</t>
-  </si>
-  <si>
-    <t>Elevene lager selv en velstrukturert digital presentasjon om et fagtema og får tilbakemelding fra medelever.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale verktøy selvstendig og profesjonelt i en presentasjon, for eksempel i en rollespilt jobbsituasjon.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene holder en velstrukturert presentasjon med digitale lysbilder etter mal (innledning – hoveddel – avslutning). Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene lager selv en velstrukturert digital presentasjon om et fagtema og får tilbakemelding fra medelever. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale verktøy selvstendig og profesjonelt i en presentasjon, for eksempel i en rollespilt jobbsituasjon. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – A2 lytte</t>
@@ -1290,13 +1596,19 @@
     <t>Forstår enkel informasjon i digitale presentasjoner og kan notere stikkord.</t>
   </si>
   <si>
-    <t>Læreren holder en enkel digital presentasjon med tydelige bilder og stopper ofte. Elevene svarer på ja/nei-spørsmål.</t>
-  </si>
-  <si>
-    <t>Elevene ser en kort digital presentasjon eller video og svarer på spørsmål om det viktigste innholdet.</t>
-  </si>
-  <si>
-    <t>Elevene ser en digital presentasjon og noterer stikkord, som de bruker til å fortelle partneren om innholdet.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren holder en enkel digital presentasjon med tydelige bilder og stopper ofte. Elevene svarer på ja/nei-spørsmål. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene ser en kort digital presentasjon eller video og svarer på spørsmål om det viktigste innholdet. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene ser en digital presentasjon og noterer stikkord, som de bruker til å fortelle partneren om innholdet. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Oppfatte viktig informasjon fra korte digitale klipp.</t>
@@ -1311,13 +1623,19 @@
     <t>Bruker nyhets- og videotjenester selvstendig for å holde seg informert.</t>
   </si>
   <si>
-    <t>Læreren spiller av et kort klipp, for eksempel en værmelding, to–tre ganger. Elevene finner viktig informasjon (temperatur, vær) med bildestøtte.</t>
-  </si>
-  <si>
-    <t>Elevene finner og spiller av korte klipp selv fra kjente kilder, for eksempel NRK, og forteller partneren hva klippet handlet om.</t>
-  </si>
-  <si>
-    <t>Elevene bruker nyhets- og videotjenester selvstendig for å følge med på nyheter, og forteller om én nyhet i klassen hver uke.</t>
+    <t xml:space="preserve">Forbered: Legg klar klippet, bilder og kort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren spiller av et kort klipp, for eksempel en værmelding, to–tre ganger. Elevene finner viktig informasjon (temperatur, vær) med bildestøtte. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene finner og spiller av korte klipp selv fra kjente kilder, for eksempel NRK, og forteller partneren hva klippet handlet om. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker nyhets- og videotjenester selvstendig for å følge med på nyheter, og forteller om én nyhet i klassen hver uke. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B1 lytte</t>
@@ -1335,13 +1653,19 @@
     <t>Bruker digitale medier selvstendig og kritisk som kilde til informasjon.</t>
   </si>
   <si>
-    <t>Læreren velger et klipp eller en podkastepisode og gir elevene spørsmål før de lytter. Elevene finner hovedpunktene med støtte.</t>
-  </si>
-  <si>
-    <t>Elevene finner og bruker podkaster og filmer i strømmetjenester, og skriver tre hovedpunkter fra det de har lyttet til.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale medier selvstendig og kritisk: de lytter til to kilder om samme tema og sammenligner hovedpunktene.</t>
+    <t xml:space="preserve">Forbered: Legg klar klippet før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren velger et klipp eller en podkastepisode og gir elevene spørsmål før de lytter. Elevene finner hovedpunktene med støtte. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene finner og bruker podkaster og filmer i strømmetjenester, og skriver tre hovedpunkter fra det de har lyttet til. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale medier selvstendig og kritisk: de lytter til to kilder om samme tema og sammenligner hovedpunktene. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Lese og forstå hverdagslige tekster på digitale flater.</t>
@@ -1356,13 +1680,19 @@
     <t>Leser og forstår hverdagslige digitale tekster og skiller mellom fakta, meninger og reklame.</t>
   </si>
   <si>
-    <t>Elevene leser en hverdagslig e-post, for eksempel fra skolen, med støtte fra læreren, og finner hva, når og hvor.</t>
-  </si>
-  <si>
-    <t>Elevene leser e-poster og innlegg på sosiale medier og svarer på spørsmål om innholdet.</t>
-  </si>
-  <si>
-    <t>Elevene leser hverdagslige digitale tekster og sorterer utsagn i fakta, meninger og reklame.</t>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene leser en hverdagslig e-post, for eksempel fra skolen, med støtte fra læreren, og finner hva, når og hvor. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene leser e-poster og innlegg på sosiale medier og svarer på spørsmål om innholdet. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene leser hverdagslige digitale tekster og sorterer utsagn i fakta, meninger og reklame. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 6 – B2 lytte</t>
@@ -1380,13 +1710,19 @@
     <t>Finner selv relevant digitalt lytte-/videomateriale og forstår det.</t>
   </si>
   <si>
-    <t>Læreren velger ut digitalt lyttestoff og gir elevene en ordliste før de lytter. Elevene svarer på spørsmål om innholdet.</t>
-  </si>
-  <si>
-    <t>Elevene finner selv relevant digitalt lytte- eller videostoff, lytter og lager et kort sammendrag.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale medier selvstendig og kritisk, og vurderer hvem som står bak, og hva hensikten er.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren velger ut digitalt lyttestoff og gir elevene en ordliste før de lytter. Elevene svarer på spørsmål om innholdet. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene finner selv relevant digitalt lytte- eller videostoff, lytter og lager et kort sammendrag. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale medier selvstendig og kritisk, og vurderer hvem som står bak, og hva hensikten er. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Forstå informasjonsutveksling i formelle og uformelle digitale tekster.</t>
@@ -1401,13 +1737,19 @@
     <t>Forstår formell og uformell digital informasjonsutveksling og oppfatter tone og hensikt.</t>
   </si>
   <si>
-    <t>Elevene leser en formell digital melding, for eksempel fra NAV eller Skatteetaten, med støtte fra læreren, og finner det vesentligste: hva må jeg gjøre, og når?</t>
-  </si>
-  <si>
-    <t>Elevene sammenligner en formell e-post og et uformelt innlegg om samme tema, og finner forskjeller i språk og tone.</t>
-  </si>
-  <si>
-    <t>Elevene leser ulike digitale tekster og vurderer tone og hensikt: Er dette en informasjon, en klage, et salgsforsøk eller en invitasjon?</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Elevene leser en formell digital melding, for eksempel fra NAV eller Skatteetaten, med støtte fra læreren, og finner det vesentligste: hva må jeg gjøre, og når? Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene sammenligner en formell e-post og et uformelt innlegg om samme tema, og finner forskjeller i språk og tone. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene leser ulike digitale tekster og vurderer tone og hensikt: Er dette en informasjon, en klage, et salgsforsøk eller en invitasjon? Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Samfunn</t>
@@ -1425,13 +1767,19 @@
     <t>Viser digital dømmekraft i egne vurderinger og kan begrunne valg med referanse til personvern og etikk.</t>
   </si>
   <si>
-    <t>Læreren forklarer begrepet digital dømmekraft med bilder av trygge og utrygge situasjoner på nett (dele passord, klikke på ukjente lenker, bruke BankID riktig). Elevene sorterer bildene i «trygt» og «utrygt» og lager sammen en liste med tre regler.</t>
-  </si>
-  <si>
-    <t>Elevene drøfter eksempler fra eget liv i par: deling av bilder, falske nyheter og svindel. De skriver ned ett eksempel og hva de gjorde eller burde ha gjort.</t>
-  </si>
-  <si>
-    <t>Elevene vurderer en ukjent situasjon (f.eks. en venneforespørsel fra en fremmed eller en melding om en «pakke på vei») og begrunner valget sitt med henvisning til personvern og etikk.</t>
+    <t xml:space="preserve">Forbered: Legg klar lenken og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren forklarer begrepet digital dømmekraft med bilder av trygge og utrygge situasjoner på nett (dele passord, klikke på ukjente lenker, bruke BankID riktig). Elevene sorterer bildene i «trygt» og «utrygt» og lager sammen en liste med tre regler. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene drøfter eksempler fra eget liv i par: deling av bilder, falske nyheter og svindel. De skriver ned ett eksempel og hva de gjorde eller burde ha gjort. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene vurderer en ukjent situasjon (f.eks. en venneforespørsel fra en fremmed eller en melding om en «pakke på vei») og begrunner valget sitt med henvisning til personvern og etikk. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 2 – Perspektivmangfold</t>
@@ -1449,13 +1797,19 @@
     <t>Finner, sammenligner og vurderer digitale kilder selvstendig.</t>
   </si>
   <si>
-    <t>Læreren gir en lenke til en offentlig nettside, og elevene finner svar på et konkret spørsmål. Deretter viser læreren en upålitelig side om samme tema, og klassen snakker om hvorfor alle kilder ikke er pålitelige.</t>
-  </si>
-  <si>
-    <t>Elevene bruker to–tre digitale kilder om samme tema, og vurderer enkelt: Hvem er avsender? Hva vil de oppnå? Er informasjonen ny?</t>
-  </si>
-  <si>
-    <t>Elevene finner, sammenligner og vurderer digitale kilder selvstendig, og lager en kort oversikt over hvilke kilder de stoler på og hvorfor.</t>
+    <t xml:space="preserve">Forbered: Legg klar lenken og nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren gir en lenke til en offentlig nettside, og elevene finner svar på et konkret spørsmål. Deretter viser læreren en upålitelig side om samme tema, og klassen snakker om hvorfor alle kilder ikke er pålitelige. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker to–tre digitale kilder om samme tema, og vurderer enkelt: Hvem er avsender? Hva vil de oppnå? Er informasjonen ny? Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene finner, sammenligner og vurderer digitale kilder selvstendig, og lager en kort oversikt over hvilke kilder de stoler på og hvorfor. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 4 – Digitale ferdigheter</t>
@@ -1473,13 +1827,19 @@
     <t>Tilegner seg selvstendig informasjon og kunnskap gjennom digital teknologi.</t>
   </si>
   <si>
-    <t>Læreren viser viktige digitale kanaler for samfunnsinformasjon, for eksempel kommunens nettside, nav.no og helsenorge.no. Elevene åpner kanalene med støtte og finner én opplysning på hver.</t>
-  </si>
-  <si>
-    <t>Elevene får oppgaver der de skal finne samfunnsinformasjon, for eksempel om skolestart eller valg, og bruker digitale kanaler delvis selvstendig.</t>
-  </si>
-  <si>
-    <t>Elevene tilegner seg informasjon selvstendig om et samfunnsspørsmål de er interessert i, og presenterer det de har lært.</t>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser viktige digitale kanaler for samfunnsinformasjon, for eksempel kommunens nettside, nav.no og helsenorge.no. Elevene åpner kanalene med støtte og finner én opplysning på hver. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene får oppgaver der de skal finne samfunnsinformasjon, for eksempel om skolestart eller valg, og bruker digitale kanaler delvis selvstendig. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene tilegner seg informasjon selvstendig om et samfunnsspørsmål de er interessert i, og presenterer det de har lært. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Utvikle digital dømmekraft og bevissthet om nettbruk.</t>
@@ -1494,13 +1854,19 @@
     <t>Viser digital dømmekraft og bevisst nettbruk og kan veilede andre.</t>
   </si>
   <si>
-    <t>Læreren forklarer med bilder hva Norge som digitalt samfunn betyr: BankID, digital postkasse og digitale tjenester. Elevene kobler bilde og ord, og forteller hvilke tjenester de har brukt.</t>
-  </si>
-  <si>
-    <t>Elevene drøfter i par muligheter og utfordringer ved digital samhandling, for eksempel at det er raskt, men at ikke alle har tilgang. De skriver to fordeler og to ulemper.</t>
-  </si>
-  <si>
-    <t>Elevene viser digital dømmekraft og bevisst nettbruk ved å veilede en medelev eller et familiemedlem i å bruke en digital tjeneste trygt.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren forklarer med bilder hva Norge som digitalt samfunn betyr: BankID, digital postkasse og digitale tjenester. Elevene kobler bilde og ord, og forteller hvilke tjenester de har brukt. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene drøfter i par muligheter og utfordringer ved digital samhandling, for eksempel at det er raskt, men at ikke alle har tilgang. De skriver to fordeler og to ulemper. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene viser digital dømmekraft og bevisst nettbruk ved å veilede en medelev eller et familiemedlem i å bruke en digital tjeneste trygt. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Vise etisk refleksjon og vurdering av egen rolle på nett.</t>
@@ -1515,13 +1881,19 @@
     <t>Reflekterer selvstendig og etisk over egen rolle på nett og handler tilsvarende.</t>
   </si>
   <si>
-    <t>Læreren viser eksempler på enkle etiske regler for sosiale medier: spør før du deler bilder, vær vennlig og ikke del falske nyheter. Elevene kobler hver regel til et eksempel.</t>
-  </si>
-  <si>
-    <t>Elevene drøfter dilemmaer knyttet til egen rolle på nett, for eksempel om man skal dele en video av en krangel, og vurderer egne vaner.</t>
-  </si>
-  <si>
-    <t>Elevene reflekterer selvstendig og etisk over sin egen rolle på nett, og lager tre personlige regler de vil følge.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser eksempler på enkle etiske regler for sosiale medier: spør før du deler bilder, vær vennlig og ikke del falske nyheter. Elevene kobler hver regel til et eksempel. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene drøfter dilemmaer knyttet til egen rolle på nett, for eksempel om man skal dele en video av en krangel, og vurderer egne vaner. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene reflekterer selvstendig og etisk over sin egen rolle på nett, og lager tre personlige regler de vil følge. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Forstå at digitale ferdigheter er forutsetning for arbeids- og samfunnsliv.</t>
@@ -1536,13 +1908,19 @@
     <t>Bruker digitale ferdigheter selvstendig til videre læring og deltakelse.</t>
   </si>
   <si>
-    <t>Læreren viser bilder av ulike yrker og hvilke digitale ferdigheter som trengs (f.eks. vaktliste i app for en renholder, e-post for en kontorarbeider). Elevene kobler yrke og ferdighet.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale verktøy som brukes i utdanning og arbeid, for eksempel for å registrere seg som arbeidssøker eller søke på et kurs.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale ferdigheter selvstendig til videre læring og deltakelse, for eksempel ved å finne og melde seg på et relevant kurs.</t>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser bilder av ulike yrker og hvilke digitale ferdigheter som trengs (f.eks. vaktliste i app for en renholder, e-post for en kontorarbeider). Elevene kobler yrke og ferdighet. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker digitale verktøy som brukes i utdanning og arbeid, for eksempel for å registrere seg som arbeidssøker eller søke på et kurs. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale ferdigheter selvstendig til videre læring og deltakelse, for eksempel ved å finne og melde seg på et relevant kurs. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Personvern og opphavsrett</t>
@@ -1560,13 +1938,19 @@
     <t>Bruker kunnskapen selvstendig og vurderer rettigheter i nye digitale situasjoner.</t>
   </si>
   <si>
-    <t>Læreren forklarer grunnreglene for personvern og opphavsrett med eksempler: ikke del andres bilder uten lov, og ikke bruk bilder fra nett uten å sjekke om det er lov. Elevene sorterer eksempler i «lov» og «ikke lov».</t>
-  </si>
-  <si>
-    <t>Elevene bruker det de har lært i konkrete situasjoner: de finner bilder med fri bruk til en presentasjon og spør medelever om lov før de tar bilder.</t>
-  </si>
-  <si>
-    <t>Elevene vurderer rettigheter i nye situasjoner, for eksempel ved deling av video fra et arrangement eller bruk av musikk i en video, og begrunner valgene.</t>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren forklarer grunnreglene for personvern og opphavsrett med eksempler: ikke del andres bilder uten lov, og ikke bruk bilder fra nett uten å sjekke om det er lov. Elevene sorterer eksempler i «lov» og «ikke lov». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker det de har lært i konkrete situasjoner: de finner bilder med fri bruk til en presentasjon og spør medelever om lov før de tar bilder. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene vurderer rettigheter i nye situasjoner, for eksempel ved deling av video fra et arrangement eller bruk av musikk i en video, og begrunner valgene. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Kritisk tenkning</t>
@@ -1584,13 +1968,19 @@
     <t>Drøfter selvstendig betydningen av digital dømmekraft og begrunner standpunkt.</t>
   </si>
   <si>
-    <t>Læreren leder en samtale med bilder og enkle spørsmål: Hvorfor er det viktig å tenke kritisk på nett? Elevene svarer med setningsstartere som «Det er viktig fordi …».</t>
-  </si>
-  <si>
-    <t>Elevene samtaler i par og gir egne eksempler på kritisk tenkning i digitale sammenhenger, for eksempel om en nyhet eller et tilbud på nett.</t>
-  </si>
-  <si>
-    <t>Elevene drøfter selvstendig betydningen av digital dømmekraft i samfunnet, og begrunner sitt eget standpunkt i en kort tekst eller muntlig.</t>
+    <t xml:space="preserve">Forbered: Legg klar setningsstartere og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren leder en samtale med bilder og enkle spørsmål: Hvorfor er det viktig å tenke kritisk på nett? Elevene svarer med setningsstartere som «Det er viktig fordi …». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene samtaler i par og gir egne eksempler på kritisk tenkning i digitale sammenhenger, for eksempel om en nyhet eller et tilbud på nett. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene drøfter selvstendig betydningen av digital dømmekraft i samfunnet, og begrunner sitt eget standpunkt i en kort tekst eller muntlig. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Helsetjenester</t>
@@ -1608,13 +1998,19 @@
     <t>Bruker digitale helsetjenester selvstendig for seg selv og eventuelt familie.</t>
   </si>
   <si>
-    <t>Læreren viser helsenorge.no og viser hvordan man logger inn med BankID. Elevene øver på å logge inn med støtte.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale helsetjenester delvis selvstendig: de bestiller time hos fastlegen eller leser en melding i en øvingssituasjon.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale helsetjenester selvstendig, for seg selv og eventuelt for barna sine, og viser en medelev hvordan det gjøres.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser helsenorge.no og viser hvordan man logger inn med BankID. Elevene øver på å logge inn med støtte. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker digitale helsetjenester delvis selvstendig: de bestiller time hos fastlegen eller leser en melding i en øvingssituasjon. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale helsetjenester selvstendig, for seg selv og eventuelt for barna sine, og viser en medelev hvordan det gjøres. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Rettigheter</t>
@@ -1632,13 +2028,19 @@
     <t>Bruker digitale tjenester selvstendig og finner nye ved behov.</t>
   </si>
   <si>
-    <t>Læreren viser digitale tjenester som gjelder elevenes rettigheter, for eksempel NAV og Skatteetaten. Elevene åpner tjenestene med støtte og finner én opplysning.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale offentlige tjenester delvis selvstendig, for eksempel for å sjekke skattekortet eller sende en melding til NAV.</t>
-  </si>
-  <si>
-    <t>Elevene bruker digitale tjenester selvstendig og finner nye tjenester ved behov, for eksempel når de flytter eller får barn.</t>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser digitale tjenester som gjelder elevenes rettigheter, for eksempel NAV og Skatteetaten. Elevene åpner tjenestene med støtte og finner én opplysning. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar kort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene bruker digitale offentlige tjenester delvis selvstendig, for eksempel for å sjekke skattekortet eller sende en melding til NAV. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene bruker digitale tjenester selvstendig og finner nye tjenester ved behov, for eksempel når de flytter eller får barn. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Samfunnsdeltakelse</t>
@@ -1656,13 +2058,19 @@
     <t>Deltar aktivt og selvstendig på digitale sosiale og frivillige arenaer.</t>
   </si>
   <si>
-    <t>Læreren viser hvordan en lokal forening (f.eks. idrettslag eller frivilligsentral) bruker nettside og sosiale medier. Elevene ser på kanalene sammen med læreren.</t>
-  </si>
-  <si>
-    <t>Elevene finner relevante digitale fellesskap i nærmiljøet og melder seg inn i ett av dem, delvis selvstendig.</t>
-  </si>
-  <si>
-    <t>Elevene deltar aktivt og selvstendig på digitale sosiale og frivillige arenaer, og forteller klassen om hva de deltar i.</t>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser hvordan en lokal forening (f.eks. idrettslag eller frivilligsentral) bruker nettside og sosiale medier. Elevene ser på kanalene sammen med læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene finner relevante digitale fellesskap i nærmiljøet og melder seg inn i ett av dem, delvis selvstendig. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene deltar aktivt og selvstendig på digitale sosiale og frivillige arenaer, og forteller klassen om hva de deltar i. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
   <si>
     <t>Kap. 5 – Kunnskapssøking</t>
@@ -1680,13 +2088,19 @@
     <t>Driver selvstendig kunnskapssøking i digitale kilder og vurderer dem kritisk.</t>
   </si>
   <si>
-    <t>Læreren gir elevene anviste digitale ressurser, for eksempel en lettlest nettside om et samfunnstema, og elevene finner mer kunnskap med støtte.</t>
-  </si>
-  <si>
-    <t>Elevene søker selv etter mer kunnskap i anbefalte digitale kilder og noterer hva de fant.</t>
-  </si>
-  <si>
-    <t>Elevene søker selvstendig etter kunnskap i digitale kilder, vurderer kildene kritisk og presenterer det de har lært.</t>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren gir elevene anviste digitale ressurser, for eksempel en lettlest nettside om et samfunnstema, og elevene finner mer kunnskap med støtte. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Elevene søker selv etter mer kunnskap i anbefalte digitale kilder og noterer hva de fant. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Elevene søker selvstendig etter kunnskap i digitale kilder, vurderer kildene kritisk og presenterer det de har lært. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Legg til FOV, ny startside, søk, sortering og avkryssingsliste
- FOV-arkene er flyttet inn i kildefilen og datafilen (eget «FOV – »-prefiks),
  med klasseromseksempler for alle 34 målene. Den ubrukte kopien i src/data er fjernet.
- Ny startside med to valg: norsk og samfunnskunnskap, eller FOV.
- Toppfeltet heter «IKT-plan for Molde voksenopplæringssenter» og har Hjem-knapp.
- «Alle mål»: søk med vekting, stammer og toleranse for skrivefeil, filter på fag,
  sortering, gruppering og visning som liste, kort eller tabell.
- Avkryssingsliste i Word med avkrysning per nivå, for hele området eller det som vises.
- Området er med i adressen (#/fov/...), og gamle lenker sendes videre.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Krd89UdHtRi9kZMHKYjeCa
</commit_message>
<xml_diff>
--- a/public/data/digitale-ferdigheter.xlsx
+++ b/public/data/digitale-ferdigheter.xlsx
@@ -10,13 +10,19 @@
     <sheet sheetId="4" name="Overordnet del" state="visible" r:id="rId4"/>
     <sheet sheetId="3" name="Norsk" state="visible" r:id="rId5"/>
     <sheet sheetId="2" name="Samfunnsfag" state="visible" r:id="rId6"/>
+    <sheet sheetId="1" name="FOV – Grunnmodul" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="FOV – Matematikk" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="FOV – Naturfag" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="FOV – Engelsk" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="FOV – Norsk" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="FOV – Samfunnsfag" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1129" uniqueCount="808">
   <si>
     <t>Nr.</t>
   </si>
@@ -2100,6 +2106,963 @@
   <si>
     <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
 Gjør: Elevene søker selvstendig etter kunnskap i digitale kilder, vurderer kildene kritisk og presenterer det de har lært. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Grunnmodul</t>
+  </si>
+  <si>
+    <t>Digitale ferdigheter</t>
+  </si>
+  <si>
+    <t>Bruke digitale verktøy og ressurser til kommunikasjon og læring</t>
+  </si>
+  <si>
+    <t>Bruker navn, adresse, fødselsdato og telefonnummer i enkelt skjema med støtte</t>
+  </si>
+  <si>
+    <t>Skriver ord og korte setninger om kjente temaer delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Lager enkle sammensatte tekster og bruker digitale ressurser selvstendig i kommunikasjon og læring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og skjemaet før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et enkelt påmeldingsskjema på storskjerm og fyller ut navn, adresse, fødselsdato og telefonnummer sammen med klassen. Deltakerne fyller ut det samme skjemaet på egen PC med navnekortet sitt ved siden av. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar setningsstartere og læringsplattformen før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne skriver en kort melding på læringsplattformen om et kjent tema, for eksempel «Min helg» eller «Familien min», med tre–fem setninger. Setningsstartere ligger framme for den som trenger dem. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar et e-posteksempel, plakaten og bilder før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne lager en enkel digital plakat om seg selv med tekst og bilder og sender den til en medelev med en kort hilsen i e-post. De velger selv hvilket verktøy de bruker. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Få grunnlag for bruk av digitale ferdigheter i hverdagssituasjoner</t>
+  </si>
+  <si>
+    <t>Bruker noen digitale ressurser og verktøy med veiledning</t>
+  </si>
+  <si>
+    <t>Bruker flere digitale ressurser delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Bruker digitale ferdigheter selvstendig i hverdagssituasjoner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, lenken og mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser på storskjerm hvordan man åpner en lenke på mobilen, finner busstider i reiseappen og tar et skjermbilde. Deltakerne gjør det samme trinn for trinn på egen mobil. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten og mobilen før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne løser tre hverdagsoppgaver på mobilen fra en sjekkliste: finne åpningstiden til legekontoret, sjekke været i morgen og finne neste buss hjem. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne får en hverdagssituasjon, for eksempel å bestille time hos fastlegen eller sende melding til barnehagen, og løser den digitalt på egen hånd. De forteller klassen hvilke steg de tok. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Matematikk</t>
+  </si>
+  <si>
+    <t>Modul 1</t>
+  </si>
+  <si>
+    <t>Lese av enkle tabeller fra dagliglivet</t>
+  </si>
+  <si>
+    <t>Leser enkle tabeller med støtte</t>
+  </si>
+  <si>
+    <t>Leser enkle tabeller delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Leser og forstår enkle tabeller selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en enkel busstabell på storskjerm og peker ut rad og kolonne. Deltakerne finner sammen når bussen går fra skolen klokka åtte, og markerer svaret på et utskrevet ark. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne leser av en åpningstidstabell og en pristabell fra en butikk og svarer på fem spørsmål i par, for eksempel «Hva koster to liter melk?». Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne finner selv en tabell fra dagliglivet på nettsiden til kommunen eller et busselskap, lager tre spørsmål til den og lar en medelev svare. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Beskrive tid ved hjelp av klokke og kalender</t>
+  </si>
+  <si>
+    <t>Beskriver tid med støtte</t>
+  </si>
+  <si>
+    <t>Bruker klokke og kalender delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Bruker klokke og kalender selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, bildekort og mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser klokka og kalenderen på mobilen på storskjerm. Deltakerne finner dagens dato og stiller en alarm til neste friminutt, med bildekort for ukedagene ved siden av. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar mobilen før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne legger inn tre avtaler i kalenderen på mobilen, for eksempel legetime, foreldremøte og norskprøve, med riktig dato og klokkeslett. De sjekker med en medelev at alt stemmer. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne planlegger en uke med jobb, skole og fritid i en digital kalender og regner ut hvor mange timer de bruker på hver aktivitet. De forklarer planen for klassen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Modul 2</t>
+  </si>
+  <si>
+    <t>Bruke referansesystem og formler i regneark</t>
+  </si>
+  <si>
+    <t>Bruker enkle regneark med veiledning</t>
+  </si>
+  <si>
+    <t>Bruker regneark delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Bruker regneark selvstendig i beregninger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren åpner et regneark på storskjerm og viser hva en celle, en rad og en kolonne er. Deltakerne skriver tall i A1 og A2 og lager formelen =A1+A2 sammen med læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne lager en enkel handleliste i regneark med vare, antall og pris, og bruker formler for å regne ut sum per vare og totalsum. Sjekklisten med formler ligger framme. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne bygger et regneark for et eget budsjett der de bruker cellereferanser og SUMMER, og tester at totalen endrer seg riktig når de endrer ett tall. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Gjøre beregninger knyttet til kjøp, salg og økonomi ved bruk av regneark</t>
+  </si>
+  <si>
+    <t>Gjør enkle beregninger med støtte</t>
+  </si>
+  <si>
+    <t>Gjør beregninger delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Gjør ulike beregninger selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et regneark med tre varer fra en butikkreklame. Deltakerne skriver inn pris og antall og regner ut totalsum sammen med læreren, ett steg om gangen. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne sammenligner prisen på samme vare i to butikker i regneark og regner ut hvor mye de sparer. De bruker en ferdig mal med kolonner for butikk, pris og forskjell. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne lager et månedsbudsjett i regneark med inntekter og utgifter, regner ut hva som blir igjen og vurderer hvor de kan spare. De presenterer budsjettet for en medelev. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Samle, sortere og presentere data i tabeller og diagrammer</t>
+  </si>
+  <si>
+    <t>Samler data med støtte</t>
+  </si>
+  <si>
+    <t>Presenterer data i tabeller delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Bruker tabeller og diagrammer selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren spør klassen hvilken frukt de liker best og fører svarene inn i en tabell på storskjerm. Deltakerne teller strekene sammen og lager et søylediagram med læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne samler inn data om hvordan medelevene kommer seg til skolen, fører svarene inn i en tabell i regneark og lager et diagram ved hjelp av et ferdig eksempel. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne velger et eget tema, samler inn data, sorterer dem i regneark og velger selv hvilket diagram som passer best. De forklarer hvorfor de valgte nettopp det diagrammet. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Modul 3</t>
+  </si>
+  <si>
+    <t>Bruke digitale verktøy i beregninger med hele tall og desimaltall</t>
+  </si>
+  <si>
+    <t>Bruker enkle verktøy med veiledning</t>
+  </si>
+  <si>
+    <t>Bruker digitale verktøy delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Velger og bruker passende verktøy selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser kalkulatoren på mobilen på storskjerm. Deltakerne regner ut prisen på tre varer sammen med læreren og lærer hvor komma-tasten er. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne regner ut pris per kilo for fem varer fra en butikkreklame med kalkulator eller regneark og sammenligner hvilke varer som er billigst. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne får et problem fra dagliglivet, for eksempel å fordele en strømregning på tre personer, og velger selv om de bruker hoderegning, kalkulator eller regneark. De begrunner valget. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Presentere data med og uten digitale verktøy</t>
+  </si>
+  <si>
+    <t>Presenterer enkle data med støtte</t>
+  </si>
+  <si>
+    <t>Presenterer data delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Velger framstilling og begrunner valg selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser samme tall som en liste, en tabell og et søylediagram på storskjerm. Deltakerne peker på hvilken framstilling som er lettest å lese, og tegner et enkelt søylediagram på papir. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne presenterer de samme dataene to ganger, én gang med blyant og papir og én gang i regneark. De sammenligner de to framstillingene i par. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne presenterer et datasett i et diagram de velger selv og forklarer for klassen hvorfor framstillingen passer til dataene og hvem som skal lese den. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>Finne sentralmål og variasjonsbredde med og uten digitale verktøy</t>
+  </si>
+  <si>
+    <t>Finner gjennomsnitt med støtte</t>
+  </si>
+  <si>
+    <t>Regner sentralmål delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Finner sentralmål og forholder seg kritisk til resultatene</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser fem temperaturer fra værmeldingen på storskjerm. Deltakerne legger sammen tallene og deler på fem med kalkulator, og finner gjennomsnittet sammen med læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne finner gjennomsnitt, median og variasjonsbredde for et lite datasett, for eksempel høydene i klassen, med regneark. Sjekklisten med formler ligger framme. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne finner sentralmål for et datasett med og uten regneark, sammenligner resultatene og vurderer hvilket sentralmål som gir det mest rettferdige bildet. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>Modul 4Y</t>
+  </si>
+  <si>
+    <t>Planlegge og gjennomføre datainnsamling ved spørreundersøkelser</t>
+  </si>
+  <si>
+    <t>Deltar i datainnsamling med støtte</t>
+  </si>
+  <si>
+    <t>Samler data delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Planlegger og gjennomfører datainnsamling selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, skjemaet og mobilen før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren lager et enkelt digitalt skjema med ett spørsmål på storskjerm. Deltakerne svarer på mobilen og ser at svarene kommer inn i en tabell. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne lager en spørreundersøkelse med tre spørsmål i et digitalt skjema, sender den til klassen og ser på resultatene i regneark. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne planlegger en spørreundersøkelse om et tema de velger selv, gjennomfører den, presenterer resultatene i diagram og vurderer hva som kunne vært gjort bedre. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Naturfag</t>
+  </si>
+  <si>
+    <t>Gjennomgående i faget</t>
+  </si>
+  <si>
+    <t>Bruke digitale ressurser til å utforske, registrere og presentere data</t>
+  </si>
+  <si>
+    <t>Bruker enkle digitale ressurser med veiledning</t>
+  </si>
+  <si>
+    <t>Bruker ressurser delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Bruker digitale ressurser selvstendig når hen utforsker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en værapp på storskjerm. Deltakerne leser av temperaturen for i dag sammen med læreren og fører den inn i en felles tabell på tavla. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne registrerer temperaturen hver dag i en uke i regneark og lager et linjediagram ved hjelp av et ferdig eksempel. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne velger et fenomen å utforske, for eksempel hvor fort vann fordamper, samler data digitalt og presenterer resultatene med bilder og diagram for klassen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Bruke søkeverktøy og vurdere relevant informasjon</t>
+  </si>
+  <si>
+    <t>Søker med støtte</t>
+  </si>
+  <si>
+    <t>Søker og vurderer delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Bruker søkestrategier og vurderer kilder selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser hvordan man skriver to–tre søkeord i en søkemotor, for eksempel «planter trenger lys». Deltakerne skriver de samme søkeordene og åpner den første nettsiden sammen med læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten og nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne søker etter svar på et naturfaglig spørsmål og velger ut to nettsider som passer. De bruker en sjekkliste med spørsmål om hvem som står bak nettsiden. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne søker etter informasjon om et selvvalgt tema, prøver ulike søkeord og vurderer hvilke kilder som er mest pålitelige. De forklarer valget for en medelev. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Gjøre målinger og skrive inn resultatene i tabell eller skjema</t>
+  </si>
+  <si>
+    <t>Gjør enkle målinger med støtte</t>
+  </si>
+  <si>
+    <t>Gjør målinger og noterer delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Gjør målinger og dokumenterer selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar skjemaet før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser hvordan man måler temperaturen i et glass vann. Deltakerne måler sammen med læreren og skriver tallet inn i et ferdig skjema på PC. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne måler lengde og vekt på fem gjenstander og fører resultatene inn i en tabell i regneark. Malen med kolonner ligger framme. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne planlegger og gjennomfører en serie målinger, lager selv tabellen i regneark og beskriver hvordan de målte, slik at andre kan gjøre det samme. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Lage sammensatte tekster med ord, setninger og bilder</t>
+  </si>
+  <si>
+    <t>Lager enkle tekster med støtte</t>
+  </si>
+  <si>
+    <t>Kombinerer tekst og bilder delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Lager sammensatte tekster selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og bildekort før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et bilde av en plante på storskjerm. Deltakerne skriver navnet på tre deler av planten under bildet i et dokument, med bildekort som støtte. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar setningsstartere og bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne lager et digitalt dokument om et dyr med bilde, overskrift og tre setninger. Setningsstartere ligger framme. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne lager en digital presentasjon om et naturfaglig tema med tekst, bilder og en enkel figur, og velger selv oppsett og verktøy. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Bruke enkle tabeller, modeller og figurer til å organisere data</t>
+  </si>
+  <si>
+    <t>Bruker tabeller med støtte</t>
+  </si>
+  <si>
+    <t>Bruker tabeller og modeller delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Bruker ulike framstillinger selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en tabell over vær i en uke på storskjerm. Deltakerne sorterer dagene i sol, regn og skyer sammen med læreren og fyller ut tabellen. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne organiserer data fra et forsøk i en tabell og lager en enkel figur, for eksempel et søylediagram, med et ferdig eksempel som modell. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne velger selv hvordan de vil organisere data fra et forsøk, i tabell, modell eller figur, og begrunner hvorfor valget gjør dataene lette å forstå. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Gi eksempler på hvor man finner naturfaglig informasjon</t>
+  </si>
+  <si>
+    <t>Kjenner til noen kilder med støtte</t>
+  </si>
+  <si>
+    <t>Finner kilder delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Søker og finner kilder selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, nettsiden og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser to nettsider om helse og natur på storskjerm, for eksempel helsenorge.no og yr.no. Deltakerne forteller hva de kan finne på hver side, med bilder som støtte. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne lager en liste med tre steder der man kan finne naturfaglig informasjon, for eksempel nettsider, leksikon og apper, og skriver hva hvert sted er godt for. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne finner selv fram til kilder om et naturfaglig spørsmål og lager en kort oversikt for klassen over hvor man kan lete og hva hver kilde er god til. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Lese naturfaglig informasjon og reflektere over kildens troverdighet</t>
+  </si>
+  <si>
+    <t>Leser med støtte</t>
+  </si>
+  <si>
+    <t>Leser og reflekterer delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Vurderer kilder kritisk selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren leser en kort tekst om sunt kosthold høyt fra en nettside og viser hvem som står bak siden. Deltakerne svarer sammen på spørsmålet «Kan vi stole på denne siden?». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten og nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne leser to korte tekster om samme tema fra ulike nettsider og bruker en sjekkliste for å vurdere hvem som står bak, når teksten er skrevet og hvorfor den er skrevet. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne finner selv en påstand om helse eller natur på nettet, undersøker hvor den kommer fra og vurderer om den er troverdig. De begrunner vurderingen for klassen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Stille spørsmål, utforske fenomener og presentere resultater</t>
+  </si>
+  <si>
+    <t>Deltar i utforsking med støtte</t>
+  </si>
+  <si>
+    <t>Samler og presenterer data delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Utforsker og presenterer selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet, mobilen og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et kort klipp om hvorfor is smelter. Deltakerne lager sammen spørsmålet «Hvor fort smelter is?», ser på forsøket og tar bilder med mobilen. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne gjennomfører et enkelt forsøk i par, tar bilder underveis og presenterer resultatet med bilder og en tabell. Malen for presentasjonen ligger framme. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne stiller sitt eget spørsmål om et fenomen, planlegger og gjennomfører en undersøkelse og presenterer resultatene digitalt for klassen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Engelsk</t>
+  </si>
+  <si>
+    <t>Bruke visuelle og digitale ressurser til å forstå og finne ord</t>
+  </si>
+  <si>
+    <t>Bruker anviste ressurser med støtte</t>
+  </si>
+  <si>
+    <t>Velger og bruker ressurser selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm, ordboka og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser bilder av ting i klasserommet med engelske ord på storskjerm. Deltakerne slår opp to ord i en bildeordbok på nettet sammen med læreren og sier dem høyt. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar ordboka og bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne finner engelske ord for ti ting hjemme med en bildeordbok eller en ordapp og lager en ordliste med bilder. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar ordboka, klippet og bilder før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne velger selv hvilke ressurser de bruker, for eksempel ordbok, bilder eller video, for å forstå en kort engelsk tekst, og forklarer hvilken ressurs som hjalp mest. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Bruke digitale ressurser og verktøy i språklæring og tekstskaping</t>
+  </si>
+  <si>
+    <t>Bruker verktøy delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Bruker digitale verktøy selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser hvordan man skriver en kort tekst på engelsk i et dokument og bruker stavekontrollen. Deltakerne skriver tre setninger om seg selv sammen med læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar setningsstartere, ordboka og et e-posteksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne skriver en kort e-post på engelsk til en tenkt venn og bruker en ordapp og stavekontroll underveis. Setningsstartere ligger framme. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne lager en kort digital tekst på engelsk, for eksempel en presentasjon av hjembyen, og velger selv verktøy for ordforråd, uttale og retting. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Finne og bruke digitale ressurser og verktøy i samhandling og læring</t>
+  </si>
+  <si>
+    <t>Bruker anviste ressurser</t>
+  </si>
+  <si>
+    <t>Finner og bruker ressurser delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Søker etter og bruker passende ressurser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en engelsk læringsapp på storskjerm. Deltakerne gjør den første oppgaven sammen med læreren og en medelev. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar læringsplattformen før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne samarbeider i par om en engelsk oppgave på læringsplattformen og finner selv ressurser for å forstå ukjente ord. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar klippet og nettsiden før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne finner selv en engelsk nettside, video eller app som passer til et tema, bruker den i en samtale med en medelev og anbefaler den til klassen. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Modul 4</t>
+  </si>
+  <si>
+    <t>Vurdere og bruke ulike digitale ressurser og verktøy</t>
+  </si>
+  <si>
+    <t>Bruker anviste ressurser med veiledning</t>
+  </si>
+  <si>
+    <t>Velger ressurser delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Vurderer og velger ressurser kritisk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser to ordbøker på nettet på storskjerm. Deltakerne slår opp det samme ordet i begge sammen med læreren og ser på forskjellen. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten, ordboka og klippet før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne prøver tre ulike digitale ressurser for å lære nye ord, for eksempel ordbok, app og video, og velger den som passer best for dem. De bruker en sjekkliste for valget. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne vurderer fordeler og ulemper ved oversettelsesverktøy og andre digitale ressurser i engelsk og lager en liste med råd til en ny medelev. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Prøve ut og bruke tilpassede digitale ressurser som støtte</t>
+  </si>
+  <si>
+    <t>Prøver ressurser med veiledning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og ordboka før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser en bildeordbok og en opplesingsfunksjon på storskjerm. Deltakerne prøver å få lest opp en kort tekst sammen med læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar ordboka før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne prøver to tilpassede ressurser, for eksempel opplesing og en ordapp, mens de leser en kort tekst, og forteller hva som hjalp dem. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne velger selv hvilke digitale ressurser de bruker når de leser og skriver en kort tekst, og forklarer hvorfor de valgte akkurat dem. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Bruke egnede digitale ressurser som støtte</t>
+  </si>
+  <si>
+    <t>Velger passende ressurser selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser hvordan stavekontroll og ordforslag fungerer når man skriver en melding. Deltakerne skriver en kort melding sammen med læreren og retter ordene som blir markert. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten og ordboka før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne skriver en kort tekst om et kjent tema og bruker ordbok og stavekontroll som støtte. Sjekklisten for retting ligger framme. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar ordboka før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne skriver en tekst og velger selv hvilke ressurser som passer, for eksempel ordbok, stavekontroll eller opplesing, og begrunner valget. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Velge ut og bruke hensiktsmessige digitale ressurser</t>
+  </si>
+  <si>
+    <t>Velger og begrunner valg selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser tre digitale ressurser for norsk på storskjerm og forteller hva hver av dem er god til. Deltakerne velger én sammen med læreren til en oppgave. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne får en skriveoppgave og velger mellom tre anviste ressurser. De forteller en medelev hvilken de valgte og hvorfor. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne finner og velger selv ressurser til en oppgave i norsk og forklarer hvorfor ressursene er hensiktsmessige for oppgaven. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Reflektere over hvordan man fremstiller seg selv i digitale medier</t>
+  </si>
+  <si>
+    <t>Reflekterer med støtte</t>
+  </si>
+  <si>
+    <t>Reflekterer delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Reflekterer kritisk selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser to profilbilder og to korte profiltekster fra et tenkt sosialt medium på storskjerm. Deltakerne sier sammen med læreren hva de tror andre tenker om personen. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar setningsstartere før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne ser på eksempler på innlegg i sosiale medier og snakker i par om hva innlegget viser om personen. De bruker setningsstartere som støtte. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne vurderer hvordan de selv framstiller seg på nett, og lager en kort profiltekst til en jobbsøknad der de forklarer hva de har valgt å ta med og hvorfor. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Vurdere og bruke ulike digitale ressurser kritisk</t>
+  </si>
+  <si>
+    <t>Bruker ressurser med veiledning</t>
+  </si>
+  <si>
+    <t>Vurderer ressurser delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Vurderer og velger kritisk selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et oversettelsesverktøy på storskjerm og oversetter en setning som blir feil. Deltakerne ser sammen på hva som ble feil, med læreren som veileder. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten og ordboka før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne sammenligner to ressurser, for eksempel ordbok og oversettelsesverktøy, på samme oppgave og skriver ned fordeler og ulemper med en sjekkliste. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne vurderer kritisk hvilke digitale ressurser de bruker i norskarbeidet, også KI-verktøy, og lager egne regler for når ressursene hjelper og når de ikke gjør det. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Samfunnsfag</t>
+  </si>
+  <si>
+    <t>Kjenne til og utforske nettsteder relevante for eget liv og helse</t>
+  </si>
+  <si>
+    <t>Utforsker nettsider med veiledning</t>
+  </si>
+  <si>
+    <t>Utforsker nettsider delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Velger og bruker nettsider selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser helsenorge.no og nettsiden til kommunen på storskjerm. Deltakerne finner telefonnummeret til legevakten sammen med læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar læringsplattformen, lenken og nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne løser tre oppgaver på nettsider som er relevante for eget liv, for eksempel å finne åpningstiden til biblioteket og informasjon om vaksiner. Lenkene ligger på læringsplattformen. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne finner selv nettsider som er nyttige for eget liv og helse, og lager en liste med anbefalinger til klassen med en kort begrunnelse for hver. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Samtale om nettvett i hverdagen</t>
+  </si>
+  <si>
+    <t>Kjenner til enkle regler med støtte</t>
+  </si>
+  <si>
+    <t>Samtaler om nettvett delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Reflekterer og handler etter nettvettsprinsippene</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar lenken og bilder før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser tre situasjoner med bilder: en ukjent lenke, en melding om premie og en venneforespørsel fra en fremmed. Deltakerne svarer sammen «trygt» eller «utrygt». Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar situasjonskort og bilder før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne snakker i par om situasjonskort med nettvett i hverdagen, for eksempel passord og deling av bilder, og blir enige om hva som er lurt å gjøre. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar plakaten før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne lager en plakat med fem råd om nettvett for nye deltakere og forklarer hvorfor hvert råd er viktig. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Bruke fysiske og digitale kart som verktøy</t>
+  </si>
+  <si>
+    <t>Bruker kart med støtte</t>
+  </si>
+  <si>
+    <t>Bruker kart delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Bruker kart kritisk og selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser et papirkart og et digitalt kart over nærmiljøet på storskjerm. Deltakerne finner skolen og butikken sammen med læreren på begge kartene. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar mobilen før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne finner veien fra skolen til biblioteket med et digitalt kart på mobilen og tegner ruten på et papirkart. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne planlegger en tur med kollektivtransport til et nytt sted med digitale kart og vurderer hvilken rute som er best når det gjelder tid og pris. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Samtale om digital dømmekraft og kildekritikk</t>
+  </si>
+  <si>
+    <t>Kjenner begrepene med støtte</t>
+  </si>
+  <si>
+    <t>Samtaler og vurderer delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Viser dømmekraft og kritikk selvstendig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser to nyhetsoverskrifter på storskjerm, én ekte og én falsk. Deltakerne sier sammen med læreren hvilken de tror er sann, og hvorfor. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar dilemmakort før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne snakker i par om dilemmakort om digital dømmekraft, for eksempel om de skal dele en nyhet de ikke vet er sann, og blir enige om et svar. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne vurderer en sak fra sosiale medier, undersøker kilden og forklarer for klassen hvordan de kom fram til at saken var troverdig eller ikke. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Sammenligne og vurdere informasjon fra ulike kilder</t>
+  </si>
+  <si>
+    <t>Sammenligner med veiledning</t>
+  </si>
+  <si>
+    <t>Vurderer kilder delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Vurderer og velger kilder kritisk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar storskjerm og nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser samme nyhet fra to ulike nettsider på storskjerm. Deltakerne finner sammen med læreren én ting som er likt og én ting som er ulikt. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar sjekklisten før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne sammenligner informasjon om samme tema fra to kilder med en sjekkliste: hvem står bak, når er det skrevet og hvorfor. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Gjør klart ett konkret eksempel før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne finner selv tre kilder om en samfunnssak, sammenligner dem og vurderer hvilken kilde som er mest pålitelig. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
+Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
+  </si>
+  <si>
+    <t>Bruke ulike metoder for å finne informasjon og reflektere over kilder</t>
+  </si>
+  <si>
+    <t>Søker med veiledning</t>
+  </si>
+  <si>
+    <t>Søker og reflekterer delvis selvstendig</t>
+  </si>
+  <si>
+    <t>Bruker metoder kritisk og vurderer algoritmer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Vis hele oppgaven selv først, med én modell deltakerne kan følge.
+Gjør: Læreren viser hvordan man søker med søkemotor og hvordan man finner informasjon på en offentlig nettside med menyen. Deltakerne prøver begge måtene sammen med læreren. Læreren viser hvert trinn og venter til deltakerne har gjort det samme.
+Se etter: Se om deltakeren får det til når du har vist det først, og om hen bruker støtten som ligger framme.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. La modellen ligge synlig, slik at deltakerne kan se på den når de trenger det.
+Gjør: Deltakerne finner svar på et samfunnsfaglig spørsmål ved å bruke både søkemotor og en offentlig nettside og skriver ned hvor de fant svaret. Læreren hjelper bare når noen står fast.
+Se etter: Se om deltakeren kommer i gang i den kjente oppgaven og ber om hjelp når hen står fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbered: Legg klar nettsiden før økten. Legg fram oppgaven uten å vise løsningen, så deltakerne kan velge arbeidsmåte selv.
+Gjør: Deltakerne bruker ulike metoder for å finne informasjon, for eksempel søkemotor, nettsider, intervju og KI-verktøy. De reflekterer over hvordan algoritmer påvirker hva de får se. Til slutt ber læreren deltakeren forklare hva hen gjorde, og prøve det samme i en ny situasjon.
 Se etter: Se om deltakeren gjennomfører uten modell og kan bruke det samme i en ny situasjon.</t>
   </si>
 </sst>
@@ -2500,6 +3463,129 @@
 </a:theme>
 </file>
 
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" customWidth="1"/>
+    <col min="6" max="6" width="47.85546875" customWidth="1"/>
+    <col min="7" max="7" width="44.140625" customWidth="1"/>
+    <col min="8" max="8" width="59.28515625" customWidth="1"/>
+    <col min="9" max="11" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>558</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>559</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>560</v>
+      </c>
+      <c r="E2" s="7"/>
+      <c r="F2" s="5" t="s">
+        <v>561</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>563</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>564</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>565</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>558</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>559</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>568</v>
+      </c>
+      <c r="E3" s="7"/>
+      <c r="F3" s="5" t="s">
+        <v>569</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>570</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>571</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>572</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>573</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>574</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K13"/>
@@ -5081,4 +6167,1345 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" customWidth="1"/>
+    <col min="6" max="6" width="47.85546875" customWidth="1"/>
+    <col min="7" max="7" width="44.140625" customWidth="1"/>
+    <col min="8" max="8" width="59.28515625" customWidth="1"/>
+    <col min="9" max="11" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>577</v>
+      </c>
+      <c r="E2" s="7"/>
+      <c r="F2" s="5" t="s">
+        <v>578</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>579</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>580</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>581</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>582</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>584</v>
+      </c>
+      <c r="E3" s="7"/>
+      <c r="F3" s="5" t="s">
+        <v>585</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>586</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>587</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>593</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>595</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>596</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>597</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>598</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>601</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="5" t="s">
+        <v>602</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>603</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>604</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>605</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>606</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>609</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="F6" s="5" t="s">
+        <v>610</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>611</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>612</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>613</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>614</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>616</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>618</v>
+      </c>
+      <c r="E7" s="7"/>
+      <c r="F7" s="5" t="s">
+        <v>619</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>620</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>621</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="E8" s="7"/>
+      <c r="F8" s="5" t="s">
+        <v>627</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>628</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>629</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>630</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>631</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>633</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>634</v>
+      </c>
+      <c r="E9" s="7"/>
+      <c r="F9" s="5" t="s">
+        <v>635</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>636</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>637</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>638</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>639</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>642</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>643</v>
+      </c>
+      <c r="E10" s="7"/>
+      <c r="F10" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>645</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>646</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>649</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" customWidth="1"/>
+    <col min="6" max="6" width="47.85546875" customWidth="1"/>
+    <col min="7" max="7" width="44.140625" customWidth="1"/>
+    <col min="8" max="8" width="59.28515625" customWidth="1"/>
+    <col min="9" max="11" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>651</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>652</v>
+      </c>
+      <c r="E2" s="7"/>
+      <c r="F2" s="5" t="s">
+        <v>653</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>654</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>651</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>659</v>
+      </c>
+      <c r="E3" s="7"/>
+      <c r="F3" s="5" t="s">
+        <v>660</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>661</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>662</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>664</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>666</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="5" t="s">
+        <v>667</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>668</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>669</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>671</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>673</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="5" t="s">
+        <v>674</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>675</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>676</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>677</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>678</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>680</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="F6" s="5" t="s">
+        <v>681</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>682</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>683</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>684</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>685</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>616</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>687</v>
+      </c>
+      <c r="E7" s="7"/>
+      <c r="F7" s="5" t="s">
+        <v>688</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>689</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>691</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>692</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>694</v>
+      </c>
+      <c r="E8" s="7"/>
+      <c r="F8" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>696</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>697</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>698</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>699</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>633</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="E9" s="7"/>
+      <c r="F9" s="5" t="s">
+        <v>702</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>703</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>705</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>706</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>707</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" customWidth="1"/>
+    <col min="6" max="6" width="47.85546875" customWidth="1"/>
+    <col min="7" max="7" width="44.140625" customWidth="1"/>
+    <col min="8" max="8" width="59.28515625" customWidth="1"/>
+    <col min="9" max="11" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>709</v>
+      </c>
+      <c r="E2" s="7"/>
+      <c r="F2" s="5" t="s">
+        <v>710</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>654</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>711</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>712</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>713</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>715</v>
+      </c>
+      <c r="E3" s="7"/>
+      <c r="F3" s="5" t="s">
+        <v>619</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>716</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>717</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>718</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>719</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>721</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="5" t="s">
+        <v>722</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>723</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>724</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>725</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>726</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>728</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>729</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="5" t="s">
+        <v>730</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>731</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>732</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>733</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>734</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>735</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" customWidth="1"/>
+    <col min="6" max="6" width="47.85546875" customWidth="1"/>
+    <col min="7" max="7" width="44.140625" customWidth="1"/>
+    <col min="8" max="8" width="59.28515625" customWidth="1"/>
+    <col min="9" max="11" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>736</v>
+      </c>
+      <c r="E2" s="7"/>
+      <c r="F2" s="5" t="s">
+        <v>737</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>654</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>711</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>738</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>739</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>741</v>
+      </c>
+      <c r="E3" s="7"/>
+      <c r="F3" s="5" t="s">
+        <v>722</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>654</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>742</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>743</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>746</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="5" t="s">
+        <v>722</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>731</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>747</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>748</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>749</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>751</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="5" t="s">
+        <v>752</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>753</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>754</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>755</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>756</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>728</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>758</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="F6" s="5" t="s">
+        <v>759</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>760</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>761</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>762</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>763</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>764</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" customWidth="1"/>
+    <col min="6" max="6" width="47.85546875" customWidth="1"/>
+    <col min="7" max="7" width="44.140625" customWidth="1"/>
+    <col min="8" max="8" width="59.28515625" customWidth="1"/>
+    <col min="9" max="11" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>765</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>766</v>
+      </c>
+      <c r="E2" s="7"/>
+      <c r="F2" s="5" t="s">
+        <v>767</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>768</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>769</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>771</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>765</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>773</v>
+      </c>
+      <c r="E3" s="7"/>
+      <c r="F3" s="5" t="s">
+        <v>774</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>775</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>776</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>777</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>778</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>765</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="5" t="s">
+        <v>781</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>782</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>783</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>784</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>785</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>765</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>787</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="5" t="s">
+        <v>788</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>789</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>790</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>791</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>792</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>765</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="F6" s="5" t="s">
+        <v>795</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>796</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>797</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>798</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>799</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>616</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>765</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>728</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="E7" s="7"/>
+      <c r="F7" s="5" t="s">
+        <v>802</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>803</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>804</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>805</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>806</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>807</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
 </file>
</xml_diff>